<commit_message>
Agrega hoja Contenedor2: costo puesto en Lima de bidones, kit 3 en 1 y Cero
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Supuestos" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Desglose" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Costo_Lima" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Contenedor2" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Costo_Lima" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="225">
   <si>
     <t xml:space="preserve">Resumen - utilidad por pedido (S/)</t>
   </si>
@@ -334,21 +335,282 @@
     <t xml:space="preserve">Excluye: PureCore / nucleo de magnesio si es otra compra, tarifa de almacen de puerto pendiente, comisiones bancarias, costos fijos de equipo e impuesto a la renta.</t>
   </si>
   <si>
+    <t xml:space="preserve">Contenedor 2 - bidones 22 L / 16 L, kit 3 en 1 y elvo· Cero (R260) - B/L COSU6464399990, 40HQ, llega a Chancay el 25-oct-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azul = dato de los documentos o supuesto editable. Negro = formula. Verde = viene de otra hoja. Lo marcado ESTIMADO sale del embarque anterior, no de un documento de este contenedor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOB unitario (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOB total (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volumen (CBM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% del volumen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% del valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bidon purificador 22 L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bidon purificador 16 L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit de filtros 3 en 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elvo· Cero R260 (100 maquinas + 20 filtros + entrega a Ningbo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuentes: factura DK-GV-2026-01 (Ningbo Dukang, 1-jun-2026) y packing list; proforma 10062026356AVR260W (Suzhou Beiang, 10-jun-2026, EXW). CBM de Cero = CBM total del B/L menos los CBM del packing list (101 cartones, ~1,014 kg).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detalle elvo· Cero (Suzhou Beiang) - pago 30% anticipo / 70% antes de embarque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concepto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maquinas R260 (agua fria y caliente, osmosis inversa, UV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro ROC de repuesto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro PAC de repuesto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega a Ningbo (monto unico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Cero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volumen y flete (B/L: flete collect, se paga en destino)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volumen total del B/L (CBM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flete maritimo (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Adjustment Factor (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISPS (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THC en destino (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total flete collect (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visto bueno de importacion Callao-Chancay (US$, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAC (US$, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otros gastos locales ESTIMADOS (US$, con IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suma de agenciamiento, transmision, handling, documentacion, descarga y gastos admin. de la factura Inca Lines del embarque anterior. Contenedor completo puede variar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguro nocional (% del FOB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mismo % que la proforma de aduana anterior (US$ 74.50 sobre FOB 7,450). Es base de impuestos, no un pago.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impuestos de aduana - ratios del embarque anterior (proforma 026/0000257)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIF anterior (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de cambio de aduana anterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IGV anterior (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IPM anterior (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percepcion anterior (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IGV + IPM como % del CIF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percepcion como % del CIF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arancel ad valorem (SUPUESTO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El embarque anterior pago 0%. Confirmar la partida arancelaria del Cero y de los bidones con el agente antes de nacionalizar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agente de aduana y transporte local - ESTIMADO (S/, sin IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comision del agente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anterior: S/ 900 sobre CIF de US$ 8.2k; este CIF es ~5 veces mayor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos de aduana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Igual que el embarque anterior.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regularizacion SADA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camion de contenedor Chancay - San Borja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anterior: S/ 620 en carga LCL. Un 40HQ completo cuesta mas; pedir cotizacion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IGV del agente (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultado del contenedor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguro nocional (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIF (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIF (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arancel (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IGV + IPM (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percepcion (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impuestos de aduana (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proveedores (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flete collect (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visto bueno + SAC con IGV (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otros gastos locales (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agente con IGV (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL DESEMBOLSADO (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IGV recuperable (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTO REAL PUESTO EN LIMA (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo real (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente de pagar: todo menos proveedores (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se asume que los dos proveedores ya estan pagados. Flete collect y visto bueno se pagan antes de retirar el contenedor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo unitario puesto en Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo neto asignado (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTO UNITARIO neto de IGV recuperable (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo unitario si NO recuperas IGV (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo unitario que se usa (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">control: debe ser 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reparto: mercaderia directa; flete, gastos locales y agente por volumen (CBM); arancel e impuestos por valor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margen INDICATIVO por pedido en Lima (S/) - precios PROVISIONALES de la tienda anterior; courier de bultos grandes probablemente mayor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bidon 22 L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bidon 16 L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit 3 en 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elvo· Cero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio de venta (con IGV) - provisional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publicidad (1 = si, 0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incluye garantia ni postventa del Cero, costo de courier de bultos grandes, ni la partida arancelaria definitiva. Precios: bidon 22 L S/ 198, bidon 16 L S/ 120 y kit S/ 85 son los de la tienda anterior (AQA); Cero S/ 1,999 del listado actual.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Costo puesto en Lima - embarque Ningbo (llegada 22-abr-2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Azul = dato de los documentos (proforma, factura Inca Lines, proforma aduana). Negro = formula. Tipo de cambio viene de la hoja Supuestos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cantidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOB unitario (US$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOB total (US$)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Filtro de caño NW-TR201-W (carcasa + cartucho CTO-10B + grifo)</t>
   </si>
   <si>
@@ -406,21 +668,12 @@
     <t xml:space="preserve">Agencia de aduana con IGV (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">Impuestos de aduana (S/)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total desembolsado (S/)</t>
   </si>
   <si>
     <t xml:space="preserve">Impuestos recuperables (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">COSTO REAL PUESTO EN LIMA (S/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo real (US$)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reparto de costos compartidos (flete, puerto, aduana) por valor FOB de cada producto</t>
   </si>
   <si>
@@ -433,9 +686,6 @@
     <t xml:space="preserve">Costo asignado (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">Unidades</t>
-  </si>
-  <si>
     <t xml:space="preserve">COSTO UNITARIO (S/)</t>
   </si>
   <si>
@@ -446,9 +696,6 @@
   </si>
   <si>
     <t xml:space="preserve">Filtro de ducha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
   </si>
   <si>
     <t xml:space="preserve">Limitacion: no incluye PureCore/nucleo de magnesio (si vienen de otra compra), empaque final, comisiones bancarias ni almacen de puerto pendiente.</t>
@@ -458,7 +705,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0;\(#,##0.0\);\-"/>
@@ -467,6 +714,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.00;\(#,##0.00\);\-"/>
     <numFmt numFmtId="170" formatCode="0"/>
     <numFmt numFmtId="171" formatCode="0.00%"/>
+    <numFmt numFmtId="172" formatCode="0.00"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -608,7 +856,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -721,7 +969,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -729,11 +997,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3692,6 +3964,1140 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G92"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>804</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <f aca="false">B5*C5</f>
+        <v>7638</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>19.4313735</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <f aca="false">E5/$E$9</f>
+        <v>0.358710974709249</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <f aca="false">D5/$D$9</f>
+        <v>0.241083264945395</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>804</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <f aca="false">B6*C6</f>
+        <v>5628</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>20.848256</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <f aca="false">E6/$E$9</f>
+        <v>0.38486719586487</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <f aca="false">D6/$D$9</f>
+        <v>0.17764030048608</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>840</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <f aca="false">B7*C7</f>
+        <v>1764</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <f aca="false">E7/$E$9</f>
+        <v>0.0932250323057043</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <f aca="false">D7/$D$9</f>
+        <v>0.0556783031374282</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <f aca="false">D8/B8</f>
+        <v>166.52</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <f aca="false">D17</f>
+        <v>16652</v>
+      </c>
+      <c r="E8" s="28" t="n">
+        <f aca="false">B20-SUM(E5:E7)</f>
+        <v>8.84037050000001</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <f aca="false">E8/$E$9</f>
+        <v>0.163196797120177</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <f aca="false">D8/$D$9</f>
+        <v>0.525598131431097</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <f aca="false">SUM(D5:D8)</f>
+        <v>31682</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <f aca="false">SUM(E5:E8)</f>
+        <v>54.17</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>162</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <f aca="false">B13*C13</f>
+        <v>16200</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <f aca="false">B14*C14</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <f aca="false">B15*C15</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>152</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <f aca="false">B16*C16</f>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17" s="29" t="n">
+        <f aca="false">SUM(D13:D16)</f>
+        <v>16652</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="B20" s="31" t="n">
+        <v>54.17</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="13" t="n">
+        <v>6580</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="13" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="13" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" s="29" t="n">
+        <f aca="false">SUM(B21:B24)</f>
+        <v>7386</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" s="13" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="13" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" s="32" t="n">
+        <v>606.21</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B29" s="33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>8189.581</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>3.444</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B34" s="13" t="n">
+        <v>4370</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B35" s="13" t="n">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B36" s="13" t="n">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="B37" s="17" t="n">
+        <f aca="false">(B34+B35)/(B32*B33)</f>
+        <v>0.179968620594731</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B38" s="17" t="n">
+        <f aca="false">B36/(B32*B33)</f>
+        <v>0.0313775077278047</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B39" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B42" s="32" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B43" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B44" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B45" s="32" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B46" s="14" t="n">
+        <f aca="false">SUM(B42:B45)*Supuestos!B4</f>
+        <v>666</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="34" t="n">
+        <f aca="false">Supuestos!B5</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B50" s="18" t="n">
+        <f aca="false">D9</f>
+        <v>31682</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B51" s="18" t="n">
+        <f aca="false">D9*B29</f>
+        <v>316.82</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B52" s="18" t="n">
+        <f aca="false">B50+B25+B51</f>
+        <v>39384.82</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B53" s="24" t="n">
+        <f aca="false">B52*B49</f>
+        <v>137846.87</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B54" s="24" t="n">
+        <f aca="false">B53*B39</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B55" s="24" t="n">
+        <f aca="false">(B53+B54)*B37</f>
+        <v>24808.1110472012</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B56" s="24" t="n">
+        <f aca="false">B53*B38</f>
+        <v>4325.29122867869</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="B57" s="26" t="n">
+        <f aca="false">SUM(B54:B56)</f>
+        <v>29133.4022758799</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B58" s="24" t="n">
+        <f aca="false">B50*B49</f>
+        <v>110887</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B59" s="24" t="n">
+        <f aca="false">B25*B49</f>
+        <v>25851</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B60" s="24" t="n">
+        <f aca="false">(B26+B27)*(1+Supuestos!B4)*B49</f>
+        <v>826</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="B61" s="24" t="n">
+        <f aca="false">B28*B49</f>
+        <v>2121.735</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B62" s="24" t="n">
+        <f aca="false">SUM(B42:B45)+B46</f>
+        <v>4366</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="B63" s="26" t="n">
+        <f aca="false">B58+B59+B60+B61+B57+B62</f>
+        <v>173185.13727588</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B64" s="6" t="n">
+        <f aca="false">Costo_Lima!B19*(B55+B56+B46+(B60-B60/(1+Supuestos!B4))+(B61-B61/(1+Supuestos!B4)))</f>
+        <v>30249.0567674053</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="25" t="s">
+        <v>174</v>
+      </c>
+      <c r="B65" s="27" t="n">
+        <f aca="false">B63-B64</f>
+        <v>142936.080508475</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="B66" s="18" t="n">
+        <f aca="false">B65/B49</f>
+        <v>40838.8801452785</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B67" s="27" t="n">
+        <f aca="false">B59+B60+B61+B57+B62</f>
+        <v>62298.1372758799</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="9"/>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="10" t="str">
+        <f aca="false">A5</f>
+        <v>Bidon purificador 22 L</v>
+      </c>
+      <c r="B71" s="35" t="n">
+        <f aca="false">B5</f>
+        <v>804</v>
+      </c>
+      <c r="C71" s="24" t="n">
+        <f aca="false">D5*$B$49+($B$59+$B$60/(1+Supuestos!$B$4)+$B$61/(1+Supuestos!$B$4)+SUM($B$42:$B$45))*F5+$B$54*G5</f>
+        <v>38229.3569077301</v>
+      </c>
+      <c r="D71" s="36" t="n">
+        <f aca="false">C71/B71</f>
+        <v>47.5489513777738</v>
+      </c>
+      <c r="E71" s="18" t="n">
+        <f aca="false">(C71+(($B$55+$B$56)*G5)+($B$46+($B$60-$B$60/(1+Supuestos!$B$4))+($B$61-$B$61/(1+Supuestos!$B$4)))*F5)/B71</f>
+        <v>56.7825001958466</v>
+      </c>
+      <c r="F71" s="29" t="n">
+        <f aca="false">IF(Costo_Lima!$B$19=1,D71,E71)</f>
+        <v>47.5489513777738</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="10" t="str">
+        <f aca="false">A6</f>
+        <v>Bidon purificador 16 L</v>
+      </c>
+      <c r="B72" s="35" t="n">
+        <f aca="false">B6</f>
+        <v>804</v>
+      </c>
+      <c r="C72" s="24" t="n">
+        <f aca="false">D6*$B$49+($B$59+$B$60/(1+Supuestos!$B$4)+$B$61/(1+Supuestos!$B$4)+SUM($B$42:$B$45))*F6+$B$54*G6</f>
+        <v>32032.6397453441</v>
+      </c>
+      <c r="D72" s="36" t="n">
+        <f aca="false">C72/B72</f>
+        <v>39.8415917230648</v>
+      </c>
+      <c r="E72" s="18" t="n">
+        <f aca="false">(C72+(($B$55+$B$56)*G6)+($B$46+($B$60-$B$60/(1+Supuestos!$B$4))+($B$61-$B$61/(1+Supuestos!$B$4)))*F6)/B72</f>
+        <v>46.8125434023889</v>
+      </c>
+      <c r="F72" s="29" t="n">
+        <f aca="false">IF(Costo_Lima!$B$19=1,D72,E72)</f>
+        <v>39.8415917230648</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="10" t="str">
+        <f aca="false">A7</f>
+        <v>Kit de filtros 3 en 1</v>
+      </c>
+      <c r="B73" s="35" t="n">
+        <f aca="false">B7</f>
+        <v>840</v>
+      </c>
+      <c r="C73" s="24" t="n">
+        <f aca="false">D7*$B$49+($B$59+$B$60/(1+Supuestos!$B$4)+$B$61/(1+Supuestos!$B$4)+SUM($B$42:$B$45))*F7+$B$54*G7</f>
+        <v>9161.77656577066</v>
+      </c>
+      <c r="D73" s="36" t="n">
+        <f aca="false">C73/B73</f>
+        <v>10.9068768640127</v>
+      </c>
+      <c r="E73" s="18" t="n">
+        <f aca="false">(C73+(($B$55+$B$56)*G7)+($B$46+($B$60-$B$60/(1+Supuestos!$B$4))+($B$61-$B$61/(1+Supuestos!$B$4)))*F7)/B73</f>
+        <v>12.9617641608645</v>
+      </c>
+      <c r="F73" s="29" t="n">
+        <f aca="false">IF(Costo_Lima!$B$19=1,D73,E73)</f>
+        <v>10.9068768640127</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="10" t="str">
+        <f aca="false">A8</f>
+        <v>elvo· Cero R260 (100 maquinas + 20 filtros + entrega a Ningbo)</v>
+      </c>
+      <c r="B74" s="35" t="n">
+        <f aca="false">B8</f>
+        <v>100</v>
+      </c>
+      <c r="C74" s="24" t="n">
+        <f aca="false">D8*$B$49+($B$59+$B$60/(1+Supuestos!$B$4)+$B$61/(1+Supuestos!$B$4)+SUM($B$42:$B$45))*F8+$B$54*G8</f>
+        <v>63512.3072896298</v>
+      </c>
+      <c r="D74" s="36" t="n">
+        <f aca="false">C74/B74</f>
+        <v>635.123072896298</v>
+      </c>
+      <c r="E74" s="18" t="n">
+        <f aca="false">(C74+(($B$55+$B$56)*G8)+($B$46+($B$60-$B$60/(1+Supuestos!$B$4))+($B$61-$B$61/(1+Supuestos!$B$4)))*F8)/B74</f>
+        <v>790.068403277724</v>
+      </c>
+      <c r="F74" s="29" t="n">
+        <f aca="false">IF(Costo_Lima!$B$19=1,D74,E74)</f>
+        <v>635.123072896298</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="C75" s="26" t="n">
+        <f aca="false">SUM(C71:C74)</f>
+        <v>142936.080508475</v>
+      </c>
+      <c r="D75" s="18" t="n">
+        <f aca="false">C75-B65</f>
+        <v>0</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B78" s="9"/>
+      <c r="C78" s="9"/>
+      <c r="D78" s="9"/>
+      <c r="E78" s="9"/>
+      <c r="F78" s="9"/>
+      <c r="G78" s="9"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="B80" s="37" t="n">
+        <v>198</v>
+      </c>
+      <c r="C80" s="37" t="n">
+        <v>120</v>
+      </c>
+      <c r="D80" s="37" t="n">
+        <v>85</v>
+      </c>
+      <c r="E80" s="37" t="n">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B81" s="24" t="n">
+        <f aca="false">B80/(1+Supuestos!$B$4)</f>
+        <v>167.796610169492</v>
+      </c>
+      <c r="C81" s="24" t="n">
+        <f aca="false">C80/(1+Supuestos!$B$4)</f>
+        <v>101.694915254237</v>
+      </c>
+      <c r="D81" s="24" t="n">
+        <f aca="false">D80/(1+Supuestos!$B$4)</f>
+        <v>72.0338983050848</v>
+      </c>
+      <c r="E81" s="24" t="n">
+        <f aca="false">E80/(1+Supuestos!$B$4)</f>
+        <v>1694.06779661017</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="B82" s="24" t="n">
+        <f aca="false">-F71</f>
+        <v>-47.5489513777738</v>
+      </c>
+      <c r="C82" s="24" t="n">
+        <f aca="false">-F72</f>
+        <v>-39.8415917230648</v>
+      </c>
+      <c r="D82" s="24" t="n">
+        <f aca="false">-F73</f>
+        <v>-10.9068768640127</v>
+      </c>
+      <c r="E82" s="24" t="n">
+        <f aca="false">-F74</f>
+        <v>-635.123072896298</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B83" s="6" t="n">
+        <f aca="false">-(B80*Supuestos!$B$31+Supuestos!$B$32)</f>
+        <v>-6.47366</v>
+      </c>
+      <c r="C83" s="6" t="n">
+        <f aca="false">-(C80*Supuestos!$B$31+Supuestos!$B$32)</f>
+        <v>-4.1204</v>
+      </c>
+      <c r="D83" s="6" t="n">
+        <f aca="false">-(D80*Supuestos!$B$31+Supuestos!$B$32)</f>
+        <v>-3.06445</v>
+      </c>
+      <c r="E83" s="6" t="n">
+        <f aca="false">-(E80*Supuestos!$B$31+Supuestos!$B$32)</f>
+        <v>-60.80983</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B84" s="6" t="n">
+        <f aca="false">-Supuestos!$B$16</f>
+        <v>-3.5</v>
+      </c>
+      <c r="C84" s="6" t="n">
+        <f aca="false">-Supuestos!$B$16</f>
+        <v>-3.5</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <f aca="false">-Supuestos!$B$16</f>
+        <v>-3.5</v>
+      </c>
+      <c r="E84" s="6" t="n">
+        <f aca="false">-Supuestos!$B$16</f>
+        <v>-3.5</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B85" s="6" t="n">
+        <f aca="false">-Supuestos!$B$18</f>
+        <v>-12.5</v>
+      </c>
+      <c r="C85" s="6" t="n">
+        <f aca="false">-Supuestos!$B$18</f>
+        <v>-12.5</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <f aca="false">-Supuestos!$B$18</f>
+        <v>-12.5</v>
+      </c>
+      <c r="E85" s="6" t="n">
+        <f aca="false">-Supuestos!$B$18</f>
+        <v>-12.5</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B86" s="26" t="n">
+        <f aca="false">SUM(B81:B85)</f>
+        <v>97.7739987917178</v>
+      </c>
+      <c r="C86" s="26" t="n">
+        <f aca="false">SUM(C81:C85)</f>
+        <v>41.7329235311725</v>
+      </c>
+      <c r="D86" s="26" t="n">
+        <f aca="false">SUM(D81:D85)</f>
+        <v>42.0625714410721</v>
+      </c>
+      <c r="E86" s="26" t="n">
+        <f aca="false">SUM(E81:E85)</f>
+        <v>982.134893713872</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B87" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(B81+B82+B83)</f>
+        <v>-17.0660998187577</v>
+      </c>
+      <c r="C87" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(C81+C82+C83)</f>
+        <v>-8.65993852967588</v>
+      </c>
+      <c r="D87" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(D81+D82+D83)</f>
+        <v>-8.70938571616081</v>
+      </c>
+      <c r="E87" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(E81+E82+E83)</f>
+        <v>-149.720234057081</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B88" s="26" t="n">
+        <f aca="false">B86+B87</f>
+        <v>80.7078989729601</v>
+      </c>
+      <c r="C88" s="26" t="n">
+        <f aca="false">C86+C87</f>
+        <v>33.0729850014967</v>
+      </c>
+      <c r="D88" s="26" t="n">
+        <f aca="false">D86+D87</f>
+        <v>33.3531857249113</v>
+      </c>
+      <c r="E88" s="26" t="n">
+        <f aca="false">E86+E87</f>
+        <v>832.414659656791</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B89" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C89" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="B90" s="27" t="n">
+        <f aca="false">B88-Supuestos!$B$6*B89</f>
+        <v>49.7078989729601</v>
+      </c>
+      <c r="C90" s="27" t="n">
+        <f aca="false">C88-Supuestos!$B$6*C89</f>
+        <v>2.07298500149665</v>
+      </c>
+      <c r="D90" s="27" t="n">
+        <f aca="false">D88-Supuestos!$B$6*D89</f>
+        <v>33.3531857249113</v>
+      </c>
+      <c r="E90" s="27" t="n">
+        <f aca="false">E88-Supuestos!$B$6*E89</f>
+        <v>801.414659656791</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B91" s="19" t="n">
+        <f aca="false">B90/B80</f>
+        <v>0.25104999481293</v>
+      </c>
+      <c r="C91" s="19" t="n">
+        <f aca="false">C90/C80</f>
+        <v>0.0172748750124721</v>
+      </c>
+      <c r="D91" s="19" t="n">
+        <f aca="false">D90/D80</f>
+        <v>0.392390420293074</v>
+      </c>
+      <c r="E91" s="19" t="n">
+        <f aca="false">E90/E80</f>
+        <v>0.400907783720256</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3701,12 +5107,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>104</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3714,7 +5120,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="C4" s="22" t="s">
         <v>106</v>
@@ -3725,7 +5131,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>108</v>
+        <v>195</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>1008</v>
@@ -3740,7 +5146,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>109</v>
+        <v>196</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1000</v>
@@ -3755,7 +5161,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>110</v>
+        <v>197</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>500</v>
@@ -3770,7 +5176,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>111</v>
+        <v>198</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>5</v>
@@ -3785,7 +5191,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>112</v>
+        <v>199</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>1</v>
@@ -3800,26 +5206,26 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="D10" s="28" t="n">
+        <v>200</v>
+      </c>
+      <c r="D10" s="29" t="n">
         <f aca="false">SUM(D5:D9)</f>
         <v>8004.2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>114</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>115</v>
+        <v>202</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>116</v>
+        <v>203</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>1135.87</v>
@@ -3827,7 +5233,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>117</v>
+        <v>204</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>135.13</v>
@@ -3835,7 +5241,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>118</v>
+        <v>205</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>1720</v>
@@ -3843,7 +5249,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>119</v>
+        <v>206</v>
       </c>
       <c r="B17" s="13" t="n">
         <v>309.6</v>
@@ -3851,7 +5257,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>120</v>
+        <v>207</v>
       </c>
       <c r="B18" s="13" t="n">
         <v>5961</v>
@@ -3859,7 +5265,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>121</v>
+        <v>208</v>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
@@ -3869,24 +5275,24 @@
       <c r="A20" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="29" t="n">
+      <c r="B20" s="34" t="n">
         <f aca="false">Supuestos!B5</f>
         <v>3.5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>122</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>123</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>124</v>
+        <v>211</v>
       </c>
       <c r="B24" s="18" t="n">
         <f aca="false">D10*B20</f>
@@ -3895,7 +5301,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>125</v>
+        <v>212</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">B14*B20</f>
@@ -3904,7 +5310,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>126</v>
+        <v>213</v>
       </c>
       <c r="B26" s="18" t="n">
         <f aca="false">B16+B17</f>
@@ -3913,7 +5319,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>127</v>
+        <v>166</v>
       </c>
       <c r="B27" s="18" t="n">
         <f aca="false">B18</f>
@@ -3922,16 +5328,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="B28" s="28" t="n">
+        <v>214</v>
+      </c>
+      <c r="B28" s="29" t="n">
         <f aca="false">SUM(B24:B27)</f>
         <v>39980.845</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>129</v>
+        <v>215</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -3940,16 +5346,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="B30" s="30" t="n">
+        <v>174</v>
+      </c>
+      <c r="B30" s="36" t="n">
         <f aca="false">B28-B29</f>
         <v>33237.29</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>131</v>
+        <v>175</v>
       </c>
       <c r="B31" s="18" t="n">
         <f aca="false">B30/B20</f>
@@ -3958,7 +5364,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>132</v>
+        <v>216</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3966,24 +5372,24 @@
         <v>2</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>133</v>
+        <v>217</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>134</v>
+        <v>218</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>135</v>
+        <v>219</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>136</v>
+        <v>105</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>137</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>138</v>
+        <v>221</v>
       </c>
       <c r="B35" s="18" t="n">
         <f aca="false">D5</f>
@@ -3997,18 +5403,18 @@
         <f aca="false">C35*$B$30</f>
         <v>22599.2707755844</v>
       </c>
-      <c r="E35" s="31" t="n">
+      <c r="E35" s="35" t="n">
         <f aca="false">B5</f>
         <v>1008</v>
       </c>
-      <c r="F35" s="30" t="n">
+      <c r="F35" s="36" t="n">
         <f aca="false">D35/E35</f>
         <v>22.4199114837147</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>139</v>
+        <v>222</v>
       </c>
       <c r="B36" s="18" t="n">
         <f aca="false">D6</f>
@@ -4022,18 +5428,18 @@
         <f aca="false">C36*$B$30</f>
         <v>2516.52067674348</v>
       </c>
-      <c r="E36" s="31" t="n">
+      <c r="E36" s="35" t="n">
         <f aca="false">B6</f>
         <v>1000</v>
       </c>
-      <c r="F36" s="30" t="n">
+      <c r="F36" s="36" t="n">
         <f aca="false">D36/E36</f>
         <v>2.51652067674348</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>140</v>
+        <v>223</v>
       </c>
       <c r="B37" s="18" t="n">
         <f aca="false">D7</f>
@@ -4047,35 +5453,35 @@
         <f aca="false">C37*$B$30</f>
         <v>8121.49854767215</v>
       </c>
-      <c r="E37" s="31" t="n">
+      <c r="E37" s="35" t="n">
         <f aca="false">B7</f>
         <v>500</v>
       </c>
-      <c r="F37" s="30" t="n">
+      <c r="F37" s="36" t="n">
         <f aca="false">D37/E37</f>
         <v>16.2429970953443</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="25" t="s">
-        <v>141</v>
-      </c>
-      <c r="B38" s="28" t="n">
+        <v>115</v>
+      </c>
+      <c r="B38" s="29" t="n">
         <f aca="false">SUM(B35:B37)</f>
         <v>7264.2</v>
       </c>
-      <c r="C38" s="32" t="n">
+      <c r="C38" s="38" t="n">
         <f aca="false">SUM(C35:C37)</f>
         <v>1</v>
       </c>
-      <c r="D38" s="28" t="n">
+      <c r="D38" s="29" t="n">
         <f aca="false">SUM(D35:D37)</f>
         <v>33237.29</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>142</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Contenedor2: precios recomendados y provision de garantia del Cero
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="229">
   <si>
     <t xml:space="preserve">Resumen - utilidad por pedido (S/)</t>
   </si>
@@ -581,7 +581,7 @@
     <t xml:space="preserve">Reparto: mercaderia directa; flete, gastos locales y agente por volumen (CBM); arancel e impuestos por valor.</t>
   </si>
   <si>
-    <t xml:space="preserve">Margen INDICATIVO por pedido en Lima (S/) - precios PROVISIONALES de la tienda anterior; courier de bultos grandes probablemente mayor</t>
+    <t xml:space="preserve">Margen por pedido en Lima (S/) con precios RECOMENDADOS - courier de bultos grandes probablemente mayor</t>
   </si>
   <si>
     <t xml:space="preserve">Bidon 22 L</t>
@@ -596,13 +596,25 @@
     <t xml:space="preserve">elvo· Cero</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio de venta (con IGV) - provisional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Publicidad (1 = si, 0 = no)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No incluye garantia ni postventa del Cero, costo de courier de bultos grandes, ni la partida arancelaria definitiva. Precios: bidon 22 L S/ 198, bidon 16 L S/ 120 y kit S/ 85 son los de la tienda anterior (AQA); Cero S/ 1,999 del listado actual.</t>
+    <t xml:space="preserve">Precio de venta (con IGV) - recomendado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provision de garantia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publicidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrada: provision de garantia (% del precio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrada: lleva publicidad (1 = si, 0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precios recomendados: bidon 22 L S/ 219, bidon 16 L S/ 159, kit S/ 85, Cero S/ 2,299. Referencias (Sodimac Peru, busqueda oct-2026): bidon mineralizador 16 L S/ 159.90 (lista S/ 249); repuestos de filtro S/ 72.90-84.90; osmosis inversa bajo mesada de 5 etapas en Falabella Peru S/ 1,090-1,499.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garantia del Cero: 12 meses; provision de 4% del precio (~S/ 92) como SUGERENCIA, sin dato historico propio. No incluye courier de bultos grandes.</t>
   </si>
   <si>
     <t xml:space="preserve">Costo puesto en Lima - embarque Ningbo (llegada 22-abr-2026)</t>
@@ -856,7 +868,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1006,6 +1018,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3964,7 +3980,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -4838,16 +4854,16 @@
         <v>190</v>
       </c>
       <c r="B80" s="37" t="n">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="C80" s="37" t="n">
-        <v>120</v>
+        <v>159</v>
       </c>
       <c r="D80" s="37" t="n">
         <v>85</v>
       </c>
       <c r="E80" s="37" t="n">
-        <v>1999</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4856,11 +4872,11 @@
       </c>
       <c r="B81" s="24" t="n">
         <f aca="false">B80/(1+Supuestos!$B$4)</f>
-        <v>167.796610169492</v>
+        <v>185.593220338983</v>
       </c>
       <c r="C81" s="24" t="n">
         <f aca="false">C80/(1+Supuestos!$B$4)</f>
-        <v>101.694915254237</v>
+        <v>134.745762711864</v>
       </c>
       <c r="D81" s="24" t="n">
         <f aca="false">D80/(1+Supuestos!$B$4)</f>
@@ -4868,7 +4884,7 @@
       </c>
       <c r="E81" s="24" t="n">
         <f aca="false">E80/(1+Supuestos!$B$4)</f>
-        <v>1694.06779661017</v>
+        <v>1948.30508474576</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4898,11 +4914,11 @@
       </c>
       <c r="B83" s="6" t="n">
         <f aca="false">-(B80*Supuestos!$B$31+Supuestos!$B$32)</f>
-        <v>-6.47366</v>
+        <v>-7.10723</v>
       </c>
       <c r="C83" s="6" t="n">
         <f aca="false">-(C80*Supuestos!$B$31+Supuestos!$B$32)</f>
-        <v>-4.1204</v>
+        <v>-5.29703</v>
       </c>
       <c r="D83" s="6" t="n">
         <f aca="false">-(D80*Supuestos!$B$31+Supuestos!$B$32)</f>
@@ -4910,7 +4926,7 @@
       </c>
       <c r="E83" s="6" t="n">
         <f aca="false">-(E80*Supuestos!$B$31+Supuestos!$B$32)</f>
-        <v>-60.80983</v>
+        <v>-69.86083</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4957,129 +4973,193 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B86" s="26" t="n">
-        <f aca="false">SUM(B81:B85)</f>
-        <v>97.7739987917178</v>
-      </c>
-      <c r="C86" s="26" t="n">
-        <f aca="false">SUM(C81:C85)</f>
-        <v>41.7329235311725</v>
-      </c>
-      <c r="D86" s="26" t="n">
-        <f aca="false">SUM(D81:D85)</f>
-        <v>42.0625714410721</v>
-      </c>
-      <c r="E86" s="26" t="n">
-        <f aca="false">SUM(E81:E85)</f>
-        <v>982.134893713872</v>
+        <v>191</v>
+      </c>
+      <c r="B86" s="24" t="n">
+        <f aca="false">-B80*B94</f>
+        <v>-0</v>
+      </c>
+      <c r="C86" s="24" t="n">
+        <f aca="false">-C80*C94</f>
+        <v>-0</v>
+      </c>
+      <c r="D86" s="24" t="n">
+        <f aca="false">-D80*D94</f>
+        <v>-0</v>
+      </c>
+      <c r="E86" s="24" t="n">
+        <f aca="false">-E80*E94</f>
+        <v>-91.96</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B87" s="26" t="n">
+        <f aca="false">SUM(B81:B86)</f>
+        <v>114.937038961209</v>
+      </c>
+      <c r="C87" s="26" t="n">
+        <f aca="false">SUM(C81:C86)</f>
+        <v>73.6071409887997</v>
+      </c>
+      <c r="D87" s="26" t="n">
+        <f aca="false">SUM(D81:D86)</f>
+        <v>42.0625714410721</v>
+      </c>
+      <c r="E87" s="26" t="n">
+        <f aca="false">SUM(E81:E86)</f>
+        <v>1135.36118184947</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B87" s="24" t="n">
-        <f aca="false">-(1-Supuestos!$B$7)*(B81+B82+B83)</f>
-        <v>-17.0660998187577</v>
-      </c>
-      <c r="C87" s="24" t="n">
-        <f aca="false">-(1-Supuestos!$B$7)*(C81+C82+C83)</f>
-        <v>-8.65993852967588</v>
-      </c>
-      <c r="D87" s="24" t="n">
-        <f aca="false">-(1-Supuestos!$B$7)*(D81+D82+D83)</f>
+      <c r="B88" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(B81+B82+B83+B86)</f>
+        <v>-19.6405558441814</v>
+      </c>
+      <c r="C88" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(C81+C82+C83+C86)</f>
+        <v>-13.44107114832</v>
+      </c>
+      <c r="D88" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(D81+D82+D83+D86)</f>
         <v>-8.70938571616081</v>
       </c>
-      <c r="E87" s="24" t="n">
-        <f aca="false">-(1-Supuestos!$B$7)*(E81+E82+E83)</f>
-        <v>-149.720234057081</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="25" t="s">
+      <c r="E88" s="24" t="n">
+        <f aca="false">-(1-Supuestos!$B$7)*(E81+E82+E83+E86)</f>
+        <v>-172.70417727742</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="B88" s="26" t="n">
-        <f aca="false">B86+B87</f>
-        <v>80.7078989729601</v>
-      </c>
-      <c r="C88" s="26" t="n">
-        <f aca="false">C86+C87</f>
-        <v>33.0729850014967</v>
-      </c>
-      <c r="D88" s="26" t="n">
-        <f aca="false">D86+D87</f>
+      <c r="B89" s="26" t="n">
+        <f aca="false">B87+B88</f>
+        <v>95.2964831170279</v>
+      </c>
+      <c r="C89" s="26" t="n">
+        <f aca="false">C87+C88</f>
+        <v>60.1660698404797</v>
+      </c>
+      <c r="D89" s="26" t="n">
+        <f aca="false">D87+D88</f>
         <v>33.3531857249113</v>
       </c>
-      <c r="E88" s="26" t="n">
-        <f aca="false">E86+E87</f>
-        <v>832.414659656791</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="B89" s="23" t="n">
+      <c r="E89" s="26" t="n">
+        <f aca="false">E87+E88</f>
+        <v>962.657004572045</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B90" s="6" t="n">
+        <f aca="false">-Supuestos!$B$6*B95</f>
+        <v>-31</v>
+      </c>
+      <c r="C90" s="6" t="n">
+        <f aca="false">-Supuestos!$B$6*C95</f>
+        <v>-31</v>
+      </c>
+      <c r="D90" s="6" t="n">
+        <f aca="false">-Supuestos!$B$6*D95</f>
+        <v>-0</v>
+      </c>
+      <c r="E90" s="6" t="n">
+        <f aca="false">-Supuestos!$B$6*E95</f>
+        <v>-31</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="B91" s="27" t="n">
+        <f aca="false">B89+B90</f>
+        <v>64.2964831170279</v>
+      </c>
+      <c r="C91" s="27" t="n">
+        <f aca="false">C89+C90</f>
+        <v>29.1660698404797</v>
+      </c>
+      <c r="D91" s="27" t="n">
+        <f aca="false">D89+D90</f>
+        <v>33.3531857249113</v>
+      </c>
+      <c r="E91" s="27" t="n">
+        <f aca="false">E89+E90</f>
+        <v>931.657004572045</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B92" s="19" t="n">
+        <f aca="false">B91/B80</f>
+        <v>0.293591247109717</v>
+      </c>
+      <c r="C92" s="19" t="n">
+        <f aca="false">C91/C80</f>
+        <v>0.183434401512451</v>
+      </c>
+      <c r="D92" s="19" t="n">
+        <f aca="false">D91/D80</f>
+        <v>0.392390420293074</v>
+      </c>
+      <c r="E92" s="19" t="n">
+        <f aca="false">E91/E80</f>
+        <v>0.405244456099193</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="B94" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="38" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="B95" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="C89" s="23" t="n">
+      <c r="C95" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D89" s="23" t="n">
+      <c r="D95" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="E89" s="23" t="n">
+      <c r="E95" s="23" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="B90" s="27" t="n">
-        <f aca="false">B88-Supuestos!$B$6*B89</f>
-        <v>49.7078989729601</v>
-      </c>
-      <c r="C90" s="27" t="n">
-        <f aca="false">C88-Supuestos!$B$6*C89</f>
-        <v>2.07298500149665</v>
-      </c>
-      <c r="D90" s="27" t="n">
-        <f aca="false">D88-Supuestos!$B$6*D89</f>
-        <v>33.3531857249113</v>
-      </c>
-      <c r="E90" s="27" t="n">
-        <f aca="false">E88-Supuestos!$B$6*E89</f>
-        <v>801.414659656791</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="B91" s="19" t="n">
-        <f aca="false">B90/B80</f>
-        <v>0.25104999481293</v>
-      </c>
-      <c r="C91" s="19" t="n">
-        <f aca="false">C90/C80</f>
-        <v>0.0172748750124721</v>
-      </c>
-      <c r="D91" s="19" t="n">
-        <f aca="false">D90/D80</f>
-        <v>0.392390420293074</v>
-      </c>
-      <c r="E91" s="19" t="n">
-        <f aca="false">E90/E80</f>
-        <v>0.400907783720256</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="2" t="s">
-        <v>192</v>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="2" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -5107,12 +5187,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5131,7 +5211,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>1008</v>
@@ -5146,7 +5226,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1000</v>
@@ -5161,7 +5241,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>500</v>
@@ -5176,7 +5256,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>5</v>
@@ -5191,7 +5271,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>1</v>
@@ -5206,7 +5286,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D10" s="29" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -5215,17 +5295,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>1135.87</v>
@@ -5233,7 +5313,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>135.13</v>
@@ -5241,7 +5321,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>1720</v>
@@ -5249,7 +5329,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B17" s="13" t="n">
         <v>309.6</v>
@@ -5257,7 +5337,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B18" s="13" t="n">
         <v>5961</v>
@@ -5265,7 +5345,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
@@ -5282,17 +5362,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B24" s="18" t="n">
         <f aca="false">D10*B20</f>
@@ -5301,7 +5381,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">B14*B20</f>
@@ -5310,7 +5390,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B26" s="18" t="n">
         <f aca="false">B16+B17</f>
@@ -5328,7 +5408,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="25" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B28" s="29" t="n">
         <f aca="false">SUM(B24:B27)</f>
@@ -5337,7 +5417,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -5364,7 +5444,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5372,24 +5452,24 @@
         <v>2</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B35" s="18" t="n">
         <f aca="false">D5</f>
@@ -5414,7 +5494,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B36" s="18" t="n">
         <f aca="false">D6</f>
@@ -5439,7 +5519,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B37" s="18" t="n">
         <f aca="false">D7</f>
@@ -5470,7 +5550,7 @@
         <f aca="false">SUM(B35:B37)</f>
         <v>7264.2</v>
       </c>
-      <c r="C38" s="38" t="n">
+      <c r="C38" s="39" t="n">
         <f aca="false">SUM(C35:C37)</f>
         <v>1</v>
       </c>
@@ -5481,7 +5561,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Entrega efectiva en Lima a 80% y hoja Courier_Hub (comparacion con The Hub)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Supuestos" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Desglose" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Contenedor2" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Costo_Lima" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Courier_Hub" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Costo_Lima" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="268">
   <si>
     <t xml:space="preserve">Resumen - utilidad por pedido (S/)</t>
   </si>
@@ -92,7 +93,7 @@
     <t xml:space="preserve">Entrega efectiva en Lima</t>
   </si>
   <si>
-    <t xml:space="preserve">Dato del usuario (85%).</t>
+    <t xml:space="preserve">Usuario: todos los pedidos de Lima son contraentrega y se entrega el 80%. (El 85% inicial era el promedio con provincia.)</t>
   </si>
   <si>
     <t xml:space="preserve">Entrega efectiva en provincia</t>
@@ -615,6 +616,123 @@
   </si>
   <si>
     <t xml:space="preserve">Garantia del Cero: 12 meses; provision de 4% del precio (~S/ 92) como SUGERENCIA, sin dato historico propio. No incluye courier de bultos grandes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Hub vs operacion actual - pedidos en Lima, todos contraentrega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azul = dato editable. Verde = viene de otra hoja. Fuentes: proforma The Hub 21-abr-2026 y Anexo 3 de tarifas. Los precios de The Hub no incluyen IGV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operacion actual (empaque + courier + almacen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almacen prorrateado por pedido (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega efectiva actual en Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Hub (Business Standard)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestion por orden (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Envio estandar Lima urbano, hasta 3 kg (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proforma y tabla de codigos postales: 7.5; hoja Tarifa Lima: 8.0. Confirmar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kg adicional sobre 3 kg (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urbano 1.5, periferico 2.0, periferico 2: 2.2. Peso facturable = largo x alto x ancho / 5000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobro contraentrega (% del valor del orden)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proforma: manejo de dinero y seguro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cobra el contraentrega tambien en pedidos NO entregados? (1 = si, 0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: solo cobra lo que cobra. Confirmar con The Hub.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almacen (US$ por m3 al mes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado por el usuario: es mensual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meses que el stock permanece en The Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El resto queda en almacen propio y se envia por tandas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega efectiva con The Hub en Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Igual a la actual para comparar costos. Cambiar para probar un alza.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de cambio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparacion por pedido colocado en Lima (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio de venta (con IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margen por pedido entregado, antes de logistica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volumen por unidad (m3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso facturable (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTUAL: logistica por pedido colocado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTUAL: utilidad antes de publicidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HUB: gestion + envio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HUB: cobro contraentrega esperado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HUB: almacen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HUB: logistica por pedido colocado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HUB: utilidad antes de publicidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia Hub - actual (utilidad por pedido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alza de entrega efectiva que iguala (puntos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobro contraentrega que iguala (% del valor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura: si la diferencia es negativa, The Hub cuesta mas a igual tasa de entrega. La fila "alza de entrega" dice cuantos puntos debe mejorar la entrega para compensar; la ultima fila, el cobro contraentrega con el que quedarias igual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para bidones y Cero la operacion actual es solo una referencia: se uso el mismo courier de S/ 12.5, que probablemente es bajo para esos bultos. No incluye el beneficio tributario de la factura de The Hub (IGV y gasto deducible) ni cobros de entrega fallida.</t>
   </si>
   <si>
     <t xml:space="preserve">Costo puesto en Lima - embarque Ningbo (llegada 22-abr-2026)</t>
@@ -717,7 +835,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0;\(#,##0.0\);\-"/>
@@ -727,6 +845,8 @@
     <numFmt numFmtId="170" formatCode="0"/>
     <numFmt numFmtId="171" formatCode="0.00%"/>
     <numFmt numFmtId="172" formatCode="0.00"/>
+    <numFmt numFmtId="173" formatCode="0.0"/>
+    <numFmt numFmtId="174" formatCode="0.0000"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -868,7 +988,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1025,7 +1145,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="173" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1335,15 +1467,15 @@
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">Desglose!B21</f>
-        <v>172.231725671046</v>
+        <v>161.159271219808</v>
       </c>
       <c r="D5" s="6" t="n">
         <f aca="false">Desglose!B23</f>
-        <v>141.231725671046</v>
+        <v>130.159271219808</v>
       </c>
       <c r="E5" s="7" t="n">
         <f aca="false">Desglose!B24</f>
-        <v>0.472346908598816</v>
+        <v>0.435315288360562</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">Desglose!B36</f>
@@ -1369,15 +1501,15 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">Desglose!C21</f>
-        <v>204.827407248356</v>
+        <v>191.837559763159</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">Desglose!C23</f>
-        <v>173.827407248356</v>
+        <v>160.837559763159</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">Desglose!C24</f>
-        <v>0.498072800138557</v>
+        <v>0.460852606771229</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">Desglose!C36</f>
@@ -1403,15 +1535,15 @@
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">Desglose!D21</f>
-        <v>235.284046250435</v>
+        <v>220.502631765115</v>
       </c>
       <c r="D7" s="6" t="n">
         <f aca="false">Desglose!D23</f>
-        <v>204.284046250435</v>
+        <v>189.502631765115</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">Desglose!D24</f>
-        <v>0.51199009085322</v>
+        <v>0.47494393926094</v>
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">Desglose!D36</f>
@@ -1437,15 +1569,15 @@
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">Desglose!E21</f>
-        <v>102.762277365961</v>
+        <v>95.7762610503164</v>
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">Desglose!E23</f>
-        <v>71.7622773659612</v>
+        <v>64.7762610503164</v>
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">Desglose!E24</f>
-        <v>0.360614459125433</v>
+        <v>0.325508849499078</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">Desglose!E36</f>
@@ -1471,15 +1603,15 @@
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">Desglose!F21</f>
-        <v>135.357958943272</v>
+        <v>126.454549593667</v>
       </c>
       <c r="D9" s="6" t="n">
         <f aca="false">Desglose!F23</f>
-        <v>104.357958943272</v>
+        <v>95.4545495936674</v>
       </c>
       <c r="E9" s="7" t="n">
         <f aca="false">Desglose!F24</f>
-        <v>0.41910826884848</v>
+        <v>0.383351604793845</v>
       </c>
       <c r="F9" s="6" t="n">
         <f aca="false">Desglose!F36</f>
@@ -1505,15 +1637,15 @@
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">Desglose!G21</f>
-        <v>186.655432436876</v>
+        <v>174.734524646471</v>
       </c>
       <c r="D10" s="6" t="n">
         <f aca="false">Desglose!G23</f>
-        <v>155.655432436876</v>
+        <v>143.734524646471</v>
       </c>
       <c r="E10" s="7" t="n">
         <f aca="false">Desglose!G24</f>
-        <v>0.473116815917555</v>
+        <v>0.43688305363669</v>
       </c>
       <c r="F10" s="6" t="n">
         <f aca="false">Desglose!G36</f>
@@ -1539,15 +1671,15 @@
       </c>
       <c r="C11" s="6" t="n">
         <f aca="false">Desglose!H21</f>
-        <v>38.5432062909913</v>
+        <v>35.3347823915212</v>
       </c>
       <c r="D11" s="6" t="n">
         <f aca="false">Desglose!H23</f>
-        <v>7.54320629099126</v>
+        <v>4.33478239152119</v>
       </c>
       <c r="E11" s="7" t="n">
         <f aca="false">Desglose!H24</f>
-        <v>0.0761940029393056</v>
+        <v>0.0437856807224362</v>
       </c>
       <c r="F11" s="6" t="n">
         <f aca="false">Desglose!H36</f>
@@ -1573,15 +1705,15 @@
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">Desglose!I21</f>
-        <v>24.7366587599486</v>
+        <v>22.3403847152458</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">Desglose!I23</f>
-        <v>-6.26334124005139</v>
+        <v>-8.65961528475424</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">Desglose!I24</f>
-        <v>-0.0632660731318322</v>
+        <v>-0.0874708614621641</v>
       </c>
       <c r="F12" s="6" t="n">
         <f aca="false">Desglose!I36</f>
@@ -1607,15 +1739,15 @@
       </c>
       <c r="C13" s="6" t="n">
         <f aca="false">Desglose!J21</f>
-        <v>52.6991223419311</v>
+        <v>48.6579974982881</v>
       </c>
       <c r="D13" s="6" t="n">
         <f aca="false">Desglose!J23</f>
-        <v>21.6991223419311</v>
+        <v>17.6579974982881</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">Desglose!J24</f>
-        <v>0.121224147161626</v>
+        <v>0.0986480307166934</v>
       </c>
       <c r="F13" s="6" t="n">
         <f aca="false">Desglose!J36</f>
@@ -1641,15 +1773,15 @@
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">Desglose!K21</f>
-        <v>73.7146410934052</v>
+        <v>68.4373092643813</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">Desglose!K23</f>
-        <v>42.7146410934052</v>
+        <v>37.4373092643813</v>
       </c>
       <c r="E14" s="7" t="n">
         <f aca="false">Desglose!K24</f>
-        <v>0.171544743347009</v>
+        <v>0.150350639615989</v>
       </c>
       <c r="F14" s="6" t="n">
         <f aca="false">Desglose!K36</f>
@@ -1675,15 +1807,15 @@
       </c>
       <c r="C15" s="6" t="n">
         <f aca="false">Desglose!L21</f>
-        <v>119.680159551887</v>
+        <v>111.698973695893</v>
       </c>
       <c r="D15" s="6" t="n">
         <f aca="false">Desglose!L23</f>
-        <v>119.680159551887</v>
+        <v>111.698973695893</v>
       </c>
       <c r="E15" s="7" t="n">
         <f aca="false">Desglose!L24</f>
-        <v>0.601407836944154</v>
+        <v>0.561301375356248</v>
       </c>
       <c r="F15" s="6" t="n">
         <f aca="false">Desglose!L36</f>
@@ -1709,15 +1841,15 @@
       </c>
       <c r="C16" s="6" t="n">
         <f aca="false">Desglose!M21</f>
-        <v>50.210711246802</v>
+        <v>46.3159635264018</v>
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">Desglose!M23</f>
-        <v>50.210711246802</v>
+        <v>46.3159635264018</v>
       </c>
       <c r="E16" s="7" t="n">
         <f aca="false">Desglose!M24</f>
-        <v>0.507178901482848</v>
+        <v>0.4678380154182</v>
       </c>
       <c r="F16" s="6" t="n">
         <f aca="false">Desglose!M36</f>
@@ -1743,15 +1875,15 @@
       </c>
       <c r="C17" s="6" t="n">
         <f aca="false">Desglose!N21</f>
-        <v>3.80848213844888</v>
+        <v>2.64327730677542</v>
       </c>
       <c r="D17" s="6" t="n">
         <f aca="false">Desglose!N23</f>
-        <v>3.80848213844888</v>
+        <v>2.64327730677542</v>
       </c>
       <c r="E17" s="7" t="n">
         <f aca="false">Desglose!N24</f>
-        <v>0.077724125274467</v>
+        <v>0.0539444348321514</v>
       </c>
       <c r="F17" s="6" t="n">
         <f aca="false">Desglose!N36</f>
@@ -1855,7 +1987,7 @@
         <v>21</v>
       </c>
       <c r="B7" s="11" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>22</v>
@@ -2916,55 +3048,55 @@
       </c>
       <c r="B20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(B14+B15+B16)</f>
-        <v>-33.217363353714</v>
+        <v>-44.289817804952</v>
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(C14+C15+C16)</f>
-        <v>-38.9695424555923</v>
+        <v>-51.9593899407897</v>
       </c>
       <c r="D20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(D14+D15+D16)</f>
-        <v>-44.3442434559591</v>
+        <v>-59.1256579412788</v>
       </c>
       <c r="E20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(E14+E15+E16)</f>
-        <v>-20.9580489469343</v>
+        <v>-27.9440652625791</v>
       </c>
       <c r="F20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(F14+F15+F16)</f>
-        <v>-26.7102280488126</v>
+        <v>-35.6136373984168</v>
       </c>
       <c r="G20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(G14+G15+G16)</f>
-        <v>-35.7627233712133</v>
+        <v>-47.6836311616178</v>
       </c>
       <c r="H20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(H14+H15+H16)</f>
-        <v>-9.62527169841022</v>
+        <v>-12.8336955978803</v>
       </c>
       <c r="I20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(I14+I15+I16)</f>
-        <v>-7.18882213410858</v>
+        <v>-9.58509617881144</v>
       </c>
       <c r="J20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(J14+J15+J16)</f>
-        <v>-12.123374530929</v>
+        <v>-16.164499374572</v>
       </c>
       <c r="K20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(K14+K15+K16)</f>
-        <v>-15.8319954870715</v>
+        <v>-21.1093273160953</v>
       </c>
       <c r="L20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(L14+L15+L16)</f>
-        <v>-23.94355756798</v>
+        <v>-31.9247434239733</v>
       </c>
       <c r="M20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(M14+M15+M16)</f>
-        <v>-11.6842431612003</v>
+        <v>-15.5789908816005</v>
       </c>
       <c r="N20" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(N14+N15+N16)</f>
-        <v>-3.49561449502039</v>
+        <v>-4.66081932669385</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2973,55 +3105,55 @@
       </c>
       <c r="B21" s="26" t="n">
         <f aca="false">B19+B20</f>
-        <v>172.231725671046</v>
+        <v>161.159271219808</v>
       </c>
       <c r="C21" s="26" t="n">
         <f aca="false">C19+C20</f>
-        <v>204.827407248356</v>
+        <v>191.837559763159</v>
       </c>
       <c r="D21" s="26" t="n">
         <f aca="false">D19+D20</f>
-        <v>235.284046250435</v>
+        <v>220.502631765115</v>
       </c>
       <c r="E21" s="26" t="n">
         <f aca="false">E19+E20</f>
-        <v>102.762277365961</v>
+        <v>95.7762610503164</v>
       </c>
       <c r="F21" s="26" t="n">
         <f aca="false">F19+F20</f>
-        <v>135.357958943272</v>
+        <v>126.454549593667</v>
       </c>
       <c r="G21" s="26" t="n">
         <f aca="false">G19+G20</f>
-        <v>186.655432436876</v>
+        <v>174.734524646471</v>
       </c>
       <c r="H21" s="26" t="n">
         <f aca="false">H19+H20</f>
-        <v>38.5432062909913</v>
+        <v>35.3347823915212</v>
       </c>
       <c r="I21" s="26" t="n">
         <f aca="false">I19+I20</f>
-        <v>24.7366587599486</v>
+        <v>22.3403847152458</v>
       </c>
       <c r="J21" s="26" t="n">
         <f aca="false">J19+J20</f>
-        <v>52.6991223419311</v>
+        <v>48.6579974982881</v>
       </c>
       <c r="K21" s="26" t="n">
         <f aca="false">K19+K20</f>
-        <v>73.7146410934052</v>
+        <v>68.4373092643813</v>
       </c>
       <c r="L21" s="26" t="n">
         <f aca="false">L19+L20</f>
-        <v>119.680159551887</v>
+        <v>111.698973695893</v>
       </c>
       <c r="M21" s="26" t="n">
         <f aca="false">M19+M20</f>
-        <v>50.210711246802</v>
+        <v>46.3159635264018</v>
       </c>
       <c r="N21" s="26" t="n">
         <f aca="false">N19+N20</f>
-        <v>3.80848213844888</v>
+        <v>2.64327730677542</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3087,55 +3219,55 @@
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">B21+B22</f>
-        <v>141.231725671046</v>
+        <v>130.159271219808</v>
       </c>
       <c r="C23" s="27" t="n">
         <f aca="false">C21+C22</f>
-        <v>173.827407248356</v>
+        <v>160.837559763159</v>
       </c>
       <c r="D23" s="27" t="n">
         <f aca="false">D21+D22</f>
-        <v>204.284046250435</v>
+        <v>189.502631765115</v>
       </c>
       <c r="E23" s="27" t="n">
         <f aca="false">E21+E22</f>
-        <v>71.7622773659612</v>
+        <v>64.7762610503164</v>
       </c>
       <c r="F23" s="27" t="n">
         <f aca="false">F21+F22</f>
-        <v>104.357958943272</v>
+        <v>95.4545495936674</v>
       </c>
       <c r="G23" s="27" t="n">
         <f aca="false">G21+G22</f>
-        <v>155.655432436876</v>
+        <v>143.734524646471</v>
       </c>
       <c r="H23" s="27" t="n">
         <f aca="false">H21+H22</f>
-        <v>7.54320629099126</v>
+        <v>4.33478239152119</v>
       </c>
       <c r="I23" s="27" t="n">
         <f aca="false">I21+I22</f>
-        <v>-6.26334124005139</v>
+        <v>-8.65961528475424</v>
       </c>
       <c r="J23" s="27" t="n">
         <f aca="false">J21+J22</f>
-        <v>21.6991223419311</v>
+        <v>17.6579974982881</v>
       </c>
       <c r="K23" s="27" t="n">
         <f aca="false">K21+K22</f>
-        <v>42.7146410934052</v>
+        <v>37.4373092643813</v>
       </c>
       <c r="L23" s="27" t="n">
         <f aca="false">L21+L22</f>
-        <v>119.680159551887</v>
+        <v>111.698973695893</v>
       </c>
       <c r="M23" s="27" t="n">
         <f aca="false">M21+M22</f>
-        <v>50.210711246802</v>
+        <v>46.3159635264018</v>
       </c>
       <c r="N23" s="27" t="n">
         <f aca="false">N21+N22</f>
-        <v>3.80848213844888</v>
+        <v>2.64327730677542</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3144,55 +3276,55 @@
       </c>
       <c r="B24" s="19" t="n">
         <f aca="false">B23/B5</f>
-        <v>0.472346908598816</v>
+        <v>0.435315288360562</v>
       </c>
       <c r="C24" s="19" t="n">
         <f aca="false">C23/C5</f>
-        <v>0.498072800138557</v>
+        <v>0.460852606771229</v>
       </c>
       <c r="D24" s="19" t="n">
         <f aca="false">D23/D5</f>
-        <v>0.51199009085322</v>
+        <v>0.47494393926094</v>
       </c>
       <c r="E24" s="19" t="n">
         <f aca="false">E23/E5</f>
-        <v>0.360614459125433</v>
+        <v>0.325508849499078</v>
       </c>
       <c r="F24" s="19" t="n">
         <f aca="false">F23/F5</f>
-        <v>0.41910826884848</v>
+        <v>0.383351604793845</v>
       </c>
       <c r="G24" s="19" t="n">
         <f aca="false">G23/G5</f>
-        <v>0.473116815917555</v>
+        <v>0.43688305363669</v>
       </c>
       <c r="H24" s="19" t="n">
         <f aca="false">H23/H5</f>
-        <v>0.0761940029393056</v>
+        <v>0.0437856807224362</v>
       </c>
       <c r="I24" s="19" t="n">
         <f aca="false">I23/I5</f>
-        <v>-0.0632660731318322</v>
+        <v>-0.0874708614621641</v>
       </c>
       <c r="J24" s="19" t="n">
         <f aca="false">J23/J5</f>
-        <v>0.121224147161626</v>
+        <v>0.0986480307166934</v>
       </c>
       <c r="K24" s="19" t="n">
         <f aca="false">K23/K5</f>
-        <v>0.171544743347009</v>
+        <v>0.150350639615989</v>
       </c>
       <c r="L24" s="19" t="n">
         <f aca="false">L23/L5</f>
-        <v>0.601407836944154</v>
+        <v>0.561301375356248</v>
       </c>
       <c r="M24" s="19" t="n">
         <f aca="false">M23/M5</f>
-        <v>0.507178901482848</v>
+        <v>0.4678380154182</v>
       </c>
       <c r="N24" s="19" t="n">
         <f aca="false">N23/N5</f>
-        <v>0.077724125274467</v>
+        <v>0.0539444348321514</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3258,55 +3390,55 @@
       </c>
       <c r="B26" s="26" t="n">
         <f aca="false">B23+B25</f>
-        <v>137.231725671046</v>
+        <v>126.159271219808</v>
       </c>
       <c r="C26" s="26" t="n">
         <f aca="false">C23+C25</f>
-        <v>169.827407248356</v>
+        <v>156.837559763159</v>
       </c>
       <c r="D26" s="26" t="n">
         <f aca="false">D23+D25</f>
-        <v>200.284046250435</v>
+        <v>185.502631765115</v>
       </c>
       <c r="E26" s="26" t="n">
         <f aca="false">E23+E25</f>
-        <v>67.7622773659612</v>
+        <v>60.7762610503164</v>
       </c>
       <c r="F26" s="26" t="n">
         <f aca="false">F23+F25</f>
-        <v>100.357958943272</v>
+        <v>91.4545495936674</v>
       </c>
       <c r="G26" s="26" t="n">
         <f aca="false">G23+G25</f>
-        <v>151.655432436876</v>
+        <v>139.734524646471</v>
       </c>
       <c r="H26" s="26" t="n">
         <f aca="false">H23+H25</f>
-        <v>3.54320629099126</v>
+        <v>0.334782391521188</v>
       </c>
       <c r="I26" s="26" t="n">
         <f aca="false">I23+I25</f>
-        <v>-10.2633412400514</v>
+        <v>-12.6596152847542</v>
       </c>
       <c r="J26" s="26" t="n">
         <f aca="false">J23+J25</f>
-        <v>17.6991223419311</v>
+        <v>13.6579974982881</v>
       </c>
       <c r="K26" s="26" t="n">
         <f aca="false">K23+K25</f>
-        <v>38.7146410934052</v>
+        <v>33.4373092643813</v>
       </c>
       <c r="L26" s="26" t="n">
         <f aca="false">L23+L25</f>
-        <v>115.680159551887</v>
+        <v>107.698973695893</v>
       </c>
       <c r="M26" s="26" t="n">
         <f aca="false">M23+M25</f>
-        <v>46.210711246802</v>
+        <v>42.3159635264018</v>
       </c>
       <c r="N26" s="26" t="n">
         <f aca="false">N23+N25</f>
-        <v>-0.191517861551117</v>
+        <v>-1.35672269322458</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5019,19 +5151,19 @@
       </c>
       <c r="B88" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(B81+B82+B83+B86)</f>
-        <v>-19.6405558441814</v>
+        <v>-26.1874077922419</v>
       </c>
       <c r="C88" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(C81+C82+C83+C86)</f>
-        <v>-13.44107114832</v>
+        <v>-17.9214281977599</v>
       </c>
       <c r="D88" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(D81+D82+D83+D86)</f>
-        <v>-8.70938571616081</v>
+        <v>-11.6125142882144</v>
       </c>
       <c r="E88" s="24" t="n">
         <f aca="false">-(1-Supuestos!$B$7)*(E81+E82+E83+E86)</f>
-        <v>-172.70417727742</v>
+        <v>-230.272236369893</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5040,19 +5172,19 @@
       </c>
       <c r="B89" s="26" t="n">
         <f aca="false">B87+B88</f>
-        <v>95.2964831170279</v>
+        <v>88.7496311689675</v>
       </c>
       <c r="C89" s="26" t="n">
         <f aca="false">C87+C88</f>
-        <v>60.1660698404797</v>
+        <v>55.6857127910397</v>
       </c>
       <c r="D89" s="26" t="n">
         <f aca="false">D87+D88</f>
-        <v>33.3531857249113</v>
+        <v>30.4500571528577</v>
       </c>
       <c r="E89" s="26" t="n">
         <f aca="false">E87+E88</f>
-        <v>962.657004572045</v>
+        <v>905.088945479572</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5082,19 +5214,19 @@
       </c>
       <c r="B91" s="27" t="n">
         <f aca="false">B89+B90</f>
-        <v>64.2964831170279</v>
+        <v>57.7496311689675</v>
       </c>
       <c r="C91" s="27" t="n">
         <f aca="false">C89+C90</f>
-        <v>29.1660698404797</v>
+        <v>24.6857127910397</v>
       </c>
       <c r="D91" s="27" t="n">
         <f aca="false">D89+D90</f>
-        <v>33.3531857249113</v>
+        <v>30.4500571528577</v>
       </c>
       <c r="E91" s="27" t="n">
         <f aca="false">E89+E90</f>
-        <v>931.657004572045</v>
+        <v>874.088945479572</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5103,19 +5235,19 @@
       </c>
       <c r="B92" s="19" t="n">
         <f aca="false">B91/B80</f>
-        <v>0.293591247109717</v>
+        <v>0.26369694597702</v>
       </c>
       <c r="C92" s="19" t="n">
         <f aca="false">C91/C80</f>
-        <v>0.183434401512451</v>
+        <v>0.155256055289558</v>
       </c>
       <c r="D92" s="19" t="n">
         <f aca="false">D91/D80</f>
-        <v>0.392390420293074</v>
+        <v>0.358235966504208</v>
       </c>
       <c r="E92" s="19" t="n">
         <f aca="false">E91/E80</f>
-        <v>0.405244456099193</v>
+        <v>0.380203978025042</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5178,6 +5310,630 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="14" t="n">
+        <f aca="false">Supuestos!B16</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="14" t="n">
+        <f aca="false">Supuestos!B18</f>
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="B7" s="14" t="n">
+        <f aca="false">Supuestos!B38</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <f aca="false">Supuestos!B7</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="B16" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="B17" s="39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="B18" s="38" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="B19" s="34" t="n">
+        <f aca="false">Supuestos!B5</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <f aca="false">Desglose!B5</f>
+        <v>299</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <f aca="false">Desglose!C5</f>
+        <v>349</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <f aca="false">Desglose!D5</f>
+        <v>399</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <f aca="false">Contenedor2!B80</f>
+        <v>219</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <f aca="false">Contenedor2!C80</f>
+        <v>159</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <f aca="false">Contenedor2!E80</f>
+        <v>2299</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <f aca="false">Desglose!B14+Desglose!B15+Desglose!B16</f>
+        <v>221.44908902476</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <f aca="false">Desglose!C14+Desglose!C15+Desglose!C16</f>
+        <v>259.796949703949</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <f aca="false">Desglose!D14+Desglose!D15+Desglose!D16</f>
+        <v>295.628289706394</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <f aca="false">Contenedor2!B81+Contenedor2!B82+Contenedor2!B83+Contenedor2!B86</f>
+        <v>130.937038961209</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <f aca="false">Contenedor2!C81+Contenedor2!C82+Contenedor2!C83+Contenedor2!C86</f>
+        <v>89.6071409887996</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <f aca="false">Contenedor2!E81+Contenedor2!E82+Contenedor2!E83+Contenedor2!E86</f>
+        <v>1151.36118184947</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="C25" s="40" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="D25" s="40" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="E25" s="40" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="F25" s="40" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="G25" s="40" t="n">
+        <v>0.0875</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B26" s="31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C26" s="31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D26" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="31" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="F26" s="31" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="G26" s="31" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="B27" s="24" t="n">
+        <f aca="false">$B$5+$B$6+$B$7</f>
+        <v>20</v>
+      </c>
+      <c r="C27" s="24" t="n">
+        <f aca="false">$B$5+$B$6+$B$7</f>
+        <v>20</v>
+      </c>
+      <c r="D27" s="24" t="n">
+        <f aca="false">$B$5+$B$6+$B$7</f>
+        <v>20</v>
+      </c>
+      <c r="E27" s="24" t="n">
+        <f aca="false">$B$5+$B$6+$B$7</f>
+        <v>20</v>
+      </c>
+      <c r="F27" s="24" t="n">
+        <f aca="false">$B$5+$B$6+$B$7</f>
+        <v>20</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <f aca="false">$B$5+$B$6+$B$7</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="25" t="s">
+        <v>225</v>
+      </c>
+      <c r="B28" s="26" t="n">
+        <f aca="false">$B$8*B24-B27</f>
+        <v>157.159271219808</v>
+      </c>
+      <c r="C28" s="26" t="n">
+        <f aca="false">$B$8*C24-C27</f>
+        <v>187.837559763159</v>
+      </c>
+      <c r="D28" s="26" t="n">
+        <f aca="false">$B$8*D24-D27</f>
+        <v>216.502631765115</v>
+      </c>
+      <c r="E28" s="26" t="n">
+        <f aca="false">$B$8*E24-E27</f>
+        <v>84.7496311689675</v>
+      </c>
+      <c r="F28" s="26" t="n">
+        <f aca="false">$B$8*F24-F27</f>
+        <v>51.6857127910397</v>
+      </c>
+      <c r="G28" s="26" t="n">
+        <f aca="false">$B$8*G24-G27</f>
+        <v>901.088945479572</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="B29" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,B26-3)*$B$13</f>
+        <v>13</v>
+      </c>
+      <c r="C29" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,C26-3)*$B$13</f>
+        <v>13</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,D26-3)*$B$13</f>
+        <v>13</v>
+      </c>
+      <c r="E29" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,E26-3)*$B$13</f>
+        <v>15.76</v>
+      </c>
+      <c r="F29" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,F26-3)*$B$13</f>
+        <v>16.27</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,G26-3)*$B$13</f>
+        <v>34.75</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B30" s="24" t="n">
+        <f aca="false">$B$14*B23*($B$18+(1-$B$18)*$B$15)</f>
+        <v>10.764</v>
+      </c>
+      <c r="C30" s="24" t="n">
+        <f aca="false">$B$14*C23*($B$18+(1-$B$18)*$B$15)</f>
+        <v>12.564</v>
+      </c>
+      <c r="D30" s="24" t="n">
+        <f aca="false">$B$14*D23*($B$18+(1-$B$18)*$B$15)</f>
+        <v>14.364</v>
+      </c>
+      <c r="E30" s="24" t="n">
+        <f aca="false">$B$14*E23*($B$18+(1-$B$18)*$B$15)</f>
+        <v>7.884</v>
+      </c>
+      <c r="F30" s="24" t="n">
+        <f aca="false">$B$14*F23*($B$18+(1-$B$18)*$B$15)</f>
+        <v>5.724</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <f aca="false">$B$14*G23*($B$18+(1-$B$18)*$B$15)</f>
+        <v>82.764</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="B31" s="24" t="n">
+        <f aca="false">B25*$B$16*$B$19*$B$17</f>
+        <v>0.2695</v>
+      </c>
+      <c r="C31" s="24" t="n">
+        <f aca="false">C25*$B$16*$B$19*$B$17</f>
+        <v>0.2695</v>
+      </c>
+      <c r="D31" s="24" t="n">
+        <f aca="false">D25*$B$16*$B$19*$B$17</f>
+        <v>0.2695</v>
+      </c>
+      <c r="E31" s="24" t="n">
+        <f aca="false">E25*$B$16*$B$19*$B$17</f>
+        <v>0.847</v>
+      </c>
+      <c r="F31" s="24" t="n">
+        <f aca="false">F25*$B$16*$B$19*$B$17</f>
+        <v>0.9065</v>
+      </c>
+      <c r="G31" s="24" t="n">
+        <f aca="false">G25*$B$16*$B$19*$B$17</f>
+        <v>3.0625</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="B32" s="24" t="n">
+        <f aca="false">B29+B30+B31</f>
+        <v>24.0335</v>
+      </c>
+      <c r="C32" s="24" t="n">
+        <f aca="false">C29+C30+C31</f>
+        <v>25.8335</v>
+      </c>
+      <c r="D32" s="24" t="n">
+        <f aca="false">D29+D30+D31</f>
+        <v>27.6335</v>
+      </c>
+      <c r="E32" s="24" t="n">
+        <f aca="false">E29+E30+E31</f>
+        <v>24.491</v>
+      </c>
+      <c r="F32" s="24" t="n">
+        <f aca="false">F29+F30+F31</f>
+        <v>22.9005</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <f aca="false">G29+G30+G31</f>
+        <v>120.5765</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="B33" s="26" t="n">
+        <f aca="false">$B$18*B24-B32</f>
+        <v>153.125771219808</v>
+      </c>
+      <c r="C33" s="26" t="n">
+        <f aca="false">$B$18*C24-C32</f>
+        <v>182.004059763159</v>
+      </c>
+      <c r="D33" s="26" t="n">
+        <f aca="false">$B$18*D24-D32</f>
+        <v>208.869131765115</v>
+      </c>
+      <c r="E33" s="26" t="n">
+        <f aca="false">$B$18*E24-E32</f>
+        <v>80.2586311689675</v>
+      </c>
+      <c r="F33" s="26" t="n">
+        <f aca="false">$B$18*F24-F32</f>
+        <v>48.7852127910397</v>
+      </c>
+      <c r="G33" s="26" t="n">
+        <f aca="false">$B$18*G24-G32</f>
+        <v>800.512445479572</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="25" t="s">
+        <v>231</v>
+      </c>
+      <c r="B34" s="27" t="n">
+        <f aca="false">B33-B28</f>
+        <v>-4.0335</v>
+      </c>
+      <c r="C34" s="27" t="n">
+        <f aca="false">C33-C28</f>
+        <v>-5.83350000000002</v>
+      </c>
+      <c r="D34" s="27" t="n">
+        <f aca="false">D33-D28</f>
+        <v>-7.6335</v>
+      </c>
+      <c r="E34" s="27" t="n">
+        <f aca="false">E33-E28</f>
+        <v>-4.491</v>
+      </c>
+      <c r="F34" s="27" t="n">
+        <f aca="false">F33-F28</f>
+        <v>-2.9005</v>
+      </c>
+      <c r="G34" s="27" t="n">
+        <f aca="false">G33-G28</f>
+        <v>-100.5765</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="B35" s="41" t="n">
+        <f aca="false">IF(B34&lt;0,-B34/B24,0)</f>
+        <v>0.0182141187293348</v>
+      </c>
+      <c r="C35" s="41" t="n">
+        <f aca="false">IF(C34&lt;0,-C34/C24,0)</f>
+        <v>0.0224540742554813</v>
+      </c>
+      <c r="D35" s="41" t="n">
+        <f aca="false">IF(D34&lt;0,-D34/D24,0)</f>
+        <v>0.0258212771436092</v>
+      </c>
+      <c r="E35" s="41" t="n">
+        <f aca="false">IF(E34&lt;0,-E34/E24,0)</f>
+        <v>0.0342989274511583</v>
+      </c>
+      <c r="F35" s="41" t="n">
+        <f aca="false">IF(F34&lt;0,-F34/F24,0)</f>
+        <v>0.0323690720180722</v>
+      </c>
+      <c r="G35" s="41" t="n">
+        <f aca="false">IF(G34&lt;0,-G34/G24,0)</f>
+        <v>0.0873544302044655</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="B36" s="42" t="n">
+        <f aca="false">(B27-B29-B31)/(B23*($B$18+(1-$B$18)*$B$15))</f>
+        <v>0.0281375418060201</v>
+      </c>
+      <c r="C36" s="42" t="n">
+        <f aca="false">(C27-C29-C31)/(C23*($B$18+(1-$B$18)*$B$15))</f>
+        <v>0.0241063753581662</v>
+      </c>
+      <c r="D36" s="42" t="n">
+        <f aca="false">(D27-D29-D31)/(D23*($B$18+(1-$B$18)*$B$15))</f>
+        <v>0.0210855263157895</v>
+      </c>
+      <c r="E36" s="42" t="n">
+        <f aca="false">(E27-E29-E31)/(E23*($B$18+(1-$B$18)*$B$15))</f>
+        <v>0.0193664383561644</v>
+      </c>
+      <c r="F36" s="42" t="n">
+        <f aca="false">(F27-F29-F31)/(F23*($B$18+(1-$B$18)*$B$15))</f>
+        <v>0.0221973270440252</v>
+      </c>
+      <c r="G36" s="42" t="n">
+        <f aca="false">(G27-G29-G31)/(G23*($B$18+(1-$B$18)*$B$15))</f>
+        <v>-0.0096849173553719</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5187,12 +5943,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>197</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>198</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5211,7 +5967,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>199</v>
+        <v>238</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>1008</v>
@@ -5226,7 +5982,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>200</v>
+        <v>239</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1000</v>
@@ -5241,7 +5997,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>201</v>
+        <v>240</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>500</v>
@@ -5256,7 +6012,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>202</v>
+        <v>241</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>5</v>
@@ -5271,7 +6027,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>203</v>
+        <v>242</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>1</v>
@@ -5286,7 +6042,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>204</v>
+        <v>243</v>
       </c>
       <c r="D10" s="29" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -5295,17 +6051,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>205</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>206</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>207</v>
+        <v>246</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>1135.87</v>
@@ -5313,7 +6069,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>135.13</v>
@@ -5321,7 +6077,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>209</v>
+        <v>248</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>1720</v>
@@ -5329,7 +6085,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>210</v>
+        <v>249</v>
       </c>
       <c r="B17" s="13" t="n">
         <v>309.6</v>
@@ -5337,7 +6093,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>211</v>
+        <v>250</v>
       </c>
       <c r="B18" s="13" t="n">
         <v>5961</v>
@@ -5345,7 +6101,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>212</v>
+        <v>251</v>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
@@ -5362,17 +6118,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>213</v>
+        <v>252</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>214</v>
+        <v>253</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>215</v>
+        <v>254</v>
       </c>
       <c r="B24" s="18" t="n">
         <f aca="false">D10*B20</f>
@@ -5381,7 +6137,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>216</v>
+        <v>255</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">B14*B20</f>
@@ -5390,7 +6146,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>217</v>
+        <v>256</v>
       </c>
       <c r="B26" s="18" t="n">
         <f aca="false">B16+B17</f>
@@ -5408,7 +6164,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="25" t="s">
-        <v>218</v>
+        <v>257</v>
       </c>
       <c r="B28" s="29" t="n">
         <f aca="false">SUM(B24:B27)</f>
@@ -5417,7 +6173,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>219</v>
+        <v>258</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -5444,7 +6200,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>220</v>
+        <v>259</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5452,24 +6208,24 @@
         <v>2</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>221</v>
+        <v>260</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>222</v>
+        <v>261</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>223</v>
+        <v>262</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>224</v>
+        <v>263</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>225</v>
+        <v>264</v>
       </c>
       <c r="B35" s="18" t="n">
         <f aca="false">D5</f>
@@ -5494,7 +6250,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="B36" s="18" t="n">
         <f aca="false">D6</f>
@@ -5519,7 +6275,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>227</v>
+        <v>266</v>
       </c>
       <c r="B37" s="18" t="n">
         <f aca="false">D7</f>
@@ -5550,7 +6306,7 @@
         <f aca="false">SUM(B35:B37)</f>
         <v>7264.2</v>
       </c>
-      <c r="C38" s="39" t="n">
+      <c r="C38" s="41" t="n">
         <f aca="false">SUM(C35:C37)</f>
         <v>1</v>
       </c>
@@ -5561,7 +6317,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>228</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Courier_Hub: condiciones confirmadas por The Hub (tarifa 8, billeteras 2.5%, retorno S/ 1)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="279">
   <si>
     <t xml:space="preserve">Resumen - utilidad por pedido (S/)</t>
   </si>
@@ -621,7 +621,7 @@
     <t xml:space="preserve">The Hub vs operacion actual - pedidos en Lima, todos contraentrega</t>
   </si>
   <si>
-    <t xml:space="preserve">Azul = dato editable. Verde = viene de otra hoja. Fuentes: proforma The Hub 21-abr-2026 y Anexo 3 de tarifas. Los precios de The Hub no incluyen IGV.</t>
+    <t xml:space="preserve">Azul = dato editable. Verde = viene de otra hoja. Fuentes: proforma The Hub 21-abr-2026, Anexo 3 de tarifas y respuestas de The Hub por WhatsApp (19-oct-2026). Sin IGV.</t>
   </si>
   <si>
     <t xml:space="preserve">Operacion actual (empaque + courier + almacen)</t>
@@ -633,40 +633,61 @@
     <t xml:space="preserve">Entrega efectiva actual en Lima</t>
   </si>
   <si>
-    <t xml:space="preserve">The Hub (Business Standard)</t>
+    <t xml:space="preserve">The Hub (Business Standard) - condiciones confirmadas</t>
   </si>
   <si>
     <t xml:space="preserve">Gestion por orden (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">Envio estandar Lima urbano, hasta 3 kg (S/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proforma y tabla de codigos postales: 7.5; hoja Tarifa Lima: 8.0. Confirmar.</t>
+    <t xml:space="preserve">Proforma.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Envio estandar Lima, tarifa ponderada hasta 3 kg (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Hub: la tarifa urbana subio a S/ 8.00 (gasolina y clima); mixtos casi siempre urbano; periferico 9.50; periferico 2: 10.50. 8.75 = ponderacion ESTIMADA con una muestra de 9 pedidos.</t>
   </si>
   <si>
     <t xml:space="preserve">Kg adicional sobre 3 kg (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">Urbano 1.5, periferico 2.0, periferico 2: 2.2. Peso facturable = largo x alto x ancho / 5000.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cobro contraentrega (% del valor del orden)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proforma: manejo de dinero y seguro.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿Cobra el contraentrega tambien en pedidos NO entregados? (1 = si, 0 = no)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supuesto: solo cobra lo que cobra. Confirmar con The Hub.</t>
+    <t xml:space="preserve">Urbano 1.5, periferico 2.0. Peso facturable = largo x alto x ancho / 5000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobro contraentrega en efectivo o tarjeta (% del valor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Hub: 4.5% en efectivo o tarjeta; no lo bajan. Solo se cobra cuando cobran.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobro contraentrega en billeteras (Yape/Plin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Hub: pueden bajarlo a 2.5%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de clientes que pagan con billetera al recibir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO ilustrativo. Reemplazar con datos reales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retorno por pedido no entregado (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hay un reintento gratis; el retorno al almacen cuesta S/ 1. Reenviar vuelve a cobrar el envio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿El cobro de The Hub incluye la comision de tarjeta y cuotas? (1 = si, 0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDIENTE de confirmar. Con 0 se suman las dos comisiones (conservador).</t>
   </si>
   <si>
     <t xml:space="preserve">Almacen (US$ por m3 al mes)</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmado por el usuario: es mensual.</t>
+    <t xml:space="preserve">Confirmado: es mensual.</t>
   </si>
   <si>
     <t xml:space="preserve">Meses que el stock permanece en The Hub</t>
@@ -678,12 +699,15 @@
     <t xml:space="preserve">Entrega efectiva con The Hub en Lima</t>
   </si>
   <si>
-    <t xml:space="preserve">Igual a la actual para comparar costos. Cambiar para probar un alza.</t>
+    <t xml:space="preserve">Igual a la actual para comparar costos. Cambiar para probar un alza (el reintento gratis podria subirla).</t>
   </si>
   <si>
     <t xml:space="preserve">Tipo de cambio</t>
   </si>
   <si>
+    <t xml:space="preserve">Cobro contraentrega promedio (% del valor)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Comparacion por pedido colocado en Lima (S/)</t>
   </si>
   <si>
@@ -693,6 +717,9 @@
     <t xml:space="preserve">Margen por pedido entregado, antes de logistica</t>
   </si>
   <si>
+    <t xml:space="preserve">  incluye comision de pago (S/, negativa)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Volumen por unidad (m3)</t>
   </si>
   <si>
@@ -711,28 +738,34 @@
     <t xml:space="preserve">HUB: cobro contraentrega esperado</t>
   </si>
   <si>
+    <t xml:space="preserve">HUB: retorno de no entregados</t>
+  </si>
+  <si>
     <t xml:space="preserve">HUB: almacen</t>
   </si>
   <si>
     <t xml:space="preserve">HUB: logistica por pedido colocado</t>
   </si>
   <si>
+    <t xml:space="preserve">HUB: margen por pedido entregado (ajustado si el cobro incluye comision)</t>
+  </si>
+  <si>
     <t xml:space="preserve">HUB: utilidad antes de publicidad</t>
   </si>
   <si>
     <t xml:space="preserve">Diferencia Hub - actual (utilidad por pedido)</t>
   </si>
   <si>
-    <t xml:space="preserve">Alza de entrega efectiva que iguala (puntos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cobro contraentrega que iguala (% del valor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lectura: si la diferencia es negativa, The Hub cuesta mas a igual tasa de entrega. La fila "alza de entrega" dice cuantos puntos debe mejorar la entrega para compensar; la ultima fila, el cobro contraentrega con el que quedarias igual.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para bidones y Cero la operacion actual es solo una referencia: se uso el mismo courier de S/ 12.5, que probablemente es bajo para esos bultos. No incluye el beneficio tributario de la factura de The Hub (IGV y gasto deducible) ni cobros de entrega fallida.</t>
+    <t xml:space="preserve">Alza de entrega que iguala (puntos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobro contraentrega promedio que iguala (% del valor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura: diferencia negativa = The Hub cuesta mas a igual tasa de entrega. "Alza de entrega" = puntos que debe mejorar para compensar. Ultima fila = cobro contraentrega promedio con el que quedas igual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incluye: beneficio tributario de la factura de The Hub (IGV y gasto deducible), seguro adicional para valores sobre S/ 300 por ruta (el Cero no queda cubierto) ni el mayor costo de bultos grandes en el actual. Para bidones y Cero el courier actual (S/ 12.5) es solo una referencia.</t>
   </si>
   <si>
     <t xml:space="preserve">Costo puesto en Lima - embarque Ningbo (llegada 22-abr-2026)</t>
@@ -1149,15 +1182,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="174" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5310,10 +5343,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
   </cols>
   <sheetData>
@@ -5392,530 +5425,661 @@
       <c r="B11" s="13" t="n">
         <v>5.5</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="B12" s="13" t="n">
-        <v>7.5</v>
+        <v>205</v>
+      </c>
+      <c r="B12" s="32" t="n">
+        <v>8.75</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B13" s="13" t="n">
         <v>1.5</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>0.045</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>0</v>
+        <v>211</v>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>0.025</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="B16" s="31" t="n">
-        <v>20</v>
+        <v>213</v>
+      </c>
+      <c r="B16" s="38" t="n">
+        <v>0.25</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="B17" s="39" t="n">
-        <v>0.5</v>
+        <v>215</v>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="B18" s="38" t="n">
-        <v>0.8</v>
+        <v>217</v>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="B19" s="34" t="n">
+        <v>219</v>
+      </c>
+      <c r="B19" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B20" s="39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B21" s="38" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="B22" s="34" t="n">
         <f aca="false">Supuestos!B5</f>
         <v>3.5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="B22" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="F22" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="G22" s="22" t="s">
-        <v>189</v>
-      </c>
-    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="B23" s="5" t="n">
+        <v>226</v>
+      </c>
+      <c r="B23" s="40" t="n">
+        <f aca="false">B14*(1-B16)+B15*B16</f>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="F26" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="G26" s="22" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="B27" s="5" t="n">
         <f aca="false">Desglose!B5</f>
         <v>299</v>
       </c>
-      <c r="C23" s="5" t="n">
+      <c r="C27" s="5" t="n">
         <f aca="false">Desglose!C5</f>
         <v>349</v>
       </c>
-      <c r="D23" s="5" t="n">
+      <c r="D27" s="5" t="n">
         <f aca="false">Desglose!D5</f>
         <v>399</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E27" s="5" t="n">
         <f aca="false">Contenedor2!B80</f>
         <v>219</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F27" s="5" t="n">
         <f aca="false">Contenedor2!C80</f>
         <v>159</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G27" s="5" t="n">
         <f aca="false">Contenedor2!E80</f>
         <v>2299</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="B24" s="6" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="B28" s="6" t="n">
         <f aca="false">Desglose!B14+Desglose!B15+Desglose!B16</f>
         <v>221.44908902476</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C28" s="6" t="n">
         <f aca="false">Desglose!C14+Desglose!C15+Desglose!C16</f>
         <v>259.796949703949</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D28" s="6" t="n">
         <f aca="false">Desglose!D14+Desglose!D15+Desglose!D16</f>
         <v>295.628289706394</v>
       </c>
-      <c r="E24" s="6" t="n">
+      <c r="E28" s="6" t="n">
         <f aca="false">Contenedor2!B81+Contenedor2!B82+Contenedor2!B83+Contenedor2!B86</f>
         <v>130.937038961209</v>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F28" s="6" t="n">
         <f aca="false">Contenedor2!C81+Contenedor2!C82+Contenedor2!C83+Contenedor2!C86</f>
         <v>89.6071409887996</v>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="G28" s="6" t="n">
         <f aca="false">Contenedor2!E81+Contenedor2!E82+Contenedor2!E83+Contenedor2!E86</f>
         <v>1151.36118184947</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="B25" s="40" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="B29" s="6" t="n">
+        <f aca="false">Desglose!B16</f>
+        <v>-9.52083</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <f aca="false">Desglose!C16</f>
+        <v>-11.02933</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <f aca="false">Desglose!D16</f>
+        <v>-12.53783</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <f aca="false">Contenedor2!B83</f>
+        <v>-7.10723</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <f aca="false">Contenedor2!C83</f>
+        <v>-5.29703</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <f aca="false">Contenedor2!E83</f>
+        <v>-69.86083</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="B30" s="41" t="n">
         <v>0.0077</v>
       </c>
-      <c r="C25" s="40" t="n">
+      <c r="C30" s="41" t="n">
         <v>0.0077</v>
       </c>
-      <c r="D25" s="40" t="n">
+      <c r="D30" s="41" t="n">
         <v>0.0077</v>
       </c>
-      <c r="E25" s="40" t="n">
+      <c r="E30" s="41" t="n">
         <v>0.0242</v>
       </c>
-      <c r="F25" s="40" t="n">
+      <c r="F30" s="41" t="n">
         <v>0.0259</v>
       </c>
-      <c r="G25" s="40" t="n">
+      <c r="G30" s="41" t="n">
         <v>0.0875</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="B26" s="31" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="B31" s="31" t="n">
         <v>1.5</v>
       </c>
-      <c r="C26" s="31" t="n">
+      <c r="C31" s="31" t="n">
         <v>1.5</v>
       </c>
-      <c r="D26" s="31" t="n">
+      <c r="D31" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="31" t="n">
+      <c r="E31" s="31" t="n">
         <v>4.84</v>
       </c>
-      <c r="F26" s="31" t="n">
+      <c r="F31" s="31" t="n">
         <v>5.18</v>
       </c>
-      <c r="G26" s="31" t="n">
+      <c r="G31" s="31" t="n">
         <v>17.5</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="B27" s="24" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B32" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="C27" s="24" t="n">
+      <c r="C32" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D32" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="E27" s="24" t="n">
+      <c r="E32" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="F27" s="24" t="n">
+      <c r="F32" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="G27" s="24" t="n">
+      <c r="G32" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
-        <v>225</v>
-      </c>
-      <c r="B28" s="26" t="n">
-        <f aca="false">$B$8*B24-B27</f>
-        <v>157.159271219808</v>
-      </c>
-      <c r="C28" s="26" t="n">
-        <f aca="false">$B$8*C24-C27</f>
-        <v>187.837559763159</v>
-      </c>
-      <c r="D28" s="26" t="n">
-        <f aca="false">$B$8*D24-D27</f>
-        <v>216.502631765115</v>
-      </c>
-      <c r="E28" s="26" t="n">
-        <f aca="false">$B$8*E24-E27</f>
-        <v>84.7496311689675</v>
-      </c>
-      <c r="F28" s="26" t="n">
-        <f aca="false">$B$8*F24-F27</f>
-        <v>51.6857127910397</v>
-      </c>
-      <c r="G28" s="26" t="n">
-        <f aca="false">$B$8*G24-G27</f>
-        <v>901.088945479572</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="B29" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,B26-3)*$B$13</f>
-        <v>13</v>
-      </c>
-      <c r="C29" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,C26-3)*$B$13</f>
-        <v>13</v>
-      </c>
-      <c r="D29" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,D26-3)*$B$13</f>
-        <v>13</v>
-      </c>
-      <c r="E29" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,E26-3)*$B$13</f>
-        <v>15.76</v>
-      </c>
-      <c r="F29" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,F26-3)*$B$13</f>
-        <v>16.27</v>
-      </c>
-      <c r="G29" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,G26-3)*$B$13</f>
-        <v>34.75</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="B30" s="24" t="n">
-        <f aca="false">$B$14*B23*($B$18+(1-$B$18)*$B$15)</f>
-        <v>10.764</v>
-      </c>
-      <c r="C30" s="24" t="n">
-        <f aca="false">$B$14*C23*($B$18+(1-$B$18)*$B$15)</f>
-        <v>12.564</v>
-      </c>
-      <c r="D30" s="24" t="n">
-        <f aca="false">$B$14*D23*($B$18+(1-$B$18)*$B$15)</f>
-        <v>14.364</v>
-      </c>
-      <c r="E30" s="24" t="n">
-        <f aca="false">$B$14*E23*($B$18+(1-$B$18)*$B$15)</f>
-        <v>7.884</v>
-      </c>
-      <c r="F30" s="24" t="n">
-        <f aca="false">$B$14*F23*($B$18+(1-$B$18)*$B$15)</f>
-        <v>5.724</v>
-      </c>
-      <c r="G30" s="24" t="n">
-        <f aca="false">$B$14*G23*($B$18+(1-$B$18)*$B$15)</f>
-        <v>82.764</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="B31" s="24" t="n">
-        <f aca="false">B25*$B$16*$B$19*$B$17</f>
-        <v>0.2695</v>
-      </c>
-      <c r="C31" s="24" t="n">
-        <f aca="false">C25*$B$16*$B$19*$B$17</f>
-        <v>0.2695</v>
-      </c>
-      <c r="D31" s="24" t="n">
-        <f aca="false">D25*$B$16*$B$19*$B$17</f>
-        <v>0.2695</v>
-      </c>
-      <c r="E31" s="24" t="n">
-        <f aca="false">E25*$B$16*$B$19*$B$17</f>
-        <v>0.847</v>
-      </c>
-      <c r="F31" s="24" t="n">
-        <f aca="false">F25*$B$16*$B$19*$B$17</f>
-        <v>0.9065</v>
-      </c>
-      <c r="G31" s="24" t="n">
-        <f aca="false">G25*$B$16*$B$19*$B$17</f>
-        <v>3.0625</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="B32" s="24" t="n">
-        <f aca="false">B29+B30+B31</f>
-        <v>24.0335</v>
-      </c>
-      <c r="C32" s="24" t="n">
-        <f aca="false">C29+C30+C31</f>
-        <v>25.8335</v>
-      </c>
-      <c r="D32" s="24" t="n">
-        <f aca="false">D29+D30+D31</f>
-        <v>27.6335</v>
-      </c>
-      <c r="E32" s="24" t="n">
-        <f aca="false">E29+E30+E31</f>
-        <v>24.491</v>
-      </c>
-      <c r="F32" s="24" t="n">
-        <f aca="false">F29+F30+F31</f>
-        <v>22.9005</v>
-      </c>
-      <c r="G32" s="24" t="n">
-        <f aca="false">G29+G30+G31</f>
-        <v>120.5765</v>
-      </c>
-    </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="25" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B33" s="26" t="n">
-        <f aca="false">$B$18*B24-B32</f>
-        <v>153.125771219808</v>
+        <f aca="false">$B$8*B28-B32</f>
+        <v>157.159271219808</v>
       </c>
       <c r="C33" s="26" t="n">
-        <f aca="false">$B$18*C24-C32</f>
-        <v>182.004059763159</v>
+        <f aca="false">$B$8*C28-C32</f>
+        <v>187.837559763159</v>
       </c>
       <c r="D33" s="26" t="n">
-        <f aca="false">$B$18*D24-D32</f>
-        <v>208.869131765115</v>
+        <f aca="false">$B$8*D28-D32</f>
+        <v>216.502631765115</v>
       </c>
       <c r="E33" s="26" t="n">
-        <f aca="false">$B$18*E24-E32</f>
-        <v>80.2586311689675</v>
+        <f aca="false">$B$8*E28-E32</f>
+        <v>84.7496311689675</v>
       </c>
       <c r="F33" s="26" t="n">
-        <f aca="false">$B$18*F24-F32</f>
-        <v>48.7852127910397</v>
+        <f aca="false">$B$8*F28-F32</f>
+        <v>51.6857127910397</v>
       </c>
       <c r="G33" s="26" t="n">
-        <f aca="false">$B$18*G24-G32</f>
-        <v>800.512445479572</v>
+        <f aca="false">$B$8*G28-G32</f>
+        <v>901.088945479572</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="s">
-        <v>231</v>
-      </c>
-      <c r="B34" s="27" t="n">
-        <f aca="false">B33-B28</f>
-        <v>-4.0335</v>
-      </c>
-      <c r="C34" s="27" t="n">
-        <f aca="false">C33-C28</f>
-        <v>-5.83350000000002</v>
-      </c>
-      <c r="D34" s="27" t="n">
-        <f aca="false">D33-D28</f>
-        <v>-7.6335</v>
-      </c>
-      <c r="E34" s="27" t="n">
-        <f aca="false">E33-E28</f>
-        <v>-4.491</v>
-      </c>
-      <c r="F34" s="27" t="n">
-        <f aca="false">F33-F28</f>
-        <v>-2.9005</v>
-      </c>
-      <c r="G34" s="27" t="n">
-        <f aca="false">G33-G28</f>
-        <v>-100.5765</v>
+      <c r="A34" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B34" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,B31-3)*$B$13</f>
+        <v>14.25</v>
+      </c>
+      <c r="C34" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,C31-3)*$B$13</f>
+        <v>14.25</v>
+      </c>
+      <c r="D34" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,D31-3)*$B$13</f>
+        <v>14.25</v>
+      </c>
+      <c r="E34" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,E31-3)*$B$13</f>
+        <v>17.01</v>
+      </c>
+      <c r="F34" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,F31-3)*$B$13</f>
+        <v>17.52</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,G31-3)*$B$13</f>
+        <v>36</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="25" t="s">
-        <v>232</v>
-      </c>
-      <c r="B35" s="41" t="n">
-        <f aca="false">IF(B34&lt;0,-B34/B24,0)</f>
-        <v>0.0182141187293348</v>
-      </c>
-      <c r="C35" s="41" t="n">
-        <f aca="false">IF(C34&lt;0,-C34/C24,0)</f>
-        <v>0.0224540742554813</v>
-      </c>
-      <c r="D35" s="41" t="n">
-        <f aca="false">IF(D34&lt;0,-D34/D24,0)</f>
-        <v>0.0258212771436092</v>
-      </c>
-      <c r="E35" s="41" t="n">
-        <f aca="false">IF(E34&lt;0,-E34/E24,0)</f>
-        <v>0.0342989274511583</v>
-      </c>
-      <c r="F35" s="41" t="n">
-        <f aca="false">IF(F34&lt;0,-F34/F24,0)</f>
-        <v>0.0323690720180722</v>
-      </c>
-      <c r="G35" s="41" t="n">
-        <f aca="false">IF(G34&lt;0,-G34/G24,0)</f>
-        <v>0.0873544302044655</v>
+      <c r="A35" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="B35" s="24" t="n">
+        <f aca="false">$B$23*B27*$B$21</f>
+        <v>9.568</v>
+      </c>
+      <c r="C35" s="24" t="n">
+        <f aca="false">$B$23*C27*$B$21</f>
+        <v>11.168</v>
+      </c>
+      <c r="D35" s="24" t="n">
+        <f aca="false">$B$23*D27*$B$21</f>
+        <v>12.768</v>
+      </c>
+      <c r="E35" s="24" t="n">
+        <f aca="false">$B$23*E27*$B$21</f>
+        <v>7.008</v>
+      </c>
+      <c r="F35" s="24" t="n">
+        <f aca="false">$B$23*F27*$B$21</f>
+        <v>5.088</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <f aca="false">$B$23*G27*$B$21</f>
+        <v>73.568</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="25" t="s">
-        <v>233</v>
-      </c>
-      <c r="B36" s="42" t="n">
-        <f aca="false">(B27-B29-B31)/(B23*($B$18+(1-$B$18)*$B$15))</f>
-        <v>0.0281375418060201</v>
-      </c>
-      <c r="C36" s="42" t="n">
-        <f aca="false">(C27-C29-C31)/(C23*($B$18+(1-$B$18)*$B$15))</f>
-        <v>0.0241063753581662</v>
-      </c>
-      <c r="D36" s="42" t="n">
-        <f aca="false">(D27-D29-D31)/(D23*($B$18+(1-$B$18)*$B$15))</f>
-        <v>0.0210855263157895</v>
-      </c>
-      <c r="E36" s="42" t="n">
-        <f aca="false">(E27-E29-E31)/(E23*($B$18+(1-$B$18)*$B$15))</f>
-        <v>0.0193664383561644</v>
-      </c>
-      <c r="F36" s="42" t="n">
-        <f aca="false">(F27-F29-F31)/(F23*($B$18+(1-$B$18)*$B$15))</f>
-        <v>0.0221973270440252</v>
-      </c>
-      <c r="G36" s="42" t="n">
-        <f aca="false">(G27-G29-G31)/(G23*($B$18+(1-$B$18)*$B$15))</f>
-        <v>-0.0096849173553719</v>
+      <c r="A36" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B36" s="24" t="n">
+        <f aca="false">(1-$B$21)*$B$17</f>
+        <v>0.2</v>
+      </c>
+      <c r="C36" s="24" t="n">
+        <f aca="false">(1-$B$21)*$B$17</f>
+        <v>0.2</v>
+      </c>
+      <c r="D36" s="24" t="n">
+        <f aca="false">(1-$B$21)*$B$17</f>
+        <v>0.2</v>
+      </c>
+      <c r="E36" s="24" t="n">
+        <f aca="false">(1-$B$21)*$B$17</f>
+        <v>0.2</v>
+      </c>
+      <c r="F36" s="24" t="n">
+        <f aca="false">(1-$B$21)*$B$17</f>
+        <v>0.2</v>
+      </c>
+      <c r="G36" s="24" t="n">
+        <f aca="false">(1-$B$21)*$B$17</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B37" s="24" t="n">
+        <f aca="false">B30*$B$19*$B$22*$B$20</f>
+        <v>0.2695</v>
+      </c>
+      <c r="C37" s="24" t="n">
+        <f aca="false">C30*$B$19*$B$22*$B$20</f>
+        <v>0.2695</v>
+      </c>
+      <c r="D37" s="24" t="n">
+        <f aca="false">D30*$B$19*$B$22*$B$20</f>
+        <v>0.2695</v>
+      </c>
+      <c r="E37" s="24" t="n">
+        <f aca="false">E30*$B$19*$B$22*$B$20</f>
+        <v>0.847</v>
+      </c>
+      <c r="F37" s="24" t="n">
+        <f aca="false">F30*$B$19*$B$22*$B$20</f>
+        <v>0.9065</v>
+      </c>
+      <c r="G37" s="24" t="n">
+        <f aca="false">G30*$B$19*$B$22*$B$20</f>
+        <v>3.0625</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>234</v>
+      <c r="A38" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="B38" s="24" t="n">
+        <f aca="false">SUM(B34:B37)</f>
+        <v>24.2875</v>
+      </c>
+      <c r="C38" s="24" t="n">
+        <f aca="false">SUM(C34:C37)</f>
+        <v>25.8875</v>
+      </c>
+      <c r="D38" s="24" t="n">
+        <f aca="false">SUM(D34:D37)</f>
+        <v>27.4875</v>
+      </c>
+      <c r="E38" s="24" t="n">
+        <f aca="false">SUM(E34:E37)</f>
+        <v>25.065</v>
+      </c>
+      <c r="F38" s="24" t="n">
+        <f aca="false">SUM(F34:F37)</f>
+        <v>23.7145</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <f aca="false">SUM(G34:G37)</f>
+        <v>112.8305</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
-        <v>235</v>
+      <c r="A39" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B39" s="24" t="n">
+        <f aca="false">B28-$B$18*B29</f>
+        <v>221.44908902476</v>
+      </c>
+      <c r="C39" s="24" t="n">
+        <f aca="false">C28-$B$18*C29</f>
+        <v>259.796949703949</v>
+      </c>
+      <c r="D39" s="24" t="n">
+        <f aca="false">D28-$B$18*D29</f>
+        <v>295.628289706394</v>
+      </c>
+      <c r="E39" s="24" t="n">
+        <f aca="false">E28-$B$18*E29</f>
+        <v>130.937038961209</v>
+      </c>
+      <c r="F39" s="24" t="n">
+        <f aca="false">F28-$B$18*F29</f>
+        <v>89.6071409887996</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <f aca="false">G28-$B$18*G29</f>
+        <v>1151.36118184947</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="25" t="s">
+        <v>241</v>
+      </c>
+      <c r="B40" s="26" t="n">
+        <f aca="false">$B$21*B39-B38</f>
+        <v>152.871771219808</v>
+      </c>
+      <c r="C40" s="26" t="n">
+        <f aca="false">$B$21*C39-C38</f>
+        <v>181.950059763159</v>
+      </c>
+      <c r="D40" s="26" t="n">
+        <f aca="false">$B$21*D39-D38</f>
+        <v>209.015131765115</v>
+      </c>
+      <c r="E40" s="26" t="n">
+        <f aca="false">$B$21*E39-E38</f>
+        <v>79.6846311689675</v>
+      </c>
+      <c r="F40" s="26" t="n">
+        <f aca="false">$B$21*F39-F38</f>
+        <v>47.9712127910397</v>
+      </c>
+      <c r="G40" s="26" t="n">
+        <f aca="false">$B$21*G39-G38</f>
+        <v>808.258445479572</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="B41" s="27" t="n">
+        <f aca="false">B40-B33</f>
+        <v>-4.28749999999999</v>
+      </c>
+      <c r="C41" s="27" t="n">
+        <f aca="false">C40-C33</f>
+        <v>-5.88749999999999</v>
+      </c>
+      <c r="D41" s="27" t="n">
+        <f aca="false">D40-D33</f>
+        <v>-7.48750000000001</v>
+      </c>
+      <c r="E41" s="27" t="n">
+        <f aca="false">E40-E33</f>
+        <v>-5.065</v>
+      </c>
+      <c r="F41" s="27" t="n">
+        <f aca="false">F40-F33</f>
+        <v>-3.7145</v>
+      </c>
+      <c r="G41" s="27" t="n">
+        <f aca="false">G40-G33</f>
+        <v>-92.8305</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="25" t="s">
+        <v>243</v>
+      </c>
+      <c r="B42" s="42" t="n">
+        <f aca="false">IF(B41&lt;0,-B41/B39,0)</f>
+        <v>0.0193611092232609</v>
+      </c>
+      <c r="C42" s="42" t="n">
+        <f aca="false">IF(C41&lt;0,-C41/C39,0)</f>
+        <v>0.0226619288898853</v>
+      </c>
+      <c r="D42" s="42" t="n">
+        <f aca="false">IF(D41&lt;0,-D41/D39,0)</f>
+        <v>0.0253274137175312</v>
+      </c>
+      <c r="E42" s="42" t="n">
+        <f aca="false">IF(E41&lt;0,-E41/E39,0)</f>
+        <v>0.0386827137697877</v>
+      </c>
+      <c r="F42" s="42" t="n">
+        <f aca="false">IF(F41&lt;0,-F41/F39,0)</f>
+        <v>0.0414531694573794</v>
+      </c>
+      <c r="G42" s="42" t="n">
+        <f aca="false">IF(G41&lt;0,-G41/G39,0)</f>
+        <v>0.0806267411681221</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="25" t="s">
+        <v>244</v>
+      </c>
+      <c r="B43" s="40" t="n">
+        <f aca="false">($B$21*B39-(B34+B36+B37)-B33)/(B27*$B$21)</f>
+        <v>0.022075668896321</v>
+      </c>
+      <c r="C43" s="40" t="n">
+        <f aca="false">($B$21*C39-(C34+C36+C37)-C33)/(C27*$B$21)</f>
+        <v>0.0189129656160458</v>
+      </c>
+      <c r="D43" s="40" t="n">
+        <f aca="false">($B$21*D39-(D34+D36+D37)-D33)/(D27*$B$21)</f>
+        <v>0.0165429197994987</v>
+      </c>
+      <c r="E43" s="40" t="n">
+        <f aca="false">($B$21*E39-(E34+E36+E37)-E33)/(E27*$B$21)</f>
+        <v>0.0110901826484018</v>
+      </c>
+      <c r="F43" s="40" t="n">
+        <f aca="false">($B$21*F39-(F34+F36+F37)-F33)/(F27*$B$21)</f>
+        <v>0.0107979559748428</v>
+      </c>
+      <c r="G43" s="40" t="n">
+        <f aca="false">($B$21*G39-(G34+G36+G37)-G33)/(G27*$B$21)</f>
+        <v>-0.0104733036102654</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -5943,12 +6107,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5967,7 +6131,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>1008</v>
@@ -5982,7 +6146,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1000</v>
@@ -5997,7 +6161,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>500</v>
@@ -6012,7 +6176,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>5</v>
@@ -6027,7 +6191,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>1</v>
@@ -6042,7 +6206,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="D10" s="29" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -6051,17 +6215,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>1135.87</v>
@@ -6069,7 +6233,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>135.13</v>
@@ -6077,7 +6241,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>1720</v>
@@ -6085,7 +6249,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="B17" s="13" t="n">
         <v>309.6</v>
@@ -6093,7 +6257,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="B18" s="13" t="n">
         <v>5961</v>
@@ -6101,7 +6265,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
@@ -6118,17 +6282,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="B24" s="18" t="n">
         <f aca="false">D10*B20</f>
@@ -6137,7 +6301,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">B14*B20</f>
@@ -6146,7 +6310,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="B26" s="18" t="n">
         <f aca="false">B16+B17</f>
@@ -6164,7 +6328,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="25" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="B28" s="29" t="n">
         <f aca="false">SUM(B24:B27)</f>
@@ -6173,7 +6337,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -6200,7 +6364,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6208,24 +6372,24 @@
         <v>2</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="B35" s="18" t="n">
         <f aca="false">D5</f>
@@ -6250,7 +6414,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="B36" s="18" t="n">
         <f aca="false">D6</f>
@@ -6275,7 +6439,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="B37" s="18" t="n">
         <f aca="false">D7</f>
@@ -6306,7 +6470,7 @@
         <f aca="false">SUM(B35:B37)</f>
         <v>7264.2</v>
       </c>
-      <c r="C38" s="41" t="n">
+      <c r="C38" s="42" t="n">
         <f aca="false">SUM(C35:C37)</f>
         <v>1</v>
       </c>
@@ -6317,7 +6481,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Courier_Hub: costo de recepcion por hora-hombre y condiciones de POS y provincia
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="286">
   <si>
     <t xml:space="preserve">Resumen - utilidad por pedido (S/)</t>
   </si>
@@ -657,7 +657,7 @@
     <t xml:space="preserve">Cobro contraentrega en efectivo o tarjeta (% del valor)</t>
   </si>
   <si>
-    <t xml:space="preserve">The Hub: 4.5% en efectivo o tarjeta; no lo bajan. Solo se cobra cuando cobran.</t>
+    <t xml:space="preserve">The Hub: 4.5% en efectivo o tarjeta; no lo bajan. Solo se cobra cuando cobran. El POS permite cuotas pero NO cuotas sin intereses.</t>
   </si>
   <si>
     <t xml:space="preserve">Cobro contraentrega en billeteras (Yape/Plin)</t>
@@ -678,7 +678,7 @@
     <t xml:space="preserve">Hay un reintento gratis; el retorno al almacen cuesta S/ 1. Reenviar vuelve a cobrar el envio.</t>
   </si>
   <si>
-    <t xml:space="preserve">¿El cobro de The Hub incluye la comision de tarjeta y cuotas? (1 = si, 0 = no)</t>
+    <t xml:space="preserve">¿El cobro de The Hub incluye la comision de tarjeta? (1 = si, 0 = no)</t>
   </si>
   <si>
     <t xml:space="preserve">PENDIENTE de confirmar. Con 0 se suman las dos comisiones (conservador).</t>
@@ -702,6 +702,18 @@
     <t xml:space="preserve">Igual a la actual para comparar costos. Cambiar para probar un alza (el reintento gratis podria subirla).</t>
   </si>
   <si>
+    <t xml:space="preserve">Recepcion de mercaderia: costo por hora-hombre (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Hub: S/ 114 por hora-hombre; depende de cuanto demoren en descargar, si viene paletizado o a granel y del tamaño.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartones descargados por hora-hombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO mio (cartones de ~20 kg a mano). Pedir el dato real; paletizado seria mucho mas rapido.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tipo de cambio</t>
   </si>
   <si>
@@ -726,6 +738,9 @@
     <t xml:space="preserve">Peso facturable (kg)</t>
   </si>
   <si>
+    <t xml:space="preserve">Unidades por carton</t>
+  </si>
+  <si>
     <t xml:space="preserve">ACTUAL: logistica por pedido colocado</t>
   </si>
   <si>
@@ -744,6 +759,9 @@
     <t xml:space="preserve">HUB: almacen</t>
   </si>
   <si>
+    <t xml:space="preserve">HUB: recepcion de mercaderia por unidad</t>
+  </si>
+  <si>
     <t xml:space="preserve">HUB: logistica por pedido colocado</t>
   </si>
   <si>
@@ -765,7 +783,10 @@
     <t xml:space="preserve">Lectura: diferencia negativa = The Hub cuesta mas a igual tasa de entrega. "Alza de entrega" = puntos que debe mejorar para compensar. Ultima fila = cobro contraentrega promedio con el que quedas igual.</t>
   </si>
   <si>
-    <t xml:space="preserve">No incluye: beneficio tributario de la factura de The Hub (IGV y gasto deducible), seguro adicional para valores sobre S/ 300 por ruta (el Cero no queda cubierto) ni el mayor costo de bultos grandes en el actual. Para bidones y Cero el courier actual (S/ 12.5) es solo una referencia.</t>
+    <t xml:space="preserve">Condiciones de The Hub: el POS NO hace cuotas sin intereses (solo cuotas con interes); en provincia NO hay contraentrega (se maneja por agencias); el seguro en ruta es de S/ 300 por ruta y el del Cero depende de la agencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incluye: beneficio tributario de la factura de The Hub (IGV y gasto deducible). Para bidones y Cero el courier actual (S/ 12.5) es solo una referencia.</t>
   </si>
   <si>
     <t xml:space="preserve">Costo puesto en Lima - embarque Ningbo (llegada 22-abr-2026)</t>
@@ -5343,7 +5364,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -5543,543 +5564,622 @@
       <c r="A22" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="B22" s="34" t="n">
+      <c r="B22" s="13" t="n">
+        <v>114</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="B24" s="34" t="n">
         <f aca="false">Supuestos!B5</f>
         <v>3.5</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="B23" s="40" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="B25" s="40" t="n">
         <f aca="false">B14*(1-B16)+B15*B16</f>
         <v>0.04</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="s">
-        <v>227</v>
-      </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B28" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C28" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="D28" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E28" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="F26" s="22" t="s">
+      <c r="F28" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="G26" s="22" t="s">
+      <c r="G28" s="22" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="B27" s="5" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="B29" s="5" t="n">
         <f aca="false">Desglose!B5</f>
         <v>299</v>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C29" s="5" t="n">
         <f aca="false">Desglose!C5</f>
         <v>349</v>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="D29" s="5" t="n">
         <f aca="false">Desglose!D5</f>
         <v>399</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E29" s="5" t="n">
         <f aca="false">Contenedor2!B80</f>
         <v>219</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F29" s="5" t="n">
         <f aca="false">Contenedor2!C80</f>
         <v>159</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G29" s="5" t="n">
         <f aca="false">Contenedor2!E80</f>
         <v>2299</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="B28" s="6" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B30" s="6" t="n">
         <f aca="false">Desglose!B14+Desglose!B15+Desglose!B16</f>
         <v>221.44908902476</v>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C30" s="6" t="n">
         <f aca="false">Desglose!C14+Desglose!C15+Desglose!C16</f>
         <v>259.796949703949</v>
       </c>
-      <c r="D28" s="6" t="n">
+      <c r="D30" s="6" t="n">
         <f aca="false">Desglose!D14+Desglose!D15+Desglose!D16</f>
         <v>295.628289706394</v>
       </c>
-      <c r="E28" s="6" t="n">
+      <c r="E30" s="6" t="n">
         <f aca="false">Contenedor2!B81+Contenedor2!B82+Contenedor2!B83+Contenedor2!B86</f>
         <v>130.937038961209</v>
       </c>
-      <c r="F28" s="6" t="n">
+      <c r="F30" s="6" t="n">
         <f aca="false">Contenedor2!C81+Contenedor2!C82+Contenedor2!C83+Contenedor2!C86</f>
         <v>89.6071409887996</v>
       </c>
-      <c r="G28" s="6" t="n">
+      <c r="G30" s="6" t="n">
         <f aca="false">Contenedor2!E81+Contenedor2!E82+Contenedor2!E83+Contenedor2!E86</f>
         <v>1151.36118184947</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="B29" s="6" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="B31" s="6" t="n">
         <f aca="false">Desglose!B16</f>
         <v>-9.52083</v>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C31" s="6" t="n">
         <f aca="false">Desglose!C16</f>
         <v>-11.02933</v>
       </c>
-      <c r="D29" s="6" t="n">
+      <c r="D31" s="6" t="n">
         <f aca="false">Desglose!D16</f>
         <v>-12.53783</v>
       </c>
-      <c r="E29" s="6" t="n">
+      <c r="E31" s="6" t="n">
         <f aca="false">Contenedor2!B83</f>
         <v>-7.10723</v>
       </c>
-      <c r="F29" s="6" t="n">
+      <c r="F31" s="6" t="n">
         <f aca="false">Contenedor2!C83</f>
         <v>-5.29703</v>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="G31" s="6" t="n">
         <f aca="false">Contenedor2!E83</f>
         <v>-69.86083</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="B30" s="41" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="C30" s="41" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="D30" s="41" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="E30" s="41" t="n">
-        <v>0.0242</v>
-      </c>
-      <c r="F30" s="41" t="n">
-        <v>0.0259</v>
-      </c>
-      <c r="G30" s="41" t="n">
-        <v>0.0875</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="B31" s="31" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C31" s="31" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D31" s="31" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="31" t="n">
-        <v>4.84</v>
-      </c>
-      <c r="F31" s="31" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="G31" s="31" t="n">
-        <v>17.5</v>
-      </c>
-    </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="B32" s="24" t="n">
+        <v>235</v>
+      </c>
+      <c r="B32" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="C32" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="D32" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="E32" s="41" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="F32" s="41" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="G32" s="41" t="n">
+        <v>0.0875</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C33" s="31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D33" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="31" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="F33" s="31" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="G33" s="31" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B34" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D34" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="E34" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F34" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G34" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B35" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="C32" s="24" t="n">
+      <c r="C35" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="D32" s="24" t="n">
+      <c r="D35" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="E32" s="24" t="n">
+      <c r="E35" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="F32" s="24" t="n">
+      <c r="F35" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="G32" s="24" t="n">
+      <c r="G35" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
-        <v>234</v>
-      </c>
-      <c r="B33" s="26" t="n">
-        <f aca="false">$B$8*B28-B32</f>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="25" t="s">
+        <v>239</v>
+      </c>
+      <c r="B36" s="26" t="n">
+        <f aca="false">$B$8*B30-B35</f>
         <v>157.159271219808</v>
       </c>
-      <c r="C33" s="26" t="n">
-        <f aca="false">$B$8*C28-C32</f>
+      <c r="C36" s="26" t="n">
+        <f aca="false">$B$8*C30-C35</f>
         <v>187.837559763159</v>
       </c>
-      <c r="D33" s="26" t="n">
-        <f aca="false">$B$8*D28-D32</f>
+      <c r="D36" s="26" t="n">
+        <f aca="false">$B$8*D30-D35</f>
         <v>216.502631765115</v>
       </c>
-      <c r="E33" s="26" t="n">
-        <f aca="false">$B$8*E28-E32</f>
+      <c r="E36" s="26" t="n">
+        <f aca="false">$B$8*E30-E35</f>
         <v>84.7496311689675</v>
       </c>
-      <c r="F33" s="26" t="n">
-        <f aca="false">$B$8*F28-F32</f>
+      <c r="F36" s="26" t="n">
+        <f aca="false">$B$8*F30-F35</f>
         <v>51.6857127910397</v>
       </c>
-      <c r="G33" s="26" t="n">
-        <f aca="false">$B$8*G28-G32</f>
+      <c r="G36" s="26" t="n">
+        <f aca="false">$B$8*G30-G35</f>
         <v>901.088945479572</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="B34" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,B31-3)*$B$13</f>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B37" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,B33-3)*$B$13</f>
         <v>14.25</v>
       </c>
-      <c r="C34" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,C31-3)*$B$13</f>
+      <c r="C37" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,C33-3)*$B$13</f>
         <v>14.25</v>
       </c>
-      <c r="D34" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,D31-3)*$B$13</f>
+      <c r="D37" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,D33-3)*$B$13</f>
         <v>14.25</v>
       </c>
-      <c r="E34" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,E31-3)*$B$13</f>
+      <c r="E37" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,E33-3)*$B$13</f>
         <v>17.01</v>
       </c>
-      <c r="F34" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,F31-3)*$B$13</f>
+      <c r="F37" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,F33-3)*$B$13</f>
         <v>17.52</v>
       </c>
-      <c r="G34" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,G31-3)*$B$13</f>
+      <c r="G37" s="24" t="n">
+        <f aca="false">$B$11+$B$12+MAX(0,G33-3)*$B$13</f>
         <v>36</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="B35" s="24" t="n">
-        <f aca="false">$B$23*B27*$B$21</f>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B38" s="24" t="n">
+        <f aca="false">$B$25*B29*$B$21</f>
         <v>9.568</v>
       </c>
-      <c r="C35" s="24" t="n">
-        <f aca="false">$B$23*C27*$B$21</f>
+      <c r="C38" s="24" t="n">
+        <f aca="false">$B$25*C29*$B$21</f>
         <v>11.168</v>
       </c>
-      <c r="D35" s="24" t="n">
-        <f aca="false">$B$23*D27*$B$21</f>
+      <c r="D38" s="24" t="n">
+        <f aca="false">$B$25*D29*$B$21</f>
         <v>12.768</v>
       </c>
-      <c r="E35" s="24" t="n">
-        <f aca="false">$B$23*E27*$B$21</f>
+      <c r="E38" s="24" t="n">
+        <f aca="false">$B$25*E29*$B$21</f>
         <v>7.008</v>
       </c>
-      <c r="F35" s="24" t="n">
-        <f aca="false">$B$23*F27*$B$21</f>
+      <c r="F38" s="24" t="n">
+        <f aca="false">$B$25*F29*$B$21</f>
         <v>5.088</v>
       </c>
-      <c r="G35" s="24" t="n">
-        <f aca="false">$B$23*G27*$B$21</f>
+      <c r="G38" s="24" t="n">
+        <f aca="false">$B$25*G29*$B$21</f>
         <v>73.568</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="B36" s="24" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B39" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="C36" s="24" t="n">
+      <c r="C39" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="D36" s="24" t="n">
+      <c r="D39" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="E36" s="24" t="n">
+      <c r="E39" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="F36" s="24" t="n">
+      <c r="F39" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="G36" s="24" t="n">
+      <c r="G39" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="B37" s="24" t="n">
-        <f aca="false">B30*$B$19*$B$22*$B$20</f>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="B40" s="24" t="n">
+        <f aca="false">B32*$B$19*$B$24*$B$20</f>
         <v>0.2695</v>
       </c>
-      <c r="C37" s="24" t="n">
-        <f aca="false">C30*$B$19*$B$22*$B$20</f>
+      <c r="C40" s="24" t="n">
+        <f aca="false">C32*$B$19*$B$24*$B$20</f>
         <v>0.2695</v>
       </c>
-      <c r="D37" s="24" t="n">
-        <f aca="false">D30*$B$19*$B$22*$B$20</f>
+      <c r="D40" s="24" t="n">
+        <f aca="false">D32*$B$19*$B$24*$B$20</f>
         <v>0.2695</v>
       </c>
-      <c r="E37" s="24" t="n">
-        <f aca="false">E30*$B$19*$B$22*$B$20</f>
+      <c r="E40" s="24" t="n">
+        <f aca="false">E32*$B$19*$B$24*$B$20</f>
         <v>0.847</v>
       </c>
-      <c r="F37" s="24" t="n">
-        <f aca="false">F30*$B$19*$B$22*$B$20</f>
+      <c r="F40" s="24" t="n">
+        <f aca="false">F32*$B$19*$B$24*$B$20</f>
         <v>0.9065</v>
       </c>
-      <c r="G37" s="24" t="n">
-        <f aca="false">G30*$B$19*$B$22*$B$20</f>
+      <c r="G40" s="24" t="n">
+        <f aca="false">G32*$B$19*$B$24*$B$20</f>
         <v>3.0625</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="B38" s="24" t="n">
-        <f aca="false">SUM(B34:B37)</f>
-        <v>24.2875</v>
-      </c>
-      <c r="C38" s="24" t="n">
-        <f aca="false">SUM(C34:C37)</f>
-        <v>25.8875</v>
-      </c>
-      <c r="D38" s="24" t="n">
-        <f aca="false">SUM(D34:D37)</f>
-        <v>27.4875</v>
-      </c>
-      <c r="E38" s="24" t="n">
-        <f aca="false">SUM(E34:E37)</f>
-        <v>25.065</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <f aca="false">SUM(F34:F37)</f>
-        <v>23.7145</v>
-      </c>
-      <c r="G38" s="24" t="n">
-        <f aca="false">SUM(G34:G37)</f>
-        <v>112.8305</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="B39" s="24" t="n">
-        <f aca="false">B28-$B$18*B29</f>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="B41" s="24" t="n">
+        <f aca="false">$B$22/($B$23*B34)</f>
+        <v>0.316666666666667</v>
+      </c>
+      <c r="C41" s="24" t="n">
+        <f aca="false">$B$22/($B$23*C34)</f>
+        <v>0.316666666666667</v>
+      </c>
+      <c r="D41" s="24" t="n">
+        <f aca="false">$B$22/($B$23*D34)</f>
+        <v>0.316666666666667</v>
+      </c>
+      <c r="E41" s="24" t="n">
+        <f aca="false">$B$22/($B$23*E34)</f>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="F41" s="24" t="n">
+        <f aca="false">$B$22/($B$23*F34)</f>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="G41" s="24" t="n">
+        <f aca="false">$B$22/($B$23*G34)</f>
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B42" s="24" t="n">
+        <f aca="false">SUM(B37:B41)</f>
+        <v>24.6041666666667</v>
+      </c>
+      <c r="C42" s="24" t="n">
+        <f aca="false">SUM(C37:C41)</f>
+        <v>26.2041666666667</v>
+      </c>
+      <c r="D42" s="24" t="n">
+        <f aca="false">SUM(D37:D41)</f>
+        <v>27.8041666666667</v>
+      </c>
+      <c r="E42" s="24" t="n">
+        <f aca="false">SUM(E37:E41)</f>
+        <v>25.6983333333333</v>
+      </c>
+      <c r="F42" s="24" t="n">
+        <f aca="false">SUM(F37:F41)</f>
+        <v>24.3478333333333</v>
+      </c>
+      <c r="G42" s="24" t="n">
+        <f aca="false">SUM(G37:G41)</f>
+        <v>116.6305</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="B43" s="24" t="n">
+        <f aca="false">B30-$B$18*B31</f>
         <v>221.44908902476</v>
       </c>
-      <c r="C39" s="24" t="n">
-        <f aca="false">C28-$B$18*C29</f>
+      <c r="C43" s="24" t="n">
+        <f aca="false">C30-$B$18*C31</f>
         <v>259.796949703949</v>
       </c>
-      <c r="D39" s="24" t="n">
-        <f aca="false">D28-$B$18*D29</f>
+      <c r="D43" s="24" t="n">
+        <f aca="false">D30-$B$18*D31</f>
         <v>295.628289706394</v>
       </c>
-      <c r="E39" s="24" t="n">
-        <f aca="false">E28-$B$18*E29</f>
+      <c r="E43" s="24" t="n">
+        <f aca="false">E30-$B$18*E31</f>
         <v>130.937038961209</v>
       </c>
-      <c r="F39" s="24" t="n">
-        <f aca="false">F28-$B$18*F29</f>
+      <c r="F43" s="24" t="n">
+        <f aca="false">F30-$B$18*F31</f>
         <v>89.6071409887996</v>
       </c>
-      <c r="G39" s="24" t="n">
-        <f aca="false">G28-$B$18*G29</f>
+      <c r="G43" s="24" t="n">
+        <f aca="false">G30-$B$18*G31</f>
         <v>1151.36118184947</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="25" t="s">
-        <v>241</v>
-      </c>
-      <c r="B40" s="26" t="n">
-        <f aca="false">$B$21*B39-B38</f>
-        <v>152.871771219808</v>
-      </c>
-      <c r="C40" s="26" t="n">
-        <f aca="false">$B$21*C39-C38</f>
-        <v>181.950059763159</v>
-      </c>
-      <c r="D40" s="26" t="n">
-        <f aca="false">$B$21*D39-D38</f>
-        <v>209.015131765115</v>
-      </c>
-      <c r="E40" s="26" t="n">
-        <f aca="false">$B$21*E39-E38</f>
-        <v>79.6846311689675</v>
-      </c>
-      <c r="F40" s="26" t="n">
-        <f aca="false">$B$21*F39-F38</f>
-        <v>47.9712127910397</v>
-      </c>
-      <c r="G40" s="26" t="n">
-        <f aca="false">$B$21*G39-G38</f>
-        <v>808.258445479572</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="25" t="s">
-        <v>242</v>
-      </c>
-      <c r="B41" s="27" t="n">
-        <f aca="false">B40-B33</f>
-        <v>-4.28749999999999</v>
-      </c>
-      <c r="C41" s="27" t="n">
-        <f aca="false">C40-C33</f>
-        <v>-5.88749999999999</v>
-      </c>
-      <c r="D41" s="27" t="n">
-        <f aca="false">D40-D33</f>
-        <v>-7.48750000000001</v>
-      </c>
-      <c r="E41" s="27" t="n">
-        <f aca="false">E40-E33</f>
-        <v>-5.065</v>
-      </c>
-      <c r="F41" s="27" t="n">
-        <f aca="false">F40-F33</f>
-        <v>-3.7145</v>
-      </c>
-      <c r="G41" s="27" t="n">
-        <f aca="false">G40-G33</f>
-        <v>-92.8305</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="25" t="s">
-        <v>243</v>
-      </c>
-      <c r="B42" s="42" t="n">
-        <f aca="false">IF(B41&lt;0,-B41/B39,0)</f>
-        <v>0.0193611092232609</v>
-      </c>
-      <c r="C42" s="42" t="n">
-        <f aca="false">IF(C41&lt;0,-C41/C39,0)</f>
-        <v>0.0226619288898853</v>
-      </c>
-      <c r="D42" s="42" t="n">
-        <f aca="false">IF(D41&lt;0,-D41/D39,0)</f>
-        <v>0.0253274137175312</v>
-      </c>
-      <c r="E42" s="42" t="n">
-        <f aca="false">IF(E41&lt;0,-E41/E39,0)</f>
-        <v>0.0386827137697877</v>
-      </c>
-      <c r="F42" s="42" t="n">
-        <f aca="false">IF(F41&lt;0,-F41/F39,0)</f>
-        <v>0.0414531694573794</v>
-      </c>
-      <c r="G42" s="42" t="n">
-        <f aca="false">IF(G41&lt;0,-G41/G39,0)</f>
-        <v>0.0806267411681221</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="25" t="s">
-        <v>244</v>
-      </c>
-      <c r="B43" s="40" t="n">
-        <f aca="false">($B$21*B39-(B34+B36+B37)-B33)/(B27*$B$21)</f>
-        <v>0.022075668896321</v>
-      </c>
-      <c r="C43" s="40" t="n">
-        <f aca="false">($B$21*C39-(C34+C36+C37)-C33)/(C27*$B$21)</f>
-        <v>0.0189129656160458</v>
-      </c>
-      <c r="D43" s="40" t="n">
-        <f aca="false">($B$21*D39-(D34+D36+D37)-D33)/(D27*$B$21)</f>
-        <v>0.0165429197994987</v>
-      </c>
-      <c r="E43" s="40" t="n">
-        <f aca="false">($B$21*E39-(E34+E36+E37)-E33)/(E27*$B$21)</f>
-        <v>0.0110901826484018</v>
-      </c>
-      <c r="F43" s="40" t="n">
-        <f aca="false">($B$21*F39-(F34+F36+F37)-F33)/(F27*$B$21)</f>
-        <v>0.0107979559748428</v>
-      </c>
-      <c r="G43" s="40" t="n">
-        <f aca="false">($B$21*G39-(G34+G36+G37)-G33)/(G27*$B$21)</f>
-        <v>-0.0104733036102654</v>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="25" t="s">
+        <v>247</v>
+      </c>
+      <c r="B44" s="26" t="n">
+        <f aca="false">$B$21*B43-B42</f>
+        <v>152.555104553141</v>
+      </c>
+      <c r="C44" s="26" t="n">
+        <f aca="false">$B$21*C43-C42</f>
+        <v>181.633393096492</v>
+      </c>
+      <c r="D44" s="26" t="n">
+        <f aca="false">$B$21*D43-D42</f>
+        <v>208.698465098448</v>
+      </c>
+      <c r="E44" s="26" t="n">
+        <f aca="false">$B$21*E43-E42</f>
+        <v>79.0512978356341</v>
+      </c>
+      <c r="F44" s="26" t="n">
+        <f aca="false">$B$21*F43-F42</f>
+        <v>47.3378794577064</v>
+      </c>
+      <c r="G44" s="26" t="n">
+        <f aca="false">$B$21*G43-G42</f>
+        <v>804.458445479572</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
-        <v>245</v>
+      <c r="A45" s="25" t="s">
+        <v>248</v>
+      </c>
+      <c r="B45" s="27" t="n">
+        <f aca="false">B44-B36</f>
+        <v>-4.60416666666666</v>
+      </c>
+      <c r="C45" s="27" t="n">
+        <f aca="false">C44-C36</f>
+        <v>-6.20416666666665</v>
+      </c>
+      <c r="D45" s="27" t="n">
+        <f aca="false">D44-D36</f>
+        <v>-7.80416666666667</v>
+      </c>
+      <c r="E45" s="27" t="n">
+        <f aca="false">E44-E36</f>
+        <v>-5.69833333333332</v>
+      </c>
+      <c r="F45" s="27" t="n">
+        <f aca="false">F44-F36</f>
+        <v>-4.34783333333333</v>
+      </c>
+      <c r="G45" s="27" t="n">
+        <f aca="false">G44-G36</f>
+        <v>-96.6305</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="s">
-        <v>246</v>
+      <c r="A46" s="25" t="s">
+        <v>249</v>
+      </c>
+      <c r="B46" s="42" t="n">
+        <f aca="false">IF(B45&lt;0,-B45/B43,0)</f>
+        <v>0.0207910842484968</v>
+      </c>
+      <c r="C46" s="42" t="n">
+        <f aca="false">IF(C45&lt;0,-C45/C43,0)</f>
+        <v>0.0238808295237361</v>
+      </c>
+      <c r="D46" s="42" t="n">
+        <f aca="false">IF(D45&lt;0,-D45/D43,0)</f>
+        <v>0.026398578682769</v>
+      </c>
+      <c r="E46" s="42" t="n">
+        <f aca="false">IF(E45&lt;0,-E45/E43,0)</f>
+        <v>0.04351964408651</v>
+      </c>
+      <c r="F46" s="42" t="n">
+        <f aca="false">IF(F45&lt;0,-F45/F43,0)</f>
+        <v>0.0485210585379215</v>
+      </c>
+      <c r="G46" s="42" t="n">
+        <f aca="false">IF(G45&lt;0,-G45/G43,0)</f>
+        <v>0.0839271824717762</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B47" s="40" t="n">
+        <f aca="false">($B$21*B43-(B37+B39+B40+B41)-B36)/(B29*$B$21)</f>
+        <v>0.0207518115942029</v>
+      </c>
+      <c r="C47" s="40" t="n">
+        <f aca="false">($B$21*C43-(C37+C39+C40+C41)-C36)/(C29*$B$21)</f>
+        <v>0.0177787726838586</v>
+      </c>
+      <c r="D47" s="40" t="n">
+        <f aca="false">($B$21*D43-(D37+D39+D40+D41)-D36)/(D29*$B$21)</f>
+        <v>0.0155508563074352</v>
+      </c>
+      <c r="E47" s="40" t="n">
+        <f aca="false">($B$21*E43-(E37+E39+E40+E41)-E36)/(E29*$B$21)</f>
+        <v>0.00747526636225269</v>
+      </c>
+      <c r="F47" s="40" t="n">
+        <f aca="false">($B$21*F43-(F37+F39+F40+F41)-F36)/(F29*$B$21)</f>
+        <v>0.00581892033542977</v>
+      </c>
+      <c r="G47" s="40" t="n">
+        <f aca="false">($B$21*G43-(G37+G39+G40+G41)-G36)/(G29*$B$21)</f>
+        <v>-0.0125394193127447</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -6107,12 +6207,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6131,7 +6231,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>1008</v>
@@ -6146,7 +6246,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1000</v>
@@ -6161,7 +6261,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>500</v>
@@ -6176,7 +6276,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>5</v>
@@ -6191,7 +6291,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>1</v>
@@ -6206,7 +6306,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="D10" s="29" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -6215,17 +6315,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>1135.87</v>
@@ -6233,7 +6333,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>135.13</v>
@@ -6241,7 +6341,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>1720</v>
@@ -6249,7 +6349,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="B17" s="13" t="n">
         <v>309.6</v>
@@ -6257,7 +6357,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="B18" s="13" t="n">
         <v>5961</v>
@@ -6265,7 +6365,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
@@ -6282,17 +6382,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B24" s="18" t="n">
         <f aca="false">D10*B20</f>
@@ -6301,7 +6401,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">B14*B20</f>
@@ -6310,7 +6410,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="B26" s="18" t="n">
         <f aca="false">B16+B17</f>
@@ -6328,7 +6428,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="25" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="B28" s="29" t="n">
         <f aca="false">SUM(B24:B27)</f>
@@ -6337,7 +6437,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -6364,7 +6464,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6372,24 +6472,24 @@
         <v>2</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="B35" s="18" t="n">
         <f aca="false">D5</f>
@@ -6414,7 +6514,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B36" s="18" t="n">
         <f aca="false">D6</f>
@@ -6439,7 +6539,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="B37" s="18" t="n">
         <f aca="false">D7</f>
@@ -6481,7 +6581,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Courier_Hub: minimo de 150 pedidos, cobro que incluye tarjeta; hoja Stock_Hub con plan de tandas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Desglose" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Contenedor2" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Courier_Hub" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Costo_Lima" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Stock_Hub" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Costo_Lima" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="328">
   <si>
     <t xml:space="preserve">Resumen - utilidad por pedido (S/)</t>
   </si>
@@ -645,7 +646,7 @@
     <t xml:space="preserve">Envio estandar Lima, tarifa ponderada hasta 3 kg (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">The Hub: la tarifa urbana subio a S/ 8.00 (gasolina y clima); mixtos casi siempre urbano; periferico 9.50; periferico 2: 10.50. 8.75 = ponderacion ESTIMADA con una muestra de 9 pedidos.</t>
+    <t xml:space="preserve">The Hub: la tarifa urbana subio a S/ 8.00; mixtos casi siempre urbano; periferico 9.50; periferico 2: 10.50. 8.75 = ponderacion ESTIMADA con una muestra de 9 pedidos.</t>
   </si>
   <si>
     <t xml:space="preserve">Kg adicional sobre 3 kg (S/)</t>
@@ -681,7 +682,7 @@
     <t xml:space="preserve">¿El cobro de The Hub incluye la comision de tarjeta? (1 = si, 0 = no)</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE de confirmar. Con 0 se suman las dos comisiones (conservador).</t>
+    <t xml:space="preserve">CONFIRMADO por The Hub: el 4.5% incluye la tarjeta.</t>
   </si>
   <si>
     <t xml:space="preserve">Almacen (US$ por m3 al mes)</t>
@@ -705,13 +706,25 @@
     <t xml:space="preserve">Recepcion de mercaderia: costo por hora-hombre (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">The Hub: S/ 114 por hora-hombre; depende de cuanto demoren en descargar, si viene paletizado o a granel y del tamaño.</t>
+    <t xml:space="preserve">The Hub: S/ 114 por hora-hombre.</t>
   </si>
   <si>
     <t xml:space="preserve">Cartones descargados por hora-hombre</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPUESTO mio (cartones de ~20 kg a mano). Pedir el dato real; paletizado seria mucho mas rapido.</t>
+    <t xml:space="preserve">ESTIMACION mia (cartones de ~20 kg a mano, incluye conteo y acomodo). Paletizado seria mucho mas rapido. Pedir dato real.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos al mes que pasarian por The Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO. Ajustar a tu volumen en Lima.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimo de pedidos al mes (se paga el empaque faltante)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Hub: si no se llega a 150, se paga el empaque que falta.</t>
   </si>
   <si>
     <t xml:space="preserve">Tipo de cambio</t>
@@ -720,6 +733,9 @@
     <t xml:space="preserve">Cobro contraentrega promedio (% del valor)</t>
   </si>
   <si>
+    <t xml:space="preserve">Gestion efectiva por pedido (S/), con el minimo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Comparacion por pedido colocado en Lima (S/)</t>
   </si>
   <si>
@@ -747,7 +763,7 @@
     <t xml:space="preserve">ACTUAL: utilidad antes de publicidad</t>
   </si>
   <si>
-    <t xml:space="preserve">HUB: gestion + envio</t>
+    <t xml:space="preserve">HUB: gestion (con minimo) + envio</t>
   </si>
   <si>
     <t xml:space="preserve">HUB: cobro contraentrega esperado</t>
@@ -762,10 +778,13 @@
     <t xml:space="preserve">HUB: recepcion de mercaderia por unidad</t>
   </si>
   <si>
+    <t xml:space="preserve">HUB: transporte de tu almacen a The Hub por pedido</t>
+  </si>
+  <si>
     <t xml:space="preserve">HUB: logistica por pedido colocado</t>
   </si>
   <si>
-    <t xml:space="preserve">HUB: margen por pedido entregado (ajustado si el cobro incluye comision)</t>
+    <t xml:space="preserve">HUB: margen por pedido entregado (sin la comision de tarjeta, que incluye el cobro)</t>
   </si>
   <si>
     <t xml:space="preserve">HUB: utilidad antes de publicidad</t>
@@ -780,13 +799,121 @@
     <t xml:space="preserve">Cobro contraentrega promedio que iguala (% del valor)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lectura: diferencia negativa = The Hub cuesta mas a igual tasa de entrega. "Alza de entrega" = puntos que debe mejorar para compensar. Ultima fila = cobro contraentrega promedio con el que quedas igual.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Condiciones de The Hub: el POS NO hace cuotas sin intereses (solo cuotas con interes); en provincia NO hay contraentrega (se maneja por agencias); el seguro en ruta es de S/ 300 por ruta y el del Cero depende de la agencia.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No incluye: beneficio tributario de la factura de The Hub (IGV y gasto deducible). Para bidones y Cero el courier actual (S/ 12.5) es solo una referencia.</t>
+    <t xml:space="preserve">Sensibilidad: diferencia Hub - actual por pedido de Nativo 3 años segun pedidos al mes (por el minimo de 150)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos al mes en The Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia por pedido (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura: diferencia negativa = The Hub cuesta mas a igual tasa de entrega. "Alza de entrega" = puntos que debe mejorar para compensar. Ultima fila de la tabla = cobro contraentrega promedio con el que quedas igual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condiciones de The Hub: el POS NO hace cuotas sin intereses; en provincia NO hay contraentrega (se maneja por agencias); el seguro en ruta es de S/ 300 por ruta y el del Cero depende de la agencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incluye: beneficio tributario de la factura de The Hub (IGV y gasto deducible) (el transporte desde tu almacen a The Hub viene de la hoja Stock_Hub). Para bidones y Cero el courier actual (S/ 12.5) es solo una referencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan de stock en The Hub: tandas desde tu almacen propio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea: dejar en The Hub solo lo que se vende en unas dos semanas y reponer por tandas. Azul = supuesto editable (la mezcla de pedidos es ilustrativa).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos por dia en Lima que pasan por The Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de Courier_Hub (pedidos al mes / 30). 150 pedidos al mes = minimo de The Hub.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dias de venta que cubre cada tanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tandas mensuales: el almacen es barato (US$ 20 por m3) y cada viaje tiene costo fijo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dias de stock de seguridad en The Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horas minimas facturables por recepcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO: se asume 1 hora como minimo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transporte de tu almacen a The Hub, por tanda (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO. El anexo de tarifas trae S/ 200 por pallet para envios a CD / reposicion; confirmar si es esto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo por hora-hombre (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de pedidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidades por tanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartones por tanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m3 por unidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m3 ocupados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo mensual de tener stock en The Hub (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horas de recepcion por tanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo de recepcion por tanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tandas por mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepcion al mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transporte al mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almacen al mes (m3 ocupados al maximo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total almacen + recepcion + transporte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos al mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestion facturable al mes (con minimo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo por pedido en The Hub (sin envio ni cobro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo por pedido actual (empaque + almacen Tecretail)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia por pedido (Hub - actual)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimacion por tanda: sirve para ver el orden de magnitud. Las horas de descarga son estimadas (30 cartones por hora-hombre); si mandas en pallets, bajan mucho. El costo por pedido actual usa el empaque y el almacen de Tecretail de la hoja Supuestos.</t>
   </si>
   <si>
     <t xml:space="preserve">Costo puesto en Lima - embarque Ningbo (llegada 22-abr-2026)</t>
@@ -1042,7 +1169,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1212,6 +1339,38 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5364,10 +5523,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
   </cols>
   <sheetData>
@@ -5520,8 +5679,8 @@
       <c r="A18" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="B18" s="15" t="n">
-        <v>0</v>
+      <c r="B18" s="23" t="n">
+        <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>218</v>
@@ -5586,600 +5745,723 @@
       <c r="A24" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="B24" s="34" t="n">
+      <c r="B24" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>150</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B26" s="34" t="n">
         <f aca="false">Supuestos!B5</f>
         <v>3.5</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="B25" s="40" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="B27" s="40" t="n">
         <f aca="false">B14*(1-B16)+B15*B16</f>
         <v>0.04</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-    </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B28" s="29" t="n">
+        <f aca="false">B11*MAX(B25,B24)/B24</f>
+        <v>8.25</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B31" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C31" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="D31" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E31" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F31" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="G28" s="22" t="s">
+      <c r="G31" s="22" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="B29" s="5" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B32" s="5" t="n">
         <f aca="false">Desglose!B5</f>
         <v>299</v>
       </c>
-      <c r="C29" s="5" t="n">
+      <c r="C32" s="5" t="n">
         <f aca="false">Desglose!C5</f>
         <v>349</v>
       </c>
-      <c r="D29" s="5" t="n">
+      <c r="D32" s="5" t="n">
         <f aca="false">Desglose!D5</f>
         <v>399</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E32" s="5" t="n">
         <f aca="false">Contenedor2!B80</f>
         <v>219</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F32" s="5" t="n">
         <f aca="false">Contenedor2!C80</f>
         <v>159</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="G32" s="5" t="n">
         <f aca="false">Contenedor2!E80</f>
         <v>2299</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="B30" s="6" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B33" s="6" t="n">
         <f aca="false">Desglose!B14+Desglose!B15+Desglose!B16</f>
         <v>221.44908902476</v>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C33" s="6" t="n">
         <f aca="false">Desglose!C14+Desglose!C15+Desglose!C16</f>
         <v>259.796949703949</v>
       </c>
-      <c r="D30" s="6" t="n">
+      <c r="D33" s="6" t="n">
         <f aca="false">Desglose!D14+Desglose!D15+Desglose!D16</f>
         <v>295.628289706394</v>
       </c>
-      <c r="E30" s="6" t="n">
+      <c r="E33" s="6" t="n">
         <f aca="false">Contenedor2!B81+Contenedor2!B82+Contenedor2!B83+Contenedor2!B86</f>
         <v>130.937038961209</v>
       </c>
-      <c r="F30" s="6" t="n">
+      <c r="F33" s="6" t="n">
         <f aca="false">Contenedor2!C81+Contenedor2!C82+Contenedor2!C83+Contenedor2!C86</f>
         <v>89.6071409887996</v>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="G33" s="6" t="n">
         <f aca="false">Contenedor2!E81+Contenedor2!E82+Contenedor2!E83+Contenedor2!E86</f>
         <v>1151.36118184947</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="B31" s="6" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="B34" s="6" t="n">
         <f aca="false">Desglose!B16</f>
         <v>-9.52083</v>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C34" s="6" t="n">
         <f aca="false">Desglose!C16</f>
         <v>-11.02933</v>
       </c>
-      <c r="D31" s="6" t="n">
+      <c r="D34" s="6" t="n">
         <f aca="false">Desglose!D16</f>
         <v>-12.53783</v>
       </c>
-      <c r="E31" s="6" t="n">
+      <c r="E34" s="6" t="n">
         <f aca="false">Contenedor2!B83</f>
         <v>-7.10723</v>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="F34" s="6" t="n">
         <f aca="false">Contenedor2!C83</f>
         <v>-5.29703</v>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="G34" s="6" t="n">
         <f aca="false">Contenedor2!E83</f>
         <v>-69.86083</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="B32" s="41" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="C32" s="41" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="D32" s="41" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="E32" s="41" t="n">
-        <v>0.0242</v>
-      </c>
-      <c r="F32" s="41" t="n">
-        <v>0.0259</v>
-      </c>
-      <c r="G32" s="41" t="n">
-        <v>0.0875</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="B33" s="31" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C33" s="31" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D33" s="31" t="n">
-        <v>2</v>
-      </c>
-      <c r="E33" s="31" t="n">
-        <v>4.84</v>
-      </c>
-      <c r="F33" s="31" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="G33" s="31" t="n">
-        <v>17.5</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="B34" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="C34" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="D34" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="E34" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="F34" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G34" s="23" t="n">
-        <v>1</v>
-      </c>
-    </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="B35" s="24" t="n">
+        <v>240</v>
+      </c>
+      <c r="B35" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="C35" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="D35" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="E35" s="41" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="F35" s="41" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="G35" s="41" t="n">
+        <v>0.0875</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B36" s="31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C36" s="31" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D36" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="31" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="F36" s="31" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="G36" s="31" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B37" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D37" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="E37" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G37" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="B38" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="C35" s="24" t="n">
+      <c r="C38" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="D35" s="24" t="n">
+      <c r="D38" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="E35" s="24" t="n">
+      <c r="E38" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="F35" s="24" t="n">
+      <c r="F38" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
-      <c r="G35" s="24" t="n">
+      <c r="G38" s="24" t="n">
         <f aca="false">$B$5+$B$6+$B$7</f>
         <v>20</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="25" t="s">
-        <v>239</v>
-      </c>
-      <c r="B36" s="26" t="n">
-        <f aca="false">$B$8*B30-B35</f>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="25" t="s">
+        <v>244</v>
+      </c>
+      <c r="B39" s="26" t="n">
+        <f aca="false">$B$8*B33-B38</f>
         <v>157.159271219808</v>
       </c>
-      <c r="C36" s="26" t="n">
-        <f aca="false">$B$8*C30-C35</f>
+      <c r="C39" s="26" t="n">
+        <f aca="false">$B$8*C33-C38</f>
         <v>187.837559763159</v>
       </c>
-      <c r="D36" s="26" t="n">
-        <f aca="false">$B$8*D30-D35</f>
+      <c r="D39" s="26" t="n">
+        <f aca="false">$B$8*D33-D38</f>
         <v>216.502631765115</v>
       </c>
-      <c r="E36" s="26" t="n">
-        <f aca="false">$B$8*E30-E35</f>
+      <c r="E39" s="26" t="n">
+        <f aca="false">$B$8*E33-E38</f>
         <v>84.7496311689675</v>
       </c>
-      <c r="F36" s="26" t="n">
-        <f aca="false">$B$8*F30-F35</f>
+      <c r="F39" s="26" t="n">
+        <f aca="false">$B$8*F33-F38</f>
         <v>51.6857127910397</v>
       </c>
-      <c r="G36" s="26" t="n">
-        <f aca="false">$B$8*G30-G35</f>
+      <c r="G39" s="26" t="n">
+        <f aca="false">$B$8*G33-G38</f>
         <v>901.088945479572</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="B37" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,B33-3)*$B$13</f>
-        <v>14.25</v>
-      </c>
-      <c r="C37" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,C33-3)*$B$13</f>
-        <v>14.25</v>
-      </c>
-      <c r="D37" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,D33-3)*$B$13</f>
-        <v>14.25</v>
-      </c>
-      <c r="E37" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,E33-3)*$B$13</f>
-        <v>17.01</v>
-      </c>
-      <c r="F37" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,F33-3)*$B$13</f>
-        <v>17.52</v>
-      </c>
-      <c r="G37" s="24" t="n">
-        <f aca="false">$B$11+$B$12+MAX(0,G33-3)*$B$13</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="B38" s="24" t="n">
-        <f aca="false">$B$25*B29*$B$21</f>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B40" s="24" t="n">
+        <f aca="false">$B$28+$B$12+MAX(0,B36-3)*$B$13</f>
+        <v>17</v>
+      </c>
+      <c r="C40" s="24" t="n">
+        <f aca="false">$B$28+$B$12+MAX(0,C36-3)*$B$13</f>
+        <v>17</v>
+      </c>
+      <c r="D40" s="24" t="n">
+        <f aca="false">$B$28+$B$12+MAX(0,D36-3)*$B$13</f>
+        <v>17</v>
+      </c>
+      <c r="E40" s="24" t="n">
+        <f aca="false">$B$28+$B$12+MAX(0,E36-3)*$B$13</f>
+        <v>19.76</v>
+      </c>
+      <c r="F40" s="24" t="n">
+        <f aca="false">$B$28+$B$12+MAX(0,F36-3)*$B$13</f>
+        <v>20.27</v>
+      </c>
+      <c r="G40" s="24" t="n">
+        <f aca="false">$B$28+$B$12+MAX(0,G36-3)*$B$13</f>
+        <v>38.75</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="B41" s="24" t="n">
+        <f aca="false">$B$27*B32*$B$21</f>
         <v>9.568</v>
       </c>
-      <c r="C38" s="24" t="n">
-        <f aca="false">$B$25*C29*$B$21</f>
+      <c r="C41" s="24" t="n">
+        <f aca="false">$B$27*C32*$B$21</f>
         <v>11.168</v>
       </c>
-      <c r="D38" s="24" t="n">
-        <f aca="false">$B$25*D29*$B$21</f>
+      <c r="D41" s="24" t="n">
+        <f aca="false">$B$27*D32*$B$21</f>
         <v>12.768</v>
       </c>
-      <c r="E38" s="24" t="n">
-        <f aca="false">$B$25*E29*$B$21</f>
+      <c r="E41" s="24" t="n">
+        <f aca="false">$B$27*E32*$B$21</f>
         <v>7.008</v>
       </c>
-      <c r="F38" s="24" t="n">
-        <f aca="false">$B$25*F29*$B$21</f>
+      <c r="F41" s="24" t="n">
+        <f aca="false">$B$27*F32*$B$21</f>
         <v>5.088</v>
       </c>
-      <c r="G38" s="24" t="n">
-        <f aca="false">$B$25*G29*$B$21</f>
+      <c r="G41" s="24" t="n">
+        <f aca="false">$B$27*G32*$B$21</f>
         <v>73.568</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10" t="s">
-        <v>242</v>
-      </c>
-      <c r="B39" s="24" t="n">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="B42" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="C39" s="24" t="n">
+      <c r="C42" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="D39" s="24" t="n">
+      <c r="D42" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="E39" s="24" t="n">
+      <c r="E42" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="F39" s="24" t="n">
+      <c r="F42" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
-      <c r="G39" s="24" t="n">
+      <c r="G42" s="24" t="n">
         <f aca="false">(1-$B$21)*$B$17</f>
         <v>0.2</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="B40" s="24" t="n">
-        <f aca="false">B32*$B$19*$B$24*$B$20</f>
-        <v>0.2695</v>
-      </c>
-      <c r="C40" s="24" t="n">
-        <f aca="false">C32*$B$19*$B$24*$B$20</f>
-        <v>0.2695</v>
-      </c>
-      <c r="D40" s="24" t="n">
-        <f aca="false">D32*$B$19*$B$24*$B$20</f>
-        <v>0.2695</v>
-      </c>
-      <c r="E40" s="24" t="n">
-        <f aca="false">E32*$B$19*$B$24*$B$20</f>
-        <v>0.847</v>
-      </c>
-      <c r="F40" s="24" t="n">
-        <f aca="false">F32*$B$19*$B$24*$B$20</f>
-        <v>0.9065</v>
-      </c>
-      <c r="G40" s="24" t="n">
-        <f aca="false">G32*$B$19*$B$24*$B$20</f>
-        <v>3.0625</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="10" t="s">
-        <v>244</v>
-      </c>
-      <c r="B41" s="24" t="n">
-        <f aca="false">$B$22/($B$23*B34)</f>
-        <v>0.316666666666667</v>
-      </c>
-      <c r="C41" s="24" t="n">
-        <f aca="false">$B$22/($B$23*C34)</f>
-        <v>0.316666666666667</v>
-      </c>
-      <c r="D41" s="24" t="n">
-        <f aca="false">$B$22/($B$23*D34)</f>
-        <v>0.316666666666667</v>
-      </c>
-      <c r="E41" s="24" t="n">
-        <f aca="false">$B$22/($B$23*E34)</f>
-        <v>0.633333333333333</v>
-      </c>
-      <c r="F41" s="24" t="n">
-        <f aca="false">$B$22/($B$23*F34)</f>
-        <v>0.633333333333333</v>
-      </c>
-      <c r="G41" s="24" t="n">
-        <f aca="false">$B$22/($B$23*G34)</f>
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="B42" s="24" t="n">
-        <f aca="false">SUM(B37:B41)</f>
-        <v>24.6041666666667</v>
-      </c>
-      <c r="C42" s="24" t="n">
-        <f aca="false">SUM(C37:C41)</f>
-        <v>26.2041666666667</v>
-      </c>
-      <c r="D42" s="24" t="n">
-        <f aca="false">SUM(D37:D41)</f>
-        <v>27.8041666666667</v>
-      </c>
-      <c r="E42" s="24" t="n">
-        <f aca="false">SUM(E37:E41)</f>
-        <v>25.6983333333333</v>
-      </c>
-      <c r="F42" s="24" t="n">
-        <f aca="false">SUM(F37:F41)</f>
-        <v>24.3478333333333</v>
-      </c>
-      <c r="G42" s="24" t="n">
-        <f aca="false">SUM(G37:G41)</f>
-        <v>116.6305</v>
-      </c>
-    </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B43" s="24" t="n">
-        <f aca="false">B30-$B$18*B31</f>
-        <v>221.44908902476</v>
+        <f aca="false">B35*$B$19*$B$26*$B$20</f>
+        <v>0.2695</v>
       </c>
       <c r="C43" s="24" t="n">
-        <f aca="false">C30-$B$18*C31</f>
-        <v>259.796949703949</v>
+        <f aca="false">C35*$B$19*$B$26*$B$20</f>
+        <v>0.2695</v>
       </c>
       <c r="D43" s="24" t="n">
-        <f aca="false">D30-$B$18*D31</f>
-        <v>295.628289706394</v>
+        <f aca="false">D35*$B$19*$B$26*$B$20</f>
+        <v>0.2695</v>
       </c>
       <c r="E43" s="24" t="n">
-        <f aca="false">E30-$B$18*E31</f>
-        <v>130.937038961209</v>
+        <f aca="false">E35*$B$19*$B$26*$B$20</f>
+        <v>0.847</v>
       </c>
       <c r="F43" s="24" t="n">
-        <f aca="false">F30-$B$18*F31</f>
-        <v>89.6071409887996</v>
+        <f aca="false">F35*$B$19*$B$26*$B$20</f>
+        <v>0.9065</v>
       </c>
       <c r="G43" s="24" t="n">
-        <f aca="false">G30-$B$18*G31</f>
-        <v>1151.36118184947</v>
+        <f aca="false">G35*$B$19*$B$26*$B$20</f>
+        <v>3.0625</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="25" t="s">
-        <v>247</v>
-      </c>
-      <c r="B44" s="26" t="n">
-        <f aca="false">$B$21*B43-B42</f>
-        <v>152.555104553141</v>
-      </c>
-      <c r="C44" s="26" t="n">
-        <f aca="false">$B$21*C43-C42</f>
-        <v>181.633393096492</v>
-      </c>
-      <c r="D44" s="26" t="n">
-        <f aca="false">$B$21*D43-D42</f>
-        <v>208.698465098448</v>
-      </c>
-      <c r="E44" s="26" t="n">
-        <f aca="false">$B$21*E43-E42</f>
-        <v>79.0512978356341</v>
-      </c>
-      <c r="F44" s="26" t="n">
-        <f aca="false">$B$21*F43-F42</f>
-        <v>47.3378794577064</v>
-      </c>
-      <c r="G44" s="26" t="n">
-        <f aca="false">$B$21*G43-G42</f>
-        <v>804.458445479572</v>
+      <c r="A44" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="B44" s="24" t="n">
+        <f aca="false">$B$22/($B$23*B37)</f>
+        <v>0.316666666666667</v>
+      </c>
+      <c r="C44" s="24" t="n">
+        <f aca="false">$B$22/($B$23*C37)</f>
+        <v>0.316666666666667</v>
+      </c>
+      <c r="D44" s="24" t="n">
+        <f aca="false">$B$22/($B$23*D37)</f>
+        <v>0.316666666666667</v>
+      </c>
+      <c r="E44" s="24" t="n">
+        <f aca="false">$B$22/($B$23*E37)</f>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="F44" s="24" t="n">
+        <f aca="false">$B$22/($B$23*F37)</f>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="G44" s="24" t="n">
+        <f aca="false">$B$22/($B$23*G37)</f>
+        <v>3.8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="25" t="s">
-        <v>248</v>
-      </c>
-      <c r="B45" s="27" t="n">
-        <f aca="false">B44-B36</f>
-        <v>-4.60416666666666</v>
-      </c>
-      <c r="C45" s="27" t="n">
-        <f aca="false">C44-C36</f>
-        <v>-6.20416666666665</v>
-      </c>
-      <c r="D45" s="27" t="n">
-        <f aca="false">D44-D36</f>
-        <v>-7.80416666666667</v>
-      </c>
-      <c r="E45" s="27" t="n">
-        <f aca="false">E44-E36</f>
-        <v>-5.69833333333332</v>
-      </c>
-      <c r="F45" s="27" t="n">
-        <f aca="false">F44-F36</f>
-        <v>-4.34783333333333</v>
-      </c>
-      <c r="G45" s="27" t="n">
-        <f aca="false">G44-G36</f>
-        <v>-96.6305</v>
+      <c r="A45" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="B45" s="6" t="n">
+        <f aca="false">Stock_Hub!$B$28/Stock_Hub!$B$31</f>
+        <v>2.14285714285714</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <f aca="false">Stock_Hub!$B$28/Stock_Hub!$B$31</f>
+        <v>2.14285714285714</v>
+      </c>
+      <c r="D45" s="6" t="n">
+        <f aca="false">Stock_Hub!$B$28/Stock_Hub!$B$31</f>
+        <v>2.14285714285714</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <f aca="false">Stock_Hub!$B$28/Stock_Hub!$B$31</f>
+        <v>2.14285714285714</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <f aca="false">Stock_Hub!$B$28/Stock_Hub!$B$31</f>
+        <v>2.14285714285714</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <f aca="false">Stock_Hub!$B$28/Stock_Hub!$B$31</f>
+        <v>2.14285714285714</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="25" t="s">
-        <v>249</v>
-      </c>
-      <c r="B46" s="42" t="n">
-        <f aca="false">IF(B45&lt;0,-B45/B43,0)</f>
-        <v>0.0207910842484968</v>
-      </c>
-      <c r="C46" s="42" t="n">
-        <f aca="false">IF(C45&lt;0,-C45/C43,0)</f>
-        <v>0.0238808295237361</v>
-      </c>
-      <c r="D46" s="42" t="n">
-        <f aca="false">IF(D45&lt;0,-D45/D43,0)</f>
-        <v>0.026398578682769</v>
-      </c>
-      <c r="E46" s="42" t="n">
-        <f aca="false">IF(E45&lt;0,-E45/E43,0)</f>
-        <v>0.04351964408651</v>
-      </c>
-      <c r="F46" s="42" t="n">
-        <f aca="false">IF(F45&lt;0,-F45/F43,0)</f>
-        <v>0.0485210585379215</v>
-      </c>
-      <c r="G46" s="42" t="n">
-        <f aca="false">IF(G45&lt;0,-G45/G43,0)</f>
-        <v>0.0839271824717762</v>
+      <c r="A46" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="B46" s="24" t="n">
+        <f aca="false">SUM(B40:B45)</f>
+        <v>29.4970238095238</v>
+      </c>
+      <c r="C46" s="24" t="n">
+        <f aca="false">SUM(C40:C45)</f>
+        <v>31.0970238095238</v>
+      </c>
+      <c r="D46" s="24" t="n">
+        <f aca="false">SUM(D40:D45)</f>
+        <v>32.6970238095238</v>
+      </c>
+      <c r="E46" s="24" t="n">
+        <f aca="false">SUM(E40:E45)</f>
+        <v>30.5911904761905</v>
+      </c>
+      <c r="F46" s="24" t="n">
+        <f aca="false">SUM(F40:F45)</f>
+        <v>29.2406904761905</v>
+      </c>
+      <c r="G46" s="24" t="n">
+        <f aca="false">SUM(G40:G45)</f>
+        <v>121.523357142857</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="25" t="s">
-        <v>250</v>
-      </c>
-      <c r="B47" s="40" t="n">
-        <f aca="false">($B$21*B43-(B37+B39+B40+B41)-B36)/(B29*$B$21)</f>
-        <v>0.0207518115942029</v>
-      </c>
-      <c r="C47" s="40" t="n">
-        <f aca="false">($B$21*C43-(C37+C39+C40+C41)-C36)/(C29*$B$21)</f>
-        <v>0.0177787726838586</v>
-      </c>
-      <c r="D47" s="40" t="n">
-        <f aca="false">($B$21*D43-(D37+D39+D40+D41)-D36)/(D29*$B$21)</f>
-        <v>0.0155508563074352</v>
-      </c>
-      <c r="E47" s="40" t="n">
-        <f aca="false">($B$21*E43-(E37+E39+E40+E41)-E36)/(E29*$B$21)</f>
-        <v>0.00747526636225269</v>
-      </c>
-      <c r="F47" s="40" t="n">
-        <f aca="false">($B$21*F43-(F37+F39+F40+F41)-F36)/(F29*$B$21)</f>
-        <v>0.00581892033542977</v>
-      </c>
-      <c r="G47" s="40" t="n">
-        <f aca="false">($B$21*G43-(G37+G39+G40+G41)-G36)/(G29*$B$21)</f>
-        <v>-0.0125394193127447</v>
+      <c r="A47" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="B47" s="24" t="n">
+        <f aca="false">B33-$B$18*B34</f>
+        <v>230.96991902476</v>
+      </c>
+      <c r="C47" s="24" t="n">
+        <f aca="false">C33-$B$18*C34</f>
+        <v>270.826279703949</v>
+      </c>
+      <c r="D47" s="24" t="n">
+        <f aca="false">D33-$B$18*D34</f>
+        <v>308.166119706394</v>
+      </c>
+      <c r="E47" s="24" t="n">
+        <f aca="false">E33-$B$18*E34</f>
+        <v>138.044268961209</v>
+      </c>
+      <c r="F47" s="24" t="n">
+        <f aca="false">F33-$B$18*F34</f>
+        <v>94.9041709887997</v>
+      </c>
+      <c r="G47" s="24" t="n">
+        <f aca="false">G33-$B$18*G34</f>
+        <v>1221.22201184947</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="25" t="s">
+        <v>253</v>
+      </c>
+      <c r="B48" s="26" t="n">
+        <f aca="false">$B$21*B47-B46</f>
+        <v>155.278911410284</v>
+      </c>
+      <c r="C48" s="26" t="n">
+        <f aca="false">$B$21*C47-C46</f>
+        <v>185.563999953635</v>
+      </c>
+      <c r="D48" s="26" t="n">
+        <f aca="false">$B$21*D47-D46</f>
+        <v>213.835871955591</v>
+      </c>
+      <c r="E48" s="26" t="n">
+        <f aca="false">$B$21*E47-E46</f>
+        <v>79.844224692777</v>
+      </c>
+      <c r="F48" s="26" t="n">
+        <f aca="false">$B$21*F47-F46</f>
+        <v>46.6826463148492</v>
+      </c>
+      <c r="G48" s="26" t="n">
+        <f aca="false">$B$21*G47-G46</f>
+        <v>855.454252336715</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
-        <v>251</v>
+      <c r="A49" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="B49" s="27" t="n">
+        <f aca="false">B48-B39</f>
+        <v>-1.88035980952384</v>
+      </c>
+      <c r="C49" s="27" t="n">
+        <f aca="false">C48-C39</f>
+        <v>-2.27355980952382</v>
+      </c>
+      <c r="D49" s="27" t="n">
+        <f aca="false">D48-D39</f>
+        <v>-2.66675980952382</v>
+      </c>
+      <c r="E49" s="27" t="n">
+        <f aca="false">E48-E39</f>
+        <v>-4.90540647619049</v>
+      </c>
+      <c r="F49" s="27" t="n">
+        <f aca="false">F48-F39</f>
+        <v>-5.00306647619048</v>
+      </c>
+      <c r="G49" s="27" t="n">
+        <f aca="false">G48-G39</f>
+        <v>-45.6346931428571</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2" t="s">
-        <v>252</v>
+      <c r="A50" s="25" t="s">
+        <v>255</v>
+      </c>
+      <c r="B50" s="42" t="n">
+        <f aca="false">IF(B49&lt;0,-B49/B47,0)</f>
+        <v>0.00814114590100482</v>
+      </c>
+      <c r="C50" s="42" t="n">
+        <f aca="false">IF(C49&lt;0,-C49/C47,0)</f>
+        <v>0.00839490101185579</v>
+      </c>
+      <c r="D50" s="42" t="n">
+        <f aca="false">IF(D49&lt;0,-D49/D47,0)</f>
+        <v>0.00865364372976688</v>
+      </c>
+      <c r="E50" s="42" t="n">
+        <f aca="false">IF(E49&lt;0,-E49/E47,0)</f>
+        <v>0.0355350244751481</v>
+      </c>
+      <c r="F50" s="42" t="n">
+        <f aca="false">IF(F49&lt;0,-F49/F47,0)</f>
+        <v>0.0527170347105285</v>
+      </c>
+      <c r="G50" s="42" t="n">
+        <f aca="false">IF(G49&lt;0,-G49/G47,0)</f>
+        <v>0.0373680565041128</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="s">
-        <v>253</v>
+      <c r="A51" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="B51" s="40" t="n">
+        <f aca="false">($B$21*B47-(B40+B42+B43+B44)-B39)/(B32*$B$21)</f>
+        <v>0.0410973968784837</v>
+      </c>
+      <c r="C51" s="40" t="n">
+        <f aca="false">($B$21*C47-(C40+C42+C43+C44)-C39)/(C32*$B$21)</f>
+        <v>0.0395318672397326</v>
+      </c>
+      <c r="D51" s="40" t="n">
+        <f aca="false">($B$21*D47-(D40+D42+D43+D44)-D39)/(D32*$B$21)</f>
+        <v>0.038358700918964</v>
+      </c>
+      <c r="E51" s="40" t="n">
+        <f aca="false">($B$21*E47-(E40+E42+E43+E44)-E39)/(E32*$B$21)</f>
+        <v>0.0242320243531202</v>
+      </c>
+      <c r="F51" s="40" t="n">
+        <f aca="false">($B$21*F47-(F40+F42+F43+F44)-F39)/(F32*$B$21)</f>
+        <v>0.0175140775681342</v>
+      </c>
+      <c r="G51" s="40" t="n">
+        <f aca="false">($B$21*G47-(G40+G42+G43+G44)-G39)/(G32*$B$21)</f>
+        <v>0.0163528512396695</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="B55" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="C55" s="20" t="n">
+        <v>75</v>
+      </c>
+      <c r="D55" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E55" s="20" t="n">
+        <v>150</v>
+      </c>
+      <c r="F55" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="G55" s="20" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="25" t="s">
+        <v>259</v>
+      </c>
+      <c r="B56" s="27" t="n">
+        <f aca="false">$C$49+($B$28-$B$11*MAX($B$25,B55)/B55)</f>
+        <v>-10.5235598095238</v>
+      </c>
+      <c r="C56" s="27" t="n">
+        <f aca="false">$C$49+($B$28-$B$11*MAX($B$25,C55)/C55)</f>
+        <v>-5.02355980952382</v>
+      </c>
+      <c r="D56" s="27" t="n">
+        <f aca="false">$C$49+($B$28-$B$11*MAX($B$25,D55)/D55)</f>
+        <v>-2.27355980952382</v>
+      </c>
+      <c r="E56" s="27" t="n">
+        <f aca="false">$C$49+($B$28-$B$11*MAX($B$25,E55)/E55)</f>
+        <v>0.476440190476183</v>
+      </c>
+      <c r="F56" s="27" t="n">
+        <f aca="false">$C$49+($B$28-$B$11*MAX($B$25,F55)/F55)</f>
+        <v>0.476440190476183</v>
+      </c>
+      <c r="G56" s="27" t="n">
+        <f aca="false">$C$49+($B$28-$B$11*MAX($B$25,G55)/G55)</f>
+        <v>0.476440190476183</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -6198,6 +6480,453 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>265</v>
+      </c>
+      <c r="B4" s="43" t="n">
+        <f aca="false">Courier_Hub!B24/30</f>
+        <v>3.33333333333333</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="B7" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="B8" s="32" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B9" s="45" t="n">
+        <f aca="false">Courier_Hub!B23</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B10" s="14" t="n">
+        <f aca="false">Courier_Hub!B22</f>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B11" s="34" t="n">
+        <f aca="false">Supuestos!B5</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="46" t="n">
+        <f aca="false">Courier_Hub!B19</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>275</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>276</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>277</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>278</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="B15" s="38" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C15" s="47" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B15</f>
+        <v>62</v>
+      </c>
+      <c r="D15" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="47" t="n">
+        <f aca="false">C15/D15</f>
+        <v>5.16666666666667</v>
+      </c>
+      <c r="F15" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="G15" s="48" t="n">
+        <f aca="false">C15*F15</f>
+        <v>0.4774</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="B16" s="38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C16" s="47" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B16</f>
+        <v>10.3333333333333</v>
+      </c>
+      <c r="D16" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="47" t="n">
+        <f aca="false">C16/D16</f>
+        <v>0.861111111111111</v>
+      </c>
+      <c r="F16" s="41" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="G16" s="48" t="n">
+        <f aca="false">C16*F16</f>
+        <v>0.0795666666666667</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" s="38" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C17" s="47" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B17</f>
+        <v>12.4</v>
+      </c>
+      <c r="D17" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="47" t="n">
+        <f aca="false">C17/D17</f>
+        <v>2.06666666666667</v>
+      </c>
+      <c r="F17" s="41" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="G17" s="48" t="n">
+        <f aca="false">C17*F17</f>
+        <v>0.30008</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="B18" s="38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C18" s="47" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B18</f>
+        <v>10.3333333333333</v>
+      </c>
+      <c r="D18" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="47" t="n">
+        <f aca="false">C18/D18</f>
+        <v>1.72222222222222</v>
+      </c>
+      <c r="F18" s="41" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="G18" s="48" t="n">
+        <f aca="false">C18*F18</f>
+        <v>0.267633333333333</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="B19" s="38" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C19" s="47" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B19</f>
+        <v>3.1</v>
+      </c>
+      <c r="D19" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="47" t="n">
+        <f aca="false">C19/D19</f>
+        <v>3.1</v>
+      </c>
+      <c r="F19" s="41" t="n">
+        <v>0.0875</v>
+      </c>
+      <c r="G19" s="48" t="n">
+        <f aca="false">C19*F19</f>
+        <v>0.27125</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="B20" s="38" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C20" s="47" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B20</f>
+        <v>5.16666666666667</v>
+      </c>
+      <c r="D20" s="39" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E20" s="47" t="n">
+        <f aca="false">C20/D20</f>
+        <v>0.449275362318841</v>
+      </c>
+      <c r="F20" s="41" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="G20" s="48" t="n">
+        <f aca="false">C20*F20</f>
+        <v>0.031</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="B21" s="42" t="n">
+        <f aca="false">SUM(B15:B20)</f>
+        <v>1</v>
+      </c>
+      <c r="C21" s="49" t="n">
+        <f aca="false">SUM(C15:C20)</f>
+        <v>103.333333333333</v>
+      </c>
+      <c r="E21" s="49" t="n">
+        <f aca="false">SUM(E15:E20)</f>
+        <v>13.3659420289855</v>
+      </c>
+      <c r="G21" s="50" t="n">
+        <f aca="false">SUM(G15:G20)</f>
+        <v>1.42693</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="B24" s="47" t="n">
+        <f aca="false">MAX($B$7,E21/$B$9)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="B25" s="24" t="n">
+        <f aca="false">B24*$B$10</f>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="B26" s="47" t="n">
+        <f aca="false">30/$B$5</f>
+        <v>1.07142857142857</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="B27" s="24" t="n">
+        <f aca="false">B25*B26</f>
+        <v>122.142857142857</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="B28" s="24" t="n">
+        <f aca="false">$B$8*B26</f>
+        <v>214.285714285714</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="B29" s="24" t="n">
+        <f aca="false">G21*$B$12*$B$11</f>
+        <v>99.8851</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="25" t="s">
+        <v>289</v>
+      </c>
+      <c r="B30" s="26" t="n">
+        <f aca="false">B27+B28+B29</f>
+        <v>436.313671428571</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="B31" s="35" t="n">
+        <f aca="false">B4*30</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="B32" s="24" t="n">
+        <f aca="false">Courier_Hub!B11*MAX(Courier_Hub!B25,B31)</f>
+        <v>825</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="25" t="s">
+        <v>292</v>
+      </c>
+      <c r="B33" s="29" t="n">
+        <f aca="false">(B30+B32)/B31</f>
+        <v>12.6131367142857</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="B34" s="18" t="n">
+        <f aca="false">(Supuestos!B16*B31+Supuestos!B36)/B31</f>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="25" t="s">
+        <v>294</v>
+      </c>
+      <c r="B35" s="36" t="n">
+        <f aca="false">B33-B34</f>
+        <v>5.11313671428572</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -6207,12 +6936,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>254</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>255</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6231,7 +6960,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>256</v>
+        <v>298</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>1008</v>
@@ -6246,7 +6975,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1000</v>
@@ -6261,7 +6990,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>258</v>
+        <v>300</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>500</v>
@@ -6276,7 +7005,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>259</v>
+        <v>301</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>5</v>
@@ -6291,7 +7020,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>260</v>
+        <v>302</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>1</v>
@@ -6306,7 +7035,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>261</v>
+        <v>303</v>
       </c>
       <c r="D10" s="29" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -6315,17 +7044,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>262</v>
+        <v>304</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>263</v>
+        <v>305</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>264</v>
+        <v>306</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>1135.87</v>
@@ -6333,7 +7062,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>265</v>
+        <v>307</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>135.13</v>
@@ -6341,7 +7070,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>266</v>
+        <v>308</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>1720</v>
@@ -6349,7 +7078,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>267</v>
+        <v>309</v>
       </c>
       <c r="B17" s="13" t="n">
         <v>309.6</v>
@@ -6357,7 +7086,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>268</v>
+        <v>310</v>
       </c>
       <c r="B18" s="13" t="n">
         <v>5961</v>
@@ -6365,7 +7094,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>269</v>
+        <v>311</v>
       </c>
       <c r="B19" s="15" t="n">
         <v>1</v>
@@ -6382,17 +7111,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>270</v>
+        <v>312</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>271</v>
+        <v>313</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>272</v>
+        <v>314</v>
       </c>
       <c r="B24" s="18" t="n">
         <f aca="false">D10*B20</f>
@@ -6401,7 +7130,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>273</v>
+        <v>315</v>
       </c>
       <c r="B25" s="18" t="n">
         <f aca="false">B14*B20</f>
@@ -6410,7 +7139,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>274</v>
+        <v>316</v>
       </c>
       <c r="B26" s="18" t="n">
         <f aca="false">B16+B17</f>
@@ -6428,7 +7157,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="25" t="s">
-        <v>275</v>
+        <v>317</v>
       </c>
       <c r="B28" s="29" t="n">
         <f aca="false">SUM(B24:B27)</f>
@@ -6437,7 +7166,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>276</v>
+        <v>318</v>
       </c>
       <c r="B29" s="18" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -6464,7 +7193,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>277</v>
+        <v>319</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6472,24 +7201,24 @@
         <v>2</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>278</v>
+        <v>320</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>279</v>
+        <v>321</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>280</v>
+        <v>322</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>281</v>
+        <v>323</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>282</v>
+        <v>324</v>
       </c>
       <c r="B35" s="18" t="n">
         <f aca="false">D5</f>
@@ -6514,7 +7243,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>283</v>
+        <v>325</v>
       </c>
       <c r="B36" s="18" t="n">
         <f aca="false">D6</f>
@@ -6539,7 +7268,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>284</v>
+        <v>326</v>
       </c>
       <c r="B37" s="18" t="n">
         <f aca="false">D7</f>
@@ -6581,7 +7310,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>285</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Hoja Courier_Dinsides: comparacion del servicio de almacen y despacho de Dinsides
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -18,8 +18,9 @@
     <sheet name="Desglose" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Contenedor2" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Courier_Hub" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="Stock_Hub" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="Costo_Lima" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Courier_Dinsides" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Stock_Hub" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Costo_Lima" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="554">
   <si>
     <t xml:space="preserve">Plan hacia US$ 1M de utilidad anual - resumen de escenarios</t>
   </si>
@@ -1378,6 +1379,129 @@
   </si>
   <si>
     <t xml:space="preserve">No incluye: beneficio tributario de la factura de The Hub (IGV y gasto deducible) (el transporte desde tu almacen a The Hub viene de la hoja Stock_Hub). Para bidones y Cero el courier actual (S/ 12.5) es solo una referencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinsides (almacen + despacho) vs operacion actual vs The Hub - Lima, contraentrega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente: brochure de fulfillment de Dinsides. El brochure NO trae tarifas de envio ni cobro por contraentrega: se usa el courier actual de S/ 10-15. Azul/amarillo = supuesto o dato pendiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condiciones de Dinsides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Courier Lima por pedido (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinsides al dia siguiente: S/ 10-15 (dato del usuario).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material de empaque por pedido (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO: Dinsides exige que el cliente provea bolsas, cajas y film.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo por pedido armado y no entregado (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brochure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almacenaje y armado de pedidos (S/ por pedido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brochure: almacenaje sin costo adicional.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobro contraentrega de Dinsides (% del valor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDIENTE: el brochure no lo menciona. Confirmar efectivo, POS y cuotas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega efectiva con Dinsides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Igual a la actual para comparar costos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos al mes en Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene de Courier_Hub.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entregas por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimo de entregas por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penalidad por no cumplir el minimo (S/ por dia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brochure. Se asume que se cobra todos los dias del mes si no se cumple.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penalidad por pedido (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO: igual que The Hub, por falta de tarifa de Dinsides para bultos grandes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTUAL (Tecretail + courier): utilidad antes de publicidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINSIDES: courier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINSIDES: material de empaque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINSIDES: pedidos armados y no entregados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINSIDES: penalidad por el minimo semanal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINSIDES: cobro contraentrega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINSIDES: logistica por pedido colocado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINSIDES: utilidad antes de publicidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THE HUB: utilidad antes de publicidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinsides - actual (utilidad por pedido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinsides - The Hub (utilidad por pedido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puntos de entrega que The Hub debe ganar para igualar a Dinsides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ahorro mensual de Dinsides segun volumen (Nativo 3 años, S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinsides vs operacion actual (S/ al mes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinsides vs The Hub (S/ al mes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura: el brochure incluye almacen, armado, rotulado, seguro por robo y perdida, control de inventario 3 veces por semana y punto de recojo en su almacen. No incluye materiales de empaque.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El ahorro es de costo, no de entrega efectiva: si Dinsides entrega igual que hoy (80%), el ahorro es el de la fila 30. Por eso pedir su tasa de entrega por distrito antes de decidir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En el brochure los S/ 2.00 por pedido armado y no entregado reemplazan al costo de gestion; no hay cobro por almacenaje. Confirmar si ese cobro de S/ 2.00 es adicional al reintento o a la devolucion.</t>
   </si>
   <si>
     <t xml:space="preserve">Plan de stock en The Hub: tandas desde tu almacen propio</t>
@@ -1732,7 +1856,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1961,11 +2085,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3641,10 +3769,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
   </cols>
   <sheetData>
@@ -3658,418 +3786,710 @@
         <v>450</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+    </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>451</v>
-      </c>
-      <c r="B4" s="53" t="n">
-        <f aca="false">Courier_Hub!B24/30</f>
-        <v>3.33333333333333</v>
+        <v>452</v>
+      </c>
+      <c r="B4" s="17" t="n">
+        <f aca="false">Supuestos!B18</f>
+        <v>12.5</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>453</v>
-      </c>
-      <c r="B5" s="39" t="n">
-        <v>28</v>
+        <v>454</v>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>1.5</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>455</v>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" s="2"/>
+        <v>456</v>
+      </c>
+      <c r="B6" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>457</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="B7" s="30" t="n">
-        <v>1</v>
+        <v>458</v>
+      </c>
+      <c r="B7" s="38" t="n">
+        <v>0</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>458</v>
-      </c>
-      <c r="B8" s="23" t="n">
-        <v>200</v>
+        <v>460</v>
+      </c>
+      <c r="B8" s="51" t="n">
+        <v>0</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="B9" s="57" t="n">
-        <f aca="false">Courier_Hub!B23</f>
-        <v>30</v>
+        <v>462</v>
+      </c>
+      <c r="B9" s="36" t="n">
+        <f aca="false">Supuestos!B7</f>
+        <v>0.8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>460</v>
-      </c>
-      <c r="B10" s="17" t="n">
-        <f aca="false">Courier_Hub!B22</f>
-        <v>114</v>
+        <v>464</v>
+      </c>
+      <c r="B10" s="35" t="n">
+        <f aca="false">Courier_Hub!B24</f>
+        <v>100</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="25" t="n">
-        <f aca="false">Supuestos!B5</f>
-        <v>3.5</v>
-      </c>
+        <v>466</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <f aca="false">B10/4.33</f>
+        <v>23.094688221709</v>
+      </c>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="B12" s="58" t="n">
-        <f aca="false">Courier_Hub!B19</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="44" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="44" t="s">
-        <v>461</v>
-      </c>
-      <c r="C14" s="44" t="s">
-        <v>462</v>
-      </c>
-      <c r="D14" s="44" t="s">
-        <v>428</v>
-      </c>
-      <c r="E14" s="44" t="s">
-        <v>463</v>
-      </c>
-      <c r="F14" s="44" t="s">
-        <v>464</v>
-      </c>
-      <c r="G14" s="44" t="s">
-        <v>465</v>
-      </c>
+        <v>467</v>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B13" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="B14" s="42" t="n">
+        <f aca="false">IF(B11&lt;B12,B13*30,0)/B10</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>466</v>
-      </c>
-      <c r="B15" s="19" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <f aca="false">$B$4*($B$5+$B$6)*B15</f>
-        <v>62</v>
-      </c>
-      <c r="D15" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <f aca="false">C15/D15</f>
-        <v>5.16666666666667</v>
-      </c>
-      <c r="F15" s="55" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="G15" s="59" t="n">
-        <f aca="false">C15*F15</f>
-        <v>0.4774</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="B16" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C16" s="7" t="n">
-        <f aca="false">$B$4*($B$5+$B$6)*B16</f>
-        <v>10.3333333333333</v>
-      </c>
-      <c r="D16" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <f aca="false">C16/D16</f>
-        <v>0.861111111111111</v>
-      </c>
-      <c r="F16" s="55" t="n">
-        <v>0.0077</v>
-      </c>
-      <c r="G16" s="59" t="n">
-        <f aca="false">C16*F16</f>
-        <v>0.0795666666666667</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B15" s="57" t="n">
+        <f aca="false">Courier_Hub!B13</f>
+        <v>1.5</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="44" t="s">
+        <v>308</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>259</v>
+      </c>
+      <c r="C17" s="44" t="s">
+        <v>260</v>
+      </c>
+      <c r="D17" s="44" t="s">
+        <v>261</v>
+      </c>
+      <c r="E17" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="19" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <f aca="false">$B$4*($B$5+$B$6)*B17</f>
-        <v>12.4</v>
-      </c>
-      <c r="D17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <f aca="false">C17/D17</f>
-        <v>2.06666666666667</v>
-      </c>
-      <c r="F17" s="55" t="n">
-        <v>0.0242</v>
-      </c>
-      <c r="G17" s="59" t="n">
-        <f aca="false">C17*F17</f>
-        <v>0.30008</v>
+      <c r="F17" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" s="44" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C18" s="7" t="n">
-        <f aca="false">$B$4*($B$5+$B$6)*B18</f>
-        <v>10.3333333333333</v>
-      </c>
-      <c r="D18" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <f aca="false">C18/D18</f>
-        <v>1.72222222222222</v>
-      </c>
-      <c r="F18" s="55" t="n">
-        <v>0.0259</v>
-      </c>
-      <c r="G18" s="59" t="n">
-        <f aca="false">C18*F18</f>
-        <v>0.267633333333333</v>
+        <v>423</v>
+      </c>
+      <c r="B18" s="35" t="n">
+        <f aca="false">Courier_Hub!B32</f>
+        <v>299</v>
+      </c>
+      <c r="C18" s="35" t="n">
+        <f aca="false">Courier_Hub!C32</f>
+        <v>349</v>
+      </c>
+      <c r="D18" s="35" t="n">
+        <f aca="false">Courier_Hub!D32</f>
+        <v>399</v>
+      </c>
+      <c r="E18" s="35" t="n">
+        <f aca="false">Courier_Hub!E32</f>
+        <v>219</v>
+      </c>
+      <c r="F18" s="35" t="n">
+        <f aca="false">Courier_Hub!F32</f>
+        <v>159</v>
+      </c>
+      <c r="G18" s="35" t="n">
+        <f aca="false">Courier_Hub!G32</f>
+        <v>2299</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="19" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <f aca="false">$B$4*($B$5+$B$6)*B19</f>
-        <v>3.1</v>
-      </c>
-      <c r="D19" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <f aca="false">C19/D19</f>
-        <v>3.1</v>
-      </c>
-      <c r="F19" s="55" t="n">
-        <v>0.0875</v>
-      </c>
-      <c r="G19" s="59" t="n">
-        <f aca="false">C19*F19</f>
-        <v>0.27125</v>
+        <v>424</v>
+      </c>
+      <c r="B19" s="27" t="n">
+        <f aca="false">Courier_Hub!B33</f>
+        <v>221.44908902476</v>
+      </c>
+      <c r="C19" s="27" t="n">
+        <f aca="false">Courier_Hub!C33</f>
+        <v>259.796949703949</v>
+      </c>
+      <c r="D19" s="27" t="n">
+        <f aca="false">Courier_Hub!D33</f>
+        <v>295.628289706394</v>
+      </c>
+      <c r="E19" s="27" t="n">
+        <f aca="false">Courier_Hub!E33</f>
+        <v>130.937038961209</v>
+      </c>
+      <c r="F19" s="27" t="n">
+        <f aca="false">Courier_Hub!F33</f>
+        <v>89.6071409887996</v>
+      </c>
+      <c r="G19" s="27" t="n">
+        <f aca="false">Courier_Hub!G33</f>
+        <v>1151.36118184947</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="B20" s="19" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <f aca="false">$B$4*($B$5+$B$6)*B20</f>
-        <v>5.16666666666667</v>
-      </c>
-      <c r="D20" s="20" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <f aca="false">C20/D20</f>
-        <v>0.449275362318841</v>
-      </c>
-      <c r="F20" s="55" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="G20" s="59" t="n">
-        <f aca="false">C20*F20</f>
-        <v>0.031</v>
+        <v>427</v>
+      </c>
+      <c r="B20" s="58" t="n">
+        <f aca="false">Courier_Hub!B36</f>
+        <v>1.5</v>
+      </c>
+      <c r="C20" s="58" t="n">
+        <f aca="false">Courier_Hub!C36</f>
+        <v>1.5</v>
+      </c>
+      <c r="D20" s="58" t="n">
+        <f aca="false">Courier_Hub!D36</f>
+        <v>2</v>
+      </c>
+      <c r="E20" s="58" t="n">
+        <f aca="false">Courier_Hub!E36</f>
+        <v>4.84</v>
+      </c>
+      <c r="F20" s="58" t="n">
+        <f aca="false">Courier_Hub!F36</f>
+        <v>5.18</v>
+      </c>
+      <c r="G20" s="58" t="n">
+        <f aca="false">Courier_Hub!G36</f>
+        <v>17.5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="B21" s="56" t="n">
-        <f aca="false">SUM(B15:B20)</f>
-        <v>1</v>
-      </c>
-      <c r="C21" s="60" t="n">
-        <f aca="false">SUM(C15:C20)</f>
-        <v>103.333333333333</v>
-      </c>
-      <c r="E21" s="60" t="n">
-        <f aca="false">SUM(E15:E20)</f>
-        <v>13.3659420289855</v>
-      </c>
-      <c r="G21" s="61" t="n">
-        <f aca="false">SUM(G15:G20)</f>
-        <v>1.42693</v>
+        <v>472</v>
+      </c>
+      <c r="B21" s="27" t="n">
+        <f aca="false">Courier_Hub!B39</f>
+        <v>157.159271219808</v>
+      </c>
+      <c r="C21" s="27" t="n">
+        <f aca="false">Courier_Hub!C39</f>
+        <v>187.837559763159</v>
+      </c>
+      <c r="D21" s="27" t="n">
+        <f aca="false">Courier_Hub!D39</f>
+        <v>216.502631765115</v>
+      </c>
+      <c r="E21" s="27" t="n">
+        <f aca="false">Courier_Hub!E39</f>
+        <v>84.7496311689675</v>
+      </c>
+      <c r="F21" s="27" t="n">
+        <f aca="false">Courier_Hub!F39</f>
+        <v>51.6857127910397</v>
+      </c>
+      <c r="G21" s="27" t="n">
+        <f aca="false">Courier_Hub!G39</f>
+        <v>901.088945479572</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="B22" s="6" t="n">
+        <f aca="false">$B$4+MAX(0,B20-3)*$B$15</f>
+        <v>12.5</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <f aca="false">$B$4+MAX(0,C20-3)*$B$15</f>
+        <v>12.5</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <f aca="false">$B$4+MAX(0,D20-3)*$B$15</f>
+        <v>12.5</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <f aca="false">$B$4+MAX(0,E20-3)*$B$15</f>
+        <v>15.26</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <f aca="false">$B$4+MAX(0,F20-3)*$B$15</f>
+        <v>15.77</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <f aca="false">$B$4+MAX(0,G20-3)*$B$15</f>
+        <v>34.25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>468</v>
-      </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
+      <c r="A23" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="B23" s="6" t="n">
+        <f aca="false">$B$5</f>
+        <v>1.5</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <f aca="false">$B$5</f>
+        <v>1.5</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <f aca="false">$B$5</f>
+        <v>1.5</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <f aca="false">$B$5</f>
+        <v>1.5</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <f aca="false">$B$5</f>
+        <v>1.5</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <f aca="false">$B$5</f>
+        <v>1.5</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>469</v>
-      </c>
-      <c r="B24" s="7" t="n">
-        <f aca="false">MAX($B$7,E21/$B$9)</f>
-        <v>1</v>
+        <v>475</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <f aca="false">(1-$B$9)*$B$6</f>
+        <v>0.4</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <f aca="false">(1-$B$9)*$B$6</f>
+        <v>0.4</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <f aca="false">(1-$B$9)*$B$6</f>
+        <v>0.4</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <f aca="false">(1-$B$9)*$B$6</f>
+        <v>0.4</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <f aca="false">(1-$B$9)*$B$6</f>
+        <v>0.4</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <f aca="false">(1-$B$9)*$B$6</f>
+        <v>0.4</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="B25" s="6" t="n">
-        <f aca="false">B24*$B$10</f>
-        <v>114</v>
+        <f aca="false">$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <f aca="false">$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <f aca="false">$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <f aca="false">$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <f aca="false">$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <f aca="false">$B$14</f>
+        <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>471</v>
-      </c>
-      <c r="B26" s="7" t="n">
-        <f aca="false">30/$B$5</f>
-        <v>1.07142857142857</v>
+        <v>477</v>
+      </c>
+      <c r="B26" s="6" t="n">
+        <f aca="false">$B$8*B18*$B$9</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <f aca="false">$B$8*C18*$B$9</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <f aca="false">$B$8*D18*$B$9</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <f aca="false">$B$8*E18*$B$9</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <f aca="false">$B$8*F18*$B$9</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <f aca="false">$B$8*G18*$B$9</f>
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="B27" s="6" t="n">
-        <f aca="false">B25*B26</f>
-        <v>122.142857142857</v>
+        <f aca="false">SUM(B22:B26)+$B$7</f>
+        <v>14.4</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <f aca="false">SUM(C22:C26)+$B$7</f>
+        <v>14.4</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <f aca="false">SUM(D22:D26)+$B$7</f>
+        <v>14.4</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <f aca="false">SUM(E22:E26)+$B$7</f>
+        <v>17.16</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <f aca="false">SUM(F22:F26)+$B$7</f>
+        <v>17.67</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <f aca="false">SUM(G22:G26)+$B$7</f>
+        <v>36.15</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="B28" s="6" t="n">
-        <f aca="false">$B$8*B26</f>
-        <v>214.285714285714</v>
+      <c r="A28" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="B28" s="45" t="n">
+        <f aca="false">$B$9*B19-B27</f>
+        <v>162.759271219808</v>
+      </c>
+      <c r="C28" s="45" t="n">
+        <f aca="false">$B$9*C19-C27</f>
+        <v>193.437559763159</v>
+      </c>
+      <c r="D28" s="45" t="n">
+        <f aca="false">$B$9*D19-D27</f>
+        <v>222.102631765115</v>
+      </c>
+      <c r="E28" s="45" t="n">
+        <f aca="false">$B$9*E19-E27</f>
+        <v>87.5896311689675</v>
+      </c>
+      <c r="F28" s="45" t="n">
+        <f aca="false">$B$9*F19-F27</f>
+        <v>54.0157127910397</v>
+      </c>
+      <c r="G28" s="45" t="n">
+        <f aca="false">$B$9*G19-G27</f>
+        <v>884.938945479572</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>474</v>
-      </c>
-      <c r="B29" s="6" t="n">
-        <f aca="false">G21*$B$12*$B$11</f>
-        <v>99.8851</v>
+      <c r="A29" s="8" t="s">
+        <v>480</v>
+      </c>
+      <c r="B29" s="27" t="n">
+        <f aca="false">Courier_Hub!B48</f>
+        <v>155.278911410284</v>
+      </c>
+      <c r="C29" s="27" t="n">
+        <f aca="false">Courier_Hub!C48</f>
+        <v>185.563999953635</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <f aca="false">Courier_Hub!D48</f>
+        <v>213.835871955591</v>
+      </c>
+      <c r="E29" s="27" t="n">
+        <f aca="false">Courier_Hub!E48</f>
+        <v>79.844224692777</v>
+      </c>
+      <c r="F29" s="27" t="n">
+        <f aca="false">Courier_Hub!F48</f>
+        <v>46.6826463148492</v>
+      </c>
+      <c r="G29" s="27" t="n">
+        <f aca="false">Courier_Hub!G48</f>
+        <v>855.454252336715</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>475</v>
-      </c>
-      <c r="B30" s="45" t="n">
-        <f aca="false">B27+B28+B29</f>
-        <v>436.313671428571</v>
+        <v>481</v>
+      </c>
+      <c r="B30" s="46" t="n">
+        <f aca="false">B28-B21</f>
+        <v>5.59999999999999</v>
+      </c>
+      <c r="C30" s="46" t="n">
+        <f aca="false">C28-C21</f>
+        <v>5.59999999999999</v>
+      </c>
+      <c r="D30" s="46" t="n">
+        <f aca="false">D28-D21</f>
+        <v>5.59999999999999</v>
+      </c>
+      <c r="E30" s="46" t="n">
+        <f aca="false">E28-E21</f>
+        <v>2.84</v>
+      </c>
+      <c r="F30" s="46" t="n">
+        <f aca="false">F28-F21</f>
+        <v>2.33</v>
+      </c>
+      <c r="G30" s="46" t="n">
+        <f aca="false">G28-G21</f>
+        <v>-16.15</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>476</v>
-      </c>
-      <c r="B31" s="14" t="n">
-        <f aca="false">B4*30</f>
-        <v>100</v>
+      <c r="A31" s="8" t="s">
+        <v>482</v>
+      </c>
+      <c r="B31" s="46" t="n">
+        <f aca="false">B28-B29</f>
+        <v>7.48035980952383</v>
+      </c>
+      <c r="C31" s="46" t="n">
+        <f aca="false">C28-C29</f>
+        <v>7.87355980952381</v>
+      </c>
+      <c r="D31" s="46" t="n">
+        <f aca="false">D28-D29</f>
+        <v>8.26675980952382</v>
+      </c>
+      <c r="E31" s="46" t="n">
+        <f aca="false">E28-E29</f>
+        <v>7.7454064761905</v>
+      </c>
+      <c r="F31" s="46" t="n">
+        <f aca="false">F28-F29</f>
+        <v>7.33306647619048</v>
+      </c>
+      <c r="G31" s="46" t="n">
+        <f aca="false">G28-G29</f>
+        <v>29.4846931428572</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="B32" s="6" t="n">
-        <f aca="false">Courier_Hub!B11*MAX(Courier_Hub!B25,B31)</f>
-        <v>825</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="s">
-        <v>478</v>
-      </c>
-      <c r="B33" s="48" t="n">
-        <f aca="false">(B30+B32)/B31</f>
-        <v>12.6131367142857</v>
+      <c r="A32" s="8" t="s">
+        <v>483</v>
+      </c>
+      <c r="B32" s="56" t="n">
+        <f aca="false">IF(B31&gt;0,B31/Courier_Hub!B47,0)</f>
+        <v>0.0323867274193482</v>
+      </c>
+      <c r="C32" s="56" t="n">
+        <f aca="false">IF(C31&gt;0,C31/Courier_Hub!C47,0)</f>
+        <v>0.0290723626161048</v>
+      </c>
+      <c r="D32" s="56" t="n">
+        <f aca="false">IF(D31&gt;0,D31/Courier_Hub!D47,0)</f>
+        <v>0.0268256608396796</v>
+      </c>
+      <c r="E32" s="56" t="n">
+        <f aca="false">IF(E31&gt;0,E31/Courier_Hub!E47,0)</f>
+        <v>0.0561081349807211</v>
+      </c>
+      <c r="F32" s="56" t="n">
+        <f aca="false">IF(F31&gt;0,F31/Courier_Hub!F47,0)</f>
+        <v>0.0772681158244974</v>
+      </c>
+      <c r="G32" s="56" t="n">
+        <f aca="false">IF(G31&gt;0,G31/Courier_Hub!G47,0)</f>
+        <v>0.0241435978526168</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>479</v>
-      </c>
-      <c r="B34" s="42" t="n">
-        <f aca="false">(Supuestos!B16*B31+Supuestos!B36)/B31</f>
-        <v>7.5</v>
-      </c>
+      <c r="A34" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>480</v>
-      </c>
-      <c r="B35" s="52" t="n">
-        <f aca="false">B33-B34</f>
-        <v>5.11313671428572</v>
+        <v>464</v>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>75</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>150</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="F35" s="15" t="n">
+        <v>600</v>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="B36" s="5" t="n">
+        <f aca="false">$C$30*B35</f>
+        <v>420</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <f aca="false">$C$30*C35</f>
+        <v>559.999999999999</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <f aca="false">$C$30*D35</f>
+        <v>839.999999999999</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <f aca="false">$C$30*E35</f>
+        <v>1680</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <f aca="false">$C$30*F35</f>
+        <v>3360</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <f aca="false">$C$30*G35</f>
+        <v>5599.99999999999</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2" t="s">
-        <v>481</v>
+      <c r="A37" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="B37" s="5" t="n">
+        <f aca="false">$C$31*B35</f>
+        <v>590.516985714286</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <f aca="false">$C$31*C35</f>
+        <v>787.355980952381</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <f aca="false">$C$31*D35</f>
+        <v>1181.03397142857</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <f aca="false">$C$31*E35</f>
+        <v>2362.06794285714</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <f aca="false">$C$31*F35</f>
+        <v>4724.13588571429</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <f aca="false">$C$31*G35</f>
+        <v>7873.55980952381</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>489</v>
       </c>
     </row>
   </sheetData>
@@ -4088,6 +4508,453 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="B4" s="53" t="n">
+        <f aca="false">Courier_Hub!B24/30</f>
+        <v>3.33333333333333</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="B5" s="39" t="n">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="B7" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="B9" s="59" t="n">
+        <f aca="false">Courier_Hub!B23</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="B10" s="17" t="n">
+        <f aca="false">Courier_Hub!B22</f>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="25" t="n">
+        <f aca="false">Supuestos!B5</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B12" s="58" t="n">
+        <f aca="false">Courier_Hub!B19</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>502</v>
+      </c>
+      <c r="C14" s="44" t="s">
+        <v>503</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>428</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>504</v>
+      </c>
+      <c r="F14" s="44" t="s">
+        <v>505</v>
+      </c>
+      <c r="G14" s="44" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B15</f>
+        <v>62</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <f aca="false">C15/D15</f>
+        <v>5.16666666666667</v>
+      </c>
+      <c r="F15" s="55" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="G15" s="60" t="n">
+        <f aca="false">C15*F15</f>
+        <v>0.4774</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B16</f>
+        <v>10.3333333333333</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <f aca="false">C16/D16</f>
+        <v>0.861111111111111</v>
+      </c>
+      <c r="F16" s="55" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="G16" s="60" t="n">
+        <f aca="false">C16*F16</f>
+        <v>0.0795666666666667</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B17</f>
+        <v>12.4</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <f aca="false">C17/D17</f>
+        <v>2.06666666666667</v>
+      </c>
+      <c r="F17" s="55" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="G17" s="60" t="n">
+        <f aca="false">C17*F17</f>
+        <v>0.30008</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B18</f>
+        <v>10.3333333333333</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <f aca="false">C18/D18</f>
+        <v>1.72222222222222</v>
+      </c>
+      <c r="F18" s="55" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="G18" s="60" t="n">
+        <f aca="false">C18*F18</f>
+        <v>0.267633333333333</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B19</f>
+        <v>3.1</v>
+      </c>
+      <c r="D19" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <f aca="false">C19/D19</f>
+        <v>3.1</v>
+      </c>
+      <c r="F19" s="55" t="n">
+        <v>0.0875</v>
+      </c>
+      <c r="G19" s="60" t="n">
+        <f aca="false">C19*F19</f>
+        <v>0.27125</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <f aca="false">$B$4*($B$5+$B$6)*B20</f>
+        <v>5.16666666666667</v>
+      </c>
+      <c r="D20" s="20" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <f aca="false">C20/D20</f>
+        <v>0.449275362318841</v>
+      </c>
+      <c r="F20" s="55" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="G20" s="60" t="n">
+        <f aca="false">C20*F20</f>
+        <v>0.031</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="56" t="n">
+        <f aca="false">SUM(B15:B20)</f>
+        <v>1</v>
+      </c>
+      <c r="C21" s="61" t="n">
+        <f aca="false">SUM(C15:C20)</f>
+        <v>103.333333333333</v>
+      </c>
+      <c r="E21" s="61" t="n">
+        <f aca="false">SUM(E15:E20)</f>
+        <v>13.3659420289855</v>
+      </c>
+      <c r="G21" s="62" t="n">
+        <f aca="false">SUM(G15:G20)</f>
+        <v>1.42693</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>509</v>
+      </c>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <f aca="false">MAX($B$7,E21/$B$9)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="B25" s="6" t="n">
+        <f aca="false">B24*$B$10</f>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <f aca="false">30/$B$5</f>
+        <v>1.07142857142857</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <f aca="false">B25*B26</f>
+        <v>122.142857142857</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <f aca="false">$B$8*B26</f>
+        <v>214.285714285714</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="B29" s="6" t="n">
+        <f aca="false">G21*$B$12*$B$11</f>
+        <v>99.8851</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>516</v>
+      </c>
+      <c r="B30" s="45" t="n">
+        <f aca="false">B27+B28+B29</f>
+        <v>436.313671428571</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="B31" s="14" t="n">
+        <f aca="false">B4*30</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="B32" s="6" t="n">
+        <f aca="false">Courier_Hub!B11*MAX(Courier_Hub!B25,B31)</f>
+        <v>825</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
+        <v>519</v>
+      </c>
+      <c r="B33" s="48" t="n">
+        <f aca="false">(B30+B32)/B31</f>
+        <v>12.6131367142857</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="B34" s="42" t="n">
+        <f aca="false">(Supuestos!B16*B31+Supuestos!B36)/B31</f>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="B35" s="52" t="n">
+        <f aca="false">B33-B34</f>
+        <v>5.11313671428572</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>522</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4097,12 +4964,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>482</v>
+        <v>523</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>483</v>
+        <v>524</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4121,7 +4988,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>484</v>
+        <v>525</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>1008</v>
@@ -4136,7 +5003,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>485</v>
+        <v>526</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>1000</v>
@@ -4151,7 +5018,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>486</v>
+        <v>527</v>
       </c>
       <c r="B7" s="15" t="n">
         <v>500</v>
@@ -4166,7 +5033,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>487</v>
+        <v>528</v>
       </c>
       <c r="B8" s="15" t="n">
         <v>5</v>
@@ -4181,7 +5048,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>488</v>
+        <v>529</v>
       </c>
       <c r="B9" s="15" t="n">
         <v>1</v>
@@ -4196,7 +5063,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>489</v>
+        <v>530</v>
       </c>
       <c r="D10" s="48" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -4205,17 +5072,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>490</v>
+        <v>531</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>491</v>
+        <v>532</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>492</v>
+        <v>533</v>
       </c>
       <c r="B14" s="38" t="n">
         <v>1135.87</v>
@@ -4223,7 +5090,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>493</v>
+        <v>534</v>
       </c>
       <c r="B15" s="38" t="n">
         <v>135.13</v>
@@ -4231,7 +5098,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>494</v>
+        <v>535</v>
       </c>
       <c r="B16" s="38" t="n">
         <v>1720</v>
@@ -4239,7 +5106,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>495</v>
+        <v>536</v>
       </c>
       <c r="B17" s="38" t="n">
         <v>309.6</v>
@@ -4247,7 +5114,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>496</v>
+        <v>537</v>
       </c>
       <c r="B18" s="38" t="n">
         <v>5961</v>
@@ -4255,7 +5122,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>497</v>
+        <v>538</v>
       </c>
       <c r="B19" s="39" t="n">
         <v>1</v>
@@ -4272,7 +5139,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>498</v>
+        <v>539</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4282,7 +5149,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>499</v>
+        <v>540</v>
       </c>
       <c r="B24" s="42" t="n">
         <f aca="false">D10*B20</f>
@@ -4291,7 +5158,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>500</v>
+        <v>541</v>
       </c>
       <c r="B25" s="42" t="n">
         <f aca="false">B14*B20</f>
@@ -4300,7 +5167,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>501</v>
+        <v>542</v>
       </c>
       <c r="B26" s="42" t="n">
         <f aca="false">B16+B17</f>
@@ -4318,7 +5185,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>502</v>
+        <v>543</v>
       </c>
       <c r="B28" s="48" t="n">
         <f aca="false">SUM(B24:B27)</f>
@@ -4327,7 +5194,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>503</v>
+        <v>544</v>
       </c>
       <c r="B29" s="42" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -4354,7 +5221,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>504</v>
+        <v>545</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4362,24 +5229,24 @@
         <v>18</v>
       </c>
       <c r="B34" s="44" t="s">
-        <v>505</v>
+        <v>546</v>
       </c>
       <c r="C34" s="44" t="s">
-        <v>506</v>
+        <v>547</v>
       </c>
       <c r="D34" s="44" t="s">
-        <v>507</v>
+        <v>548</v>
       </c>
       <c r="E34" s="44" t="s">
         <v>296</v>
       </c>
       <c r="F34" s="44" t="s">
-        <v>508</v>
+        <v>549</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>509</v>
+        <v>550</v>
       </c>
       <c r="B35" s="42" t="n">
         <f aca="false">D5</f>
@@ -4404,7 +5271,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>510</v>
+        <v>551</v>
       </c>
       <c r="B36" s="42" t="n">
         <f aca="false">D6</f>
@@ -4429,7 +5296,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>511</v>
+        <v>552</v>
       </c>
       <c r="B37" s="42" t="n">
         <f aca="false">D7</f>
@@ -4471,7 +5338,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>512</v>
+        <v>553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Courier_Dinsides: tarifa premium por distrito, sin cobro por rechazados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Buo77uofKMf1g7UXANtFhU
</commit_message>
<xml_diff>
--- a/analisis/elvo-margen-por-producto.xlsx
+++ b/analisis/elvo-margen-por-producto.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="560">
   <si>
     <t xml:space="preserve">Plan hacia US$ 1M de utilidad anual - resumen de escenarios</t>
   </si>
@@ -1381,25 +1381,40 @@
     <t xml:space="preserve">No incluye: beneficio tributario de la factura de The Hub (IGV y gasto deducible) (el transporte desde tu almacen a The Hub viene de la hoja Stock_Hub). Para bidones y Cero el courier actual (S/ 12.5) es solo una referencia.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dinsides (almacen + despacho) vs operacion actual vs The Hub - Lima, contraentrega</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente: brochure de fulfillment de Dinsides. El brochure NO trae tarifas de envio ni cobro por contraentrega: se usa el courier actual de S/ 10-15. Azul/amarillo = supuesto o dato pendiente.</t>
+    <t xml:space="preserve">Dinsides (almacen + despacho, tarifa premium) vs operacion actual vs The Hub - Lima, contraentrega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuentes: brochure de fulfillment y tarifa premium de Dinsides (validez de los beneficios: hasta el 31-oct-2026). Todas sus tarifas incluyen IGV. Azul/amarillo = supuesto o dato pendiente.</t>
   </si>
   <si>
     <t xml:space="preserve">Condiciones de Dinsides</t>
   </si>
   <si>
-    <t xml:space="preserve">Courier Lima por pedido (S/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dinsides al dia siguiente: S/ 10-15 (dato del usuario).</t>
+    <t xml:space="preserve">Tarifa premium de Lima, ponderada (S/ con IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarifa por distrito: S/ 10 urbano, S/ 12 periferico, S/ 14-28 lejanos. 11.5 = promedio ESTIMADO con una muestra de 14 pedidos de Lima (11.57).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Dinsides emite factura con IGV? (1 = si, 0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDIENTE de confirmar. Con 1, el IGV de la tarifa es recuperable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarifa neta por pedido (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Se cobra el envio en pedidos rechazados o no entregados? (1 = si, 0 = no)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarifa premium: sin cobros por rechazados, espera ni devoluciones. Beneficios hasta el 31-oct: pedir que queden por escrito.</t>
   </si>
   <si>
     <t xml:space="preserve">Material de empaque por pedido (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPUESTO: Dinsides exige que el cliente provea bolsas, cajas y film.</t>
+    <t xml:space="preserve">SUPUESTO: Dinsides exige que el cliente provea bolsas, cajas y film (se pueden reutilizar paquetes sin costo).</t>
   </si>
   <si>
     <t xml:space="preserve">Costo por pedido armado y no entregado (S/)</t>
@@ -1417,7 +1432,7 @@
     <t xml:space="preserve">Cobro contraentrega de Dinsides (% del valor)</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: el brochure no lo menciona. Confirmar efectivo, POS y cuotas.</t>
+    <t xml:space="preserve">PENDIENTE: no figura en ningun documento. Confirmar efectivo, POS y cuotas.</t>
   </si>
   <si>
     <t xml:space="preserve">Entrega efectiva con Dinsides</t>
@@ -1447,13 +1462,16 @@
     <t xml:space="preserve">Penalidad por pedido (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPUESTO: igual que The Hub, por falta de tarifa de Dinsides para bultos grandes.</t>
+    <t xml:space="preserve">Kg adicional sobre 3 kg (S/ con IGV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTO: Dinsides cobra tarifa variable por tamaño y peso; se usa la de The Hub como referencia.</t>
   </si>
   <si>
     <t xml:space="preserve">ACTUAL (Tecretail + courier): utilidad antes de publicidad</t>
   </si>
   <si>
-    <t xml:space="preserve">DINSIDES: courier</t>
+    <t xml:space="preserve">DINSIDES: envio (segun entregados y rechazados)</t>
   </si>
   <si>
     <t xml:space="preserve">DINSIDES: material de empaque</t>
@@ -1495,13 +1513,13 @@
     <t xml:space="preserve">Dinsides vs The Hub (S/ al mes)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lectura: el brochure incluye almacen, armado, rotulado, seguro por robo y perdida, control de inventario 3 veces por semana y punto de recojo en su almacen. No incluye materiales de empaque.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El ahorro es de costo, no de entrega efectiva: si Dinsides entrega igual que hoy (80%), el ahorro es el de la fila 30. Por eso pedir su tasa de entrega por distrito antes de decidir.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En el brochure los S/ 2.00 por pedido armado y no entregado reemplazan al costo de gestion; no hay cobro por almacenaje. Confirmar si ese cobro de S/ 2.00 es adicional al reintento o a la devolucion.</t>
+    <t xml:space="preserve">Cobro contraentrega que iguala a la operacion actual (% del valor, Nativo 3 años)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarifa premium por zona (S/ con IGV): envio a agencias de Breña 5; retiro en Breña 8; urbano 10 (Surco, Miraflores, San Borja, Cercado, La Molina, Santa Anita, SJL y otros); 12 (Ate, Callao, Comas, Los Olivos, Puente Piedra, SJM, VES, VMT, SMP, Independencia y otros); 14 (Lurin, Huachipa, Chosica); 17 (Ancon, Cieneguilla, Chaclacayo, Manchay); 19 Pachacamac; 21-28 lejanos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beneficios hasta el 31-oct: sin cobros por espera ni rechazados, paquetes reutilizables sin costo, devoluciones y retorno sin costo (previa validacion). Pedir que se mantengan por escrito mas alla del 31-oct. El brochure no incluye cobro por contraentrega ni tarifas de bultos grandes.</t>
   </si>
   <si>
     <t xml:space="preserve">Plan de stock en The Hub: tandas desde tu almacen propio</t>
@@ -3769,10 +3787,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="17"/>
   </cols>
   <sheetData>
@@ -3797,9 +3815,8 @@
       <c r="A4" s="4" t="s">
         <v>452</v>
       </c>
-      <c r="B4" s="17" t="n">
-        <f aca="false">Supuestos!B18</f>
-        <v>12.5</v>
+      <c r="B4" s="23" t="n">
+        <v>11.5</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>453</v>
@@ -3809,8 +3826,8 @@
       <c r="A5" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="B5" s="23" t="n">
-        <v>1.5</v>
+      <c r="B5" s="39" t="n">
+        <v>0</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>455</v>
@@ -3820,676 +3837,712 @@
       <c r="A6" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="B6" s="38" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>457</v>
-      </c>
+      <c r="B6" s="42" t="n">
+        <f aca="false">B4/(1+Supuestos!B4*B5)</f>
+        <v>11.5</v>
+      </c>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="B7" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>458</v>
-      </c>
-      <c r="B7" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>460</v>
-      </c>
-      <c r="B8" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="B9" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>462</v>
-      </c>
-      <c r="B9" s="36" t="n">
-        <f aca="false">Supuestos!B7</f>
-        <v>0.8</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B10" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>464</v>
-      </c>
-      <c r="B10" s="35" t="n">
-        <f aca="false">Courier_Hub!B24</f>
-        <v>100</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="B11" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="B11" s="7" t="n">
-        <f aca="false">B10/4.33</f>
-        <v>23.094688221709</v>
-      </c>
-      <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="B12" s="24" t="n">
-        <v>15</v>
+      <c r="B12" s="36" t="n">
+        <f aca="false">Supuestos!B7</f>
+        <v>0.8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>457</v>
+        <v>468</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="B13" s="38" t="n">
-        <v>2</v>
+        <v>469</v>
+      </c>
+      <c r="B13" s="35" t="n">
+        <f aca="false">Courier_Hub!B24</f>
+        <v>100</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>470</v>
-      </c>
-      <c r="B14" s="42" t="n">
-        <f aca="false">IF(B11&lt;B12,B13*30,0)/B10</f>
-        <v>0</v>
+        <v>471</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <f aca="false">B13/4.33</f>
+        <v>23.094688221709</v>
       </c>
       <c r="C14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>394</v>
-      </c>
-      <c r="B15" s="57" t="n">
+        <v>472</v>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="B16" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="B17" s="42" t="n">
+        <f aca="false">IF(B14&lt;B15,B16*30,0)/B13</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="B18" s="57" t="n">
         <f aca="false">Courier_Hub!B13</f>
         <v>1.5</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="44" t="s">
+      <c r="C18" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="44" t="s">
         <v>308</v>
       </c>
-      <c r="B17" s="44" t="s">
+      <c r="B20" s="44" t="s">
         <v>259</v>
       </c>
-      <c r="C17" s="44" t="s">
+      <c r="C20" s="44" t="s">
         <v>260</v>
       </c>
-      <c r="D17" s="44" t="s">
+      <c r="D20" s="44" t="s">
         <v>261</v>
       </c>
-      <c r="E17" s="44" t="s">
+      <c r="E20" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="F17" s="44" t="s">
+      <c r="F20" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="G17" s="44" t="s">
+      <c r="G20" s="44" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="B18" s="35" t="n">
+      <c r="B21" s="35" t="n">
         <f aca="false">Courier_Hub!B32</f>
         <v>299</v>
       </c>
-      <c r="C18" s="35" t="n">
+      <c r="C21" s="35" t="n">
         <f aca="false">Courier_Hub!C32</f>
         <v>349</v>
       </c>
-      <c r="D18" s="35" t="n">
+      <c r="D21" s="35" t="n">
         <f aca="false">Courier_Hub!D32</f>
         <v>399</v>
       </c>
-      <c r="E18" s="35" t="n">
+      <c r="E21" s="35" t="n">
         <f aca="false">Courier_Hub!E32</f>
         <v>219</v>
       </c>
-      <c r="F18" s="35" t="n">
+      <c r="F21" s="35" t="n">
         <f aca="false">Courier_Hub!F32</f>
         <v>159</v>
       </c>
-      <c r="G18" s="35" t="n">
+      <c r="G21" s="35" t="n">
         <f aca="false">Courier_Hub!G32</f>
         <v>2299</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="B19" s="27" t="n">
+      <c r="B22" s="27" t="n">
         <f aca="false">Courier_Hub!B33</f>
         <v>221.44908902476</v>
       </c>
-      <c r="C19" s="27" t="n">
+      <c r="C22" s="27" t="n">
         <f aca="false">Courier_Hub!C33</f>
         <v>259.796949703949</v>
       </c>
-      <c r="D19" s="27" t="n">
+      <c r="D22" s="27" t="n">
         <f aca="false">Courier_Hub!D33</f>
         <v>295.628289706394</v>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E22" s="27" t="n">
         <f aca="false">Courier_Hub!E33</f>
         <v>130.937038961209</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F22" s="27" t="n">
         <f aca="false">Courier_Hub!F33</f>
         <v>89.6071409887996</v>
       </c>
-      <c r="G19" s="27" t="n">
+      <c r="G22" s="27" t="n">
         <f aca="false">Courier_Hub!G33</f>
         <v>1151.36118184947</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>427</v>
       </c>
-      <c r="B20" s="58" t="n">
+      <c r="B23" s="58" t="n">
         <f aca="false">Courier_Hub!B36</f>
         <v>1.5</v>
       </c>
-      <c r="C20" s="58" t="n">
+      <c r="C23" s="58" t="n">
         <f aca="false">Courier_Hub!C36</f>
         <v>1.5</v>
       </c>
-      <c r="D20" s="58" t="n">
+      <c r="D23" s="58" t="n">
         <f aca="false">Courier_Hub!D36</f>
         <v>2</v>
       </c>
-      <c r="E20" s="58" t="n">
+      <c r="E23" s="58" t="n">
         <f aca="false">Courier_Hub!E36</f>
         <v>4.84</v>
       </c>
-      <c r="F20" s="58" t="n">
+      <c r="F23" s="58" t="n">
         <f aca="false">Courier_Hub!F36</f>
         <v>5.18</v>
       </c>
-      <c r="G20" s="58" t="n">
+      <c r="G23" s="58" t="n">
         <f aca="false">Courier_Hub!G36</f>
         <v>17.5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
-        <v>472</v>
-      </c>
-      <c r="B21" s="27" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>478</v>
+      </c>
+      <c r="B24" s="27" t="n">
         <f aca="false">Courier_Hub!B39</f>
         <v>157.159271219808</v>
       </c>
-      <c r="C21" s="27" t="n">
+      <c r="C24" s="27" t="n">
         <f aca="false">Courier_Hub!C39</f>
         <v>187.837559763159</v>
       </c>
-      <c r="D21" s="27" t="n">
+      <c r="D24" s="27" t="n">
         <f aca="false">Courier_Hub!D39</f>
         <v>216.502631765115</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E24" s="27" t="n">
         <f aca="false">Courier_Hub!E39</f>
         <v>84.7496311689675</v>
       </c>
-      <c r="F21" s="27" t="n">
+      <c r="F24" s="27" t="n">
         <f aca="false">Courier_Hub!F39</f>
         <v>51.6857127910397</v>
       </c>
-      <c r="G21" s="27" t="n">
+      <c r="G24" s="27" t="n">
         <f aca="false">Courier_Hub!G39</f>
         <v>901.088945479572</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="B22" s="6" t="n">
-        <f aca="false">$B$4+MAX(0,B20-3)*$B$15</f>
-        <v>12.5</v>
-      </c>
-      <c r="C22" s="6" t="n">
-        <f aca="false">$B$4+MAX(0,C20-3)*$B$15</f>
-        <v>12.5</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <f aca="false">$B$4+MAX(0,D20-3)*$B$15</f>
-        <v>12.5</v>
-      </c>
-      <c r="E22" s="6" t="n">
-        <f aca="false">$B$4+MAX(0,E20-3)*$B$15</f>
-        <v>15.26</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <f aca="false">$B$4+MAX(0,F20-3)*$B$15</f>
-        <v>15.77</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <f aca="false">$B$4+MAX(0,G20-3)*$B$15</f>
-        <v>34.25</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>474</v>
-      </c>
-      <c r="B23" s="6" t="n">
-        <f aca="false">$B$5</f>
-        <v>1.5</v>
-      </c>
-      <c r="C23" s="6" t="n">
-        <f aca="false">$B$5</f>
-        <v>1.5</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <f aca="false">$B$5</f>
-        <v>1.5</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <f aca="false">$B$5</f>
-        <v>1.5</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <f aca="false">$B$5</f>
-        <v>1.5</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <f aca="false">$B$5</f>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>475</v>
-      </c>
-      <c r="B24" s="6" t="n">
-        <f aca="false">(1-$B$9)*$B$6</f>
-        <v>0.4</v>
-      </c>
-      <c r="C24" s="6" t="n">
-        <f aca="false">(1-$B$9)*$B$6</f>
-        <v>0.4</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <f aca="false">(1-$B$9)*$B$6</f>
-        <v>0.4</v>
-      </c>
-      <c r="E24" s="6" t="n">
-        <f aca="false">(1-$B$9)*$B$6</f>
-        <v>0.4</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <f aca="false">(1-$B$9)*$B$6</f>
-        <v>0.4</v>
-      </c>
-      <c r="G24" s="6" t="n">
-        <f aca="false">(1-$B$9)*$B$6</f>
-        <v>0.4</v>
-      </c>
-    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B25" s="6" t="n">
-        <f aca="false">$B$14</f>
-        <v>0</v>
+        <f aca="false">($B$6+MAX(0,B23-3)*$B$18/(1+Supuestos!$B$4*$B$5))*($B$12+(1-$B$12)*$B$7)</f>
+        <v>9.2</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">$B$14</f>
-        <v>0</v>
+        <f aca="false">($B$6+MAX(0,C23-3)*$B$18/(1+Supuestos!$B$4*$B$5))*($B$12+(1-$B$12)*$B$7)</f>
+        <v>9.2</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">$B$14</f>
-        <v>0</v>
+        <f aca="false">($B$6+MAX(0,D23-3)*$B$18/(1+Supuestos!$B$4*$B$5))*($B$12+(1-$B$12)*$B$7)</f>
+        <v>9.2</v>
       </c>
       <c r="E25" s="6" t="n">
-        <f aca="false">$B$14</f>
-        <v>0</v>
+        <f aca="false">($B$6+MAX(0,E23-3)*$B$18/(1+Supuestos!$B$4*$B$5))*($B$12+(1-$B$12)*$B$7)</f>
+        <v>11.408</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">$B$14</f>
-        <v>0</v>
+        <f aca="false">($B$6+MAX(0,F23-3)*$B$18/(1+Supuestos!$B$4*$B$5))*($B$12+(1-$B$12)*$B$7)</f>
+        <v>11.816</v>
       </c>
       <c r="G25" s="6" t="n">
-        <f aca="false">$B$14</f>
-        <v>0</v>
+        <f aca="false">($B$6+MAX(0,G23-3)*$B$18/(1+Supuestos!$B$4*$B$5))*($B$12+(1-$B$12)*$B$7)</f>
+        <v>26.6</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B26" s="6" t="n">
-        <f aca="false">$B$8*B18*$B$9</f>
-        <v>0</v>
+        <f aca="false">$B$8</f>
+        <v>1.5</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">$B$8*C18*$B$9</f>
-        <v>0</v>
+        <f aca="false">$B$8</f>
+        <v>1.5</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">$B$8*D18*$B$9</f>
-        <v>0</v>
+        <f aca="false">$B$8</f>
+        <v>1.5</v>
       </c>
       <c r="E26" s="6" t="n">
-        <f aca="false">$B$8*E18*$B$9</f>
-        <v>0</v>
+        <f aca="false">$B$8</f>
+        <v>1.5</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">$B$8*F18*$B$9</f>
-        <v>0</v>
+        <f aca="false">$B$8</f>
+        <v>1.5</v>
       </c>
       <c r="G26" s="6" t="n">
-        <f aca="false">$B$8*G18*$B$9</f>
-        <v>0</v>
+        <f aca="false">$B$8</f>
+        <v>1.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="B27" s="6" t="n">
-        <f aca="false">SUM(B22:B26)+$B$7</f>
-        <v>14.4</v>
+        <f aca="false">(1-$B$12)*$B$9</f>
+        <v>0.4</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">SUM(C22:C26)+$B$7</f>
-        <v>14.4</v>
+        <f aca="false">(1-$B$12)*$B$9</f>
+        <v>0.4</v>
       </c>
       <c r="D27" s="6" t="n">
-        <f aca="false">SUM(D22:D26)+$B$7</f>
-        <v>14.4</v>
+        <f aca="false">(1-$B$12)*$B$9</f>
+        <v>0.4</v>
       </c>
       <c r="E27" s="6" t="n">
-        <f aca="false">SUM(E22:E26)+$B$7</f>
-        <v>17.16</v>
+        <f aca="false">(1-$B$12)*$B$9</f>
+        <v>0.4</v>
       </c>
       <c r="F27" s="6" t="n">
-        <f aca="false">SUM(F22:F26)+$B$7</f>
-        <v>17.67</v>
+        <f aca="false">(1-$B$12)*$B$9</f>
+        <v>0.4</v>
       </c>
       <c r="G27" s="6" t="n">
-        <f aca="false">SUM(G22:G26)+$B$7</f>
-        <v>36.15</v>
+        <f aca="false">(1-$B$12)*$B$9</f>
+        <v>0.4</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>479</v>
-      </c>
-      <c r="B28" s="45" t="n">
-        <f aca="false">$B$9*B19-B27</f>
-        <v>162.759271219808</v>
-      </c>
-      <c r="C28" s="45" t="n">
-        <f aca="false">$B$9*C19-C27</f>
-        <v>193.437559763159</v>
-      </c>
-      <c r="D28" s="45" t="n">
-        <f aca="false">$B$9*D19-D27</f>
-        <v>222.102631765115</v>
-      </c>
-      <c r="E28" s="45" t="n">
-        <f aca="false">$B$9*E19-E27</f>
-        <v>87.5896311689675</v>
-      </c>
-      <c r="F28" s="45" t="n">
-        <f aca="false">$B$9*F19-F27</f>
-        <v>54.0157127910397</v>
-      </c>
-      <c r="G28" s="45" t="n">
-        <f aca="false">$B$9*G19-G27</f>
-        <v>884.938945479572</v>
+      <c r="A28" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <f aca="false">$B$17</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <f aca="false">$B$17</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <f aca="false">$B$17</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <f aca="false">$B$17</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <f aca="false">$B$17</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <f aca="false">$B$17</f>
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="s">
-        <v>480</v>
-      </c>
-      <c r="B29" s="27" t="n">
+      <c r="A29" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="B29" s="6" t="n">
+        <f aca="false">$B$11*B21*$B$12</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <f aca="false">$B$11*C21*$B$12</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <f aca="false">$B$11*D21*$B$12</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <f aca="false">$B$11*E21*$B$12</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <f aca="false">$B$11*F21*$B$12</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <f aca="false">$B$11*G21*$B$12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="B30" s="6" t="n">
+        <f aca="false">SUM(B25:B29)+$B$10</f>
+        <v>11.1</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <f aca="false">SUM(C25:C29)+$B$10</f>
+        <v>11.1</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <f aca="false">SUM(D25:D29)+$B$10</f>
+        <v>11.1</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <f aca="false">SUM(E25:E29)+$B$10</f>
+        <v>13.308</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <f aca="false">SUM(F25:F29)+$B$10</f>
+        <v>13.716</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <f aca="false">SUM(G25:G29)+$B$10</f>
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
+        <v>485</v>
+      </c>
+      <c r="B31" s="45" t="n">
+        <f aca="false">$B$12*B22-B30</f>
+        <v>166.059271219808</v>
+      </c>
+      <c r="C31" s="45" t="n">
+        <f aca="false">$B$12*C22-C30</f>
+        <v>196.737559763159</v>
+      </c>
+      <c r="D31" s="45" t="n">
+        <f aca="false">$B$12*D22-D30</f>
+        <v>225.402631765115</v>
+      </c>
+      <c r="E31" s="45" t="n">
+        <f aca="false">$B$12*E22-E30</f>
+        <v>91.4416311689675</v>
+      </c>
+      <c r="F31" s="45" t="n">
+        <f aca="false">$B$12*F22-F30</f>
+        <v>57.9697127910397</v>
+      </c>
+      <c r="G31" s="45" t="n">
+        <f aca="false">$B$12*G22-G30</f>
+        <v>892.588945479572</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
+        <v>486</v>
+      </c>
+      <c r="B32" s="27" t="n">
         <f aca="false">Courier_Hub!B48</f>
         <v>155.278911410284</v>
       </c>
-      <c r="C29" s="27" t="n">
+      <c r="C32" s="27" t="n">
         <f aca="false">Courier_Hub!C48</f>
         <v>185.563999953635</v>
       </c>
-      <c r="D29" s="27" t="n">
+      <c r="D32" s="27" t="n">
         <f aca="false">Courier_Hub!D48</f>
         <v>213.835871955591</v>
       </c>
-      <c r="E29" s="27" t="n">
+      <c r="E32" s="27" t="n">
         <f aca="false">Courier_Hub!E48</f>
         <v>79.844224692777</v>
       </c>
-      <c r="F29" s="27" t="n">
+      <c r="F32" s="27" t="n">
         <f aca="false">Courier_Hub!F48</f>
         <v>46.6826463148492</v>
       </c>
-      <c r="G29" s="27" t="n">
+      <c r="G32" s="27" t="n">
         <f aca="false">Courier_Hub!G48</f>
         <v>855.454252336715</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="s">
-        <v>481</v>
-      </c>
-      <c r="B30" s="46" t="n">
-        <f aca="false">B28-B21</f>
-        <v>5.59999999999999</v>
-      </c>
-      <c r="C30" s="46" t="n">
-        <f aca="false">C28-C21</f>
-        <v>5.59999999999999</v>
-      </c>
-      <c r="D30" s="46" t="n">
-        <f aca="false">D28-D21</f>
-        <v>5.59999999999999</v>
-      </c>
-      <c r="E30" s="46" t="n">
-        <f aca="false">E28-E21</f>
-        <v>2.84</v>
-      </c>
-      <c r="F30" s="46" t="n">
-        <f aca="false">F28-F21</f>
-        <v>2.33</v>
-      </c>
-      <c r="G30" s="46" t="n">
-        <f aca="false">G28-G21</f>
-        <v>-16.15</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="s">
-        <v>482</v>
-      </c>
-      <c r="B31" s="46" t="n">
-        <f aca="false">B28-B29</f>
-        <v>7.48035980952383</v>
-      </c>
-      <c r="C31" s="46" t="n">
-        <f aca="false">C28-C29</f>
-        <v>7.87355980952381</v>
-      </c>
-      <c r="D31" s="46" t="n">
-        <f aca="false">D28-D29</f>
-        <v>8.26675980952382</v>
-      </c>
-      <c r="E31" s="46" t="n">
-        <f aca="false">E28-E29</f>
-        <v>7.7454064761905</v>
-      </c>
-      <c r="F31" s="46" t="n">
-        <f aca="false">F28-F29</f>
-        <v>7.33306647619048</v>
-      </c>
-      <c r="G31" s="46" t="n">
-        <f aca="false">G28-G29</f>
-        <v>29.4846931428572</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="s">
-        <v>483</v>
-      </c>
-      <c r="B32" s="56" t="n">
-        <f aca="false">IF(B31&gt;0,B31/Courier_Hub!B47,0)</f>
-        <v>0.0323867274193482</v>
-      </c>
-      <c r="C32" s="56" t="n">
-        <f aca="false">IF(C31&gt;0,C31/Courier_Hub!C47,0)</f>
-        <v>0.0290723626161048</v>
-      </c>
-      <c r="D32" s="56" t="n">
-        <f aca="false">IF(D31&gt;0,D31/Courier_Hub!D47,0)</f>
-        <v>0.0268256608396796</v>
-      </c>
-      <c r="E32" s="56" t="n">
-        <f aca="false">IF(E31&gt;0,E31/Courier_Hub!E47,0)</f>
-        <v>0.0561081349807211</v>
-      </c>
-      <c r="F32" s="56" t="n">
-        <f aca="false">IF(F31&gt;0,F31/Courier_Hub!F47,0)</f>
-        <v>0.0772681158244974</v>
-      </c>
-      <c r="G32" s="56" t="n">
-        <f aca="false">IF(G31&gt;0,G31/Courier_Hub!G47,0)</f>
-        <v>0.0241435978526168</v>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
+        <v>487</v>
+      </c>
+      <c r="B33" s="46" t="n">
+        <f aca="false">B31-B24</f>
+        <v>8.90000000000001</v>
+      </c>
+      <c r="C33" s="46" t="n">
+        <f aca="false">C31-C24</f>
+        <v>8.90000000000001</v>
+      </c>
+      <c r="D33" s="46" t="n">
+        <f aca="false">D31-D24</f>
+        <v>8.90000000000001</v>
+      </c>
+      <c r="E33" s="46" t="n">
+        <f aca="false">E31-E24</f>
+        <v>6.69199999999999</v>
+      </c>
+      <c r="F33" s="46" t="n">
+        <f aca="false">F31-F24</f>
+        <v>6.284</v>
+      </c>
+      <c r="G33" s="46" t="n">
+        <f aca="false">G31-G24</f>
+        <v>-8.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="s">
-        <v>484</v>
-      </c>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
+      <c r="A34" s="8" t="s">
+        <v>488</v>
+      </c>
+      <c r="B34" s="46" t="n">
+        <f aca="false">B31-B32</f>
+        <v>10.7803598095238</v>
+      </c>
+      <c r="C34" s="46" t="n">
+        <f aca="false">C31-C32</f>
+        <v>11.1735598095238</v>
+      </c>
+      <c r="D34" s="46" t="n">
+        <f aca="false">D31-D32</f>
+        <v>11.5667598095238</v>
+      </c>
+      <c r="E34" s="46" t="n">
+        <f aca="false">E31-E32</f>
+        <v>11.5974064761905</v>
+      </c>
+      <c r="F34" s="46" t="n">
+        <f aca="false">F31-F32</f>
+        <v>11.2870664761905</v>
+      </c>
+      <c r="G34" s="46" t="n">
+        <f aca="false">G31-G32</f>
+        <v>37.1346931428571</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>464</v>
-      </c>
-      <c r="B35" s="15" t="n">
+        <v>489</v>
+      </c>
+      <c r="B35" s="56" t="n">
+        <f aca="false">IF(B34&gt;0,B34/Courier_Hub!B47,0)</f>
+        <v>0.0466743022426578</v>
+      </c>
+      <c r="C35" s="56" t="n">
+        <f aca="false">IF(C34&gt;0,C34/Courier_Hub!C47,0)</f>
+        <v>0.0412572953471801</v>
+      </c>
+      <c r="D35" s="56" t="n">
+        <f aca="false">IF(D34&gt;0,D34/Courier_Hub!D47,0)</f>
+        <v>0.0375341709223068</v>
+      </c>
+      <c r="E35" s="56" t="n">
+        <f aca="false">IF(E34&gt;0,E34/Courier_Hub!E47,0)</f>
+        <v>0.0840122271171531</v>
+      </c>
+      <c r="F35" s="56" t="n">
+        <f aca="false">IF(F34&gt;0,F34/Courier_Hub!F47,0)</f>
+        <v>0.118931195105456</v>
+      </c>
+      <c r="G35" s="56" t="n">
+        <f aca="false">IF(G34&gt;0,G34/Courier_Hub!G47,0)</f>
+        <v>0.0304078151085886</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="B38" s="15" t="n">
         <v>75</v>
       </c>
-      <c r="C35" s="15" t="n">
+      <c r="C38" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="D35" s="15" t="n">
+      <c r="D38" s="15" t="n">
         <v>150</v>
       </c>
-      <c r="E35" s="15" t="n">
+      <c r="E38" s="15" t="n">
         <v>300</v>
       </c>
-      <c r="F35" s="15" t="n">
+      <c r="F38" s="15" t="n">
         <v>600</v>
       </c>
-      <c r="G35" s="15" t="n">
+      <c r="G38" s="15" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>485</v>
-      </c>
-      <c r="B36" s="5" t="n">
-        <f aca="false">$C$30*B35</f>
-        <v>420</v>
-      </c>
-      <c r="C36" s="5" t="n">
-        <f aca="false">$C$30*C35</f>
-        <v>559.999999999999</v>
-      </c>
-      <c r="D36" s="5" t="n">
-        <f aca="false">$C$30*D35</f>
-        <v>839.999999999999</v>
-      </c>
-      <c r="E36" s="5" t="n">
-        <f aca="false">$C$30*E35</f>
-        <v>1680</v>
-      </c>
-      <c r="F36" s="5" t="n">
-        <f aca="false">$C$30*F35</f>
-        <v>3360</v>
-      </c>
-      <c r="G36" s="5" t="n">
-        <f aca="false">$C$30*G35</f>
-        <v>5599.99999999999</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>486</v>
-      </c>
-      <c r="B37" s="5" t="n">
-        <f aca="false">$C$31*B35</f>
-        <v>590.516985714286</v>
-      </c>
-      <c r="C37" s="5" t="n">
-        <f aca="false">$C$31*C35</f>
-        <v>787.355980952381</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <f aca="false">$C$31*D35</f>
-        <v>1181.03397142857</v>
-      </c>
-      <c r="E37" s="5" t="n">
-        <f aca="false">$C$31*E35</f>
-        <v>2362.06794285714</v>
-      </c>
-      <c r="F37" s="5" t="n">
-        <f aca="false">$C$31*F35</f>
-        <v>4724.13588571429</v>
-      </c>
-      <c r="G37" s="5" t="n">
-        <f aca="false">$C$31*G35</f>
-        <v>7873.55980952381</v>
-      </c>
-    </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
-        <v>487</v>
+      <c r="A39" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="B39" s="5" t="n">
+        <f aca="false">$C$33*B38</f>
+        <v>667.500000000001</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <f aca="false">$C$33*C38</f>
+        <v>890.000000000001</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <f aca="false">$C$33*D38</f>
+        <v>1335</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <f aca="false">$C$33*E38</f>
+        <v>2670</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <f aca="false">$C$33*F38</f>
+        <v>5340</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <f aca="false">$C$33*G38</f>
+        <v>8900.00000000001</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2" t="s">
-        <v>489</v>
+      <c r="A40" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="B40" s="5" t="n">
+        <f aca="false">$C$34*B38</f>
+        <v>838.016985714287</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <f aca="false">$C$34*C38</f>
+        <v>1117.35598095238</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <f aca="false">$C$34*D38</f>
+        <v>1676.03397142857</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <f aca="false">$C$34*E38</f>
+        <v>3352.06794285715</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <f aca="false">$C$34*F38</f>
+        <v>6704.13588571429</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <f aca="false">$C$34*G38</f>
+        <v>11173.5598095238</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="s">
+        <v>493</v>
+      </c>
+      <c r="C42" s="54" t="n">
+        <f aca="false">C33/(C21*$B$12)+$B$11</f>
+        <v>0.0318767908309456</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>495</v>
       </c>
     </row>
   </sheetData>
@@ -4517,40 +4570,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="B4" s="53" t="n">
         <f aca="false">Courier_Hub!B24/30</f>
         <v>3.33333333333333</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="B5" s="39" t="n">
         <v>28</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="B6" s="24" t="n">
         <v>3</v>
@@ -4559,24 +4612,24 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="B7" s="30" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="B8" s="23" t="n">
         <v>200</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4590,7 +4643,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">Courier_Hub!B22</f>
@@ -4620,27 +4673,27 @@
         <v>18</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="D14" s="44" t="s">
         <v>428</v>
       </c>
       <c r="E14" s="44" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="F14" s="44" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="G14" s="44" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="B15" s="19" t="n">
         <v>0.6</v>
@@ -4666,7 +4719,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="B16" s="19" t="n">
         <v>0.1</v>
@@ -4817,7 +4870,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -4828,7 +4881,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="B24" s="7" t="n">
         <f aca="false">MAX($B$7,E21/$B$9)</f>
@@ -4837,7 +4890,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="B25" s="6" t="n">
         <f aca="false">B24*$B$10</f>
@@ -4846,7 +4899,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="B26" s="7" t="n">
         <f aca="false">30/$B$5</f>
@@ -4855,7 +4908,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="B27" s="6" t="n">
         <f aca="false">B25*B26</f>
@@ -4864,7 +4917,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="B28" s="6" t="n">
         <f aca="false">$B$8*B26</f>
@@ -4873,7 +4926,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="B29" s="6" t="n">
         <f aca="false">G21*$B$12*$B$11</f>
@@ -4882,7 +4935,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="B30" s="45" t="n">
         <f aca="false">B27+B28+B29</f>
@@ -4891,7 +4944,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="B31" s="14" t="n">
         <f aca="false">B4*30</f>
@@ -4900,7 +4953,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="B32" s="6" t="n">
         <f aca="false">Courier_Hub!B11*MAX(Courier_Hub!B25,B31)</f>
@@ -4909,7 +4962,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="B33" s="48" t="n">
         <f aca="false">(B30+B32)/B31</f>
@@ -4918,7 +4971,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="B34" s="42" t="n">
         <f aca="false">(Supuestos!B16*B31+Supuestos!B36)/B31</f>
@@ -4927,7 +4980,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="B35" s="52" t="n">
         <f aca="false">B33-B34</f>
@@ -4936,7 +4989,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
     </row>
   </sheetData>
@@ -4964,12 +5017,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4988,7 +5041,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>1008</v>
@@ -5003,7 +5056,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>1000</v>
@@ -5018,7 +5071,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="B7" s="15" t="n">
         <v>500</v>
@@ -5033,7 +5086,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="B8" s="15" t="n">
         <v>5</v>
@@ -5048,7 +5101,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="B9" s="15" t="n">
         <v>1</v>
@@ -5063,7 +5116,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="D10" s="48" t="n">
         <f aca="false">SUM(D5:D9)</f>
@@ -5072,17 +5125,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="B14" s="38" t="n">
         <v>1135.87</v>
@@ -5090,7 +5143,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="B15" s="38" t="n">
         <v>135.13</v>
@@ -5098,7 +5151,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="B16" s="38" t="n">
         <v>1720</v>
@@ -5106,7 +5159,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="B17" s="38" t="n">
         <v>309.6</v>
@@ -5114,7 +5167,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="B18" s="38" t="n">
         <v>5961</v>
@@ -5122,7 +5175,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="B19" s="39" t="n">
         <v>1</v>
@@ -5139,7 +5192,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5149,7 +5202,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="B24" s="42" t="n">
         <f aca="false">D10*B20</f>
@@ -5158,7 +5211,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="B25" s="42" t="n">
         <f aca="false">B14*B20</f>
@@ -5167,7 +5220,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B26" s="42" t="n">
         <f aca="false">B16+B17</f>
@@ -5185,7 +5238,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="B28" s="48" t="n">
         <f aca="false">SUM(B24:B27)</f>
@@ -5194,7 +5247,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="B29" s="42" t="n">
         <f aca="false">B19*(B18+B17+B15*B20)</f>
@@ -5221,7 +5274,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5229,24 +5282,24 @@
         <v>18</v>
       </c>
       <c r="B34" s="44" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="C34" s="44" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="D34" s="44" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E34" s="44" t="s">
         <v>296</v>
       </c>
       <c r="F34" s="44" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="B35" s="42" t="n">
         <f aca="false">D5</f>
@@ -5271,7 +5324,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="B36" s="42" t="n">
         <f aca="false">D6</f>
@@ -5296,7 +5349,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B37" s="42" t="n">
         <f aca="false">D7</f>
@@ -5338,7 +5391,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
     </row>
   </sheetData>

</xml_diff>